<commit_message>
Data update. Fixed update bug with renv::init() and updating dependencies.
</commit_message>
<xml_diff>
--- a/dashboard/data/watchdb.all_tables.xlsx
+++ b/dashboard/data/watchdb.all_tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tpd0001/github/watch-wv/patchr/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tpd0001/github/watch-wv/dashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C064E69-35E9-9649-8B94-8E02FDA8AB14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{708742ED-15FB-E540-99E1-6A8BAE0D7908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="24500" windowHeight="18980" activeTab="1" xr2:uid="{ABEE2980-A2EF-284E-9534-8BF6C1D1D8CC}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="24500" windowHeight="18980" xr2:uid="{ABEE2980-A2EF-284E-9534-8BF6C1D1D8CC}"/>
   </bookViews>
   <sheets>
     <sheet name="location" sheetId="1" r:id="rId1"/>
@@ -7430,7 +7430,7 @@
         <v>351</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>103</v>
+        <v>60</v>
       </c>
       <c r="E83" s="2" t="s">
         <v>630</v>

</xml_diff>

<commit_message>
gplotly no longer accepts facet_wrap, so had to remove for now.
</commit_message>
<xml_diff>
--- a/dashboard/data/watchdb.all_tables.xlsx
+++ b/dashboard/data/watchdb.all_tables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tpd0001/github/watch-wv/dashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{708742ED-15FB-E540-99E1-6A8BAE0D7908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E14FB625-3840-BB43-97EF-8D5713EFC8B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="24500" windowHeight="18980" xr2:uid="{ABEE2980-A2EF-284E-9534-8BF6C1D1D8CC}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="24500" windowHeight="18980" activeTab="5" xr2:uid="{ABEE2980-A2EF-284E-9534-8BF6C1D1D8CC}"/>
   </bookViews>
   <sheets>
     <sheet name="location" sheetId="1" r:id="rId1"/>
@@ -1194,18 +1194,12 @@
     <t>Homo sapiens</t>
   </si>
   <si>
-    <t>Influenza Virus A (FluA)</t>
-  </si>
-  <si>
     <t>Flu A</t>
   </si>
   <si>
     <t>FluA</t>
   </si>
   <si>
-    <t>Influenza Virus B (FluB)</t>
-  </si>
-  <si>
     <t>Flu B</t>
   </si>
   <si>
@@ -1707,27 +1701,9 @@
     <t>Enterococcus</t>
   </si>
   <si>
-    <t>Escherichia coli, Shiga toxin-producing (STEC)</t>
-  </si>
-  <si>
-    <t>Human Immunodeficiency Virus 1 (HIV-1)</t>
-  </si>
-  <si>
-    <t>Human Immunodeficiency Virus 2 (HIV-2)</t>
-  </si>
-  <si>
     <t>Legionella</t>
   </si>
   <si>
-    <t>Pepper Mild Mottle Virus (PMMoV)</t>
-  </si>
-  <si>
-    <t>Respiratory Syncitial Virus, Bovine (BRSV)</t>
-  </si>
-  <si>
-    <t>Respiratory Syncitial Virus, Human (RSV)</t>
-  </si>
-  <si>
     <t>Salmonella enterica subsp. enterica serovar Enteritidis</t>
   </si>
   <si>
@@ -1743,12 +1719,6 @@
     <t>HIV-2</t>
   </si>
   <si>
-    <t>Mpox Virus I (MPXV I)</t>
-  </si>
-  <si>
-    <t>Mpox Virus II (MPXV II)</t>
-  </si>
-  <si>
     <t>Ec</t>
   </si>
   <si>
@@ -1866,18 +1836,12 @@
     <t>SC2</t>
   </si>
   <si>
-    <t>Human Norovirus GII (HuNoV-GII)</t>
-  </si>
-  <si>
     <t>ORF1_2</t>
   </si>
   <si>
     <t>Other</t>
   </si>
   <si>
-    <t>Human Norovirus GI (HuNoV-GI)</t>
-  </si>
-  <si>
     <t>major_lab_method</t>
   </si>
   <si>
@@ -1954,6 +1918,42 @@
   </si>
   <si>
     <t>54067-001-01-00-00</t>
+  </si>
+  <si>
+    <t>Influenza Virus A</t>
+  </si>
+  <si>
+    <t>Influenza Virus B</t>
+  </si>
+  <si>
+    <t>Mpox Virus I</t>
+  </si>
+  <si>
+    <t>Mpox Virus II</t>
+  </si>
+  <si>
+    <t>Human Norovirus GI</t>
+  </si>
+  <si>
+    <t>Human Norovirus GII</t>
+  </si>
+  <si>
+    <t>Pepper Mild Mottle Virus</t>
+  </si>
+  <si>
+    <t>Respiratory Syncitial Virus, Bovine</t>
+  </si>
+  <si>
+    <t>Respiratory Syncitial Virus, Human</t>
+  </si>
+  <si>
+    <t>Escherichia coli, Shiga toxin-producing</t>
+  </si>
+  <si>
+    <t>Human Immunodeficiency Virus 1</t>
+  </si>
+  <si>
+    <t>Human Immunodeficiency Virus 2</t>
   </si>
 </sst>
 </file>
@@ -2682,7 +2682,7 @@
         <v>191</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="C1" s="14" t="s">
         <v>349</v>
@@ -2945,7 +2945,7 @@
         <v>7000</v>
       </c>
       <c r="M5" s="34" t="s">
-        <v>593</v>
+        <v>583</v>
       </c>
       <c r="N5" s="34">
         <v>24</v>
@@ -2969,7 +2969,7 @@
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A6" s="44" t="s">
-        <v>585</v>
+        <v>575</v>
       </c>
       <c r="B6" s="44"/>
       <c r="C6" s="44" t="s">
@@ -2979,7 +2979,7 @@
         <v>103</v>
       </c>
       <c r="E6" s="44" t="s">
-        <v>586</v>
+        <v>576</v>
       </c>
       <c r="F6" s="44" t="s">
         <v>340</v>
@@ -2994,7 +2994,7 @@
         <v>38.537901317549398</v>
       </c>
       <c r="J6" s="44" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
       <c r="K6" s="44" t="s">
         <v>159</v>
@@ -3027,7 +3027,7 @@
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A7" s="29" t="s">
-        <v>590</v>
+        <v>580</v>
       </c>
       <c r="B7" s="29"/>
       <c r="C7" s="29" t="s">
@@ -3037,7 +3037,7 @@
         <v>103</v>
       </c>
       <c r="E7" s="29" t="s">
-        <v>583</v>
+        <v>573</v>
       </c>
       <c r="F7" s="29" t="s">
         <v>340</v>
@@ -3097,7 +3097,7 @@
         <v>103</v>
       </c>
       <c r="E8" s="29" t="s">
-        <v>582</v>
+        <v>572</v>
       </c>
       <c r="F8" s="29" t="s">
         <v>340</v>
@@ -3150,7 +3150,7 @@
         <v>52</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>625</v>
+        <v>613</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>351</v>
@@ -3210,7 +3210,7 @@
         <v>109</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>351</v>
@@ -3270,7 +3270,7 @@
         <v>62</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>351</v>
@@ -3331,7 +3331,7 @@
         <v>104</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>351</v>
@@ -3391,7 +3391,7 @@
         <v>106</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>351</v>
@@ -3451,7 +3451,7 @@
         <v>101</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>351</v>
@@ -3508,10 +3508,10 @@
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A15" s="12" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="C15" s="12" t="s">
         <v>351</v>
@@ -3520,7 +3520,7 @@
         <v>103</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="F15" s="12" t="s">
         <v>340</v>
@@ -3535,7 +3535,7 @@
         <v>37.946770700000002</v>
       </c>
       <c r="J15" s="12" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="K15" s="12" t="s">
         <v>197</v>
@@ -3571,7 +3571,7 @@
         <v>152</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>351</v>
@@ -3631,7 +3631,7 @@
         <v>108</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>351</v>
@@ -3691,7 +3691,7 @@
         <v>188</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>351</v>
@@ -3751,7 +3751,7 @@
         <v>99</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>351</v>
@@ -3807,7 +3807,7 @@
         <v>12</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>351</v>
@@ -3867,7 +3867,7 @@
         <v>8</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>351</v>
@@ -3926,7 +3926,7 @@
         <v>4</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>351</v>
@@ -3982,7 +3982,7 @@
         <v>113</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>351</v>
@@ -4041,7 +4041,7 @@
         <v>6</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>351</v>
@@ -4097,7 +4097,7 @@
         <v>93</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>351</v>
@@ -4152,7 +4152,7 @@
         <v>16</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>351</v>
@@ -4212,7 +4212,7 @@
         <v>49</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>351</v>
@@ -4268,7 +4268,7 @@
         <v>10</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>351</v>
@@ -4324,7 +4324,7 @@
         <v>2</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>351</v>
@@ -4402,14 +4402,14 @@
         <v>38.424089000000002</v>
       </c>
       <c r="J30" s="44" t="s">
-        <v>588</v>
+        <v>578</v>
       </c>
       <c r="K30" s="29" t="s">
         <v>157</v>
       </c>
       <c r="L30" s="33"/>
       <c r="M30" s="33" t="s">
-        <v>593</v>
+        <v>583</v>
       </c>
       <c r="N30" s="33">
         <v>5</v>
@@ -4430,7 +4430,7 @@
         <v>25703</v>
       </c>
       <c r="T30" s="44" t="s">
-        <v>595</v>
+        <v>585</v>
       </c>
     </row>
     <row r="31" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
@@ -4469,7 +4469,7 @@
         <v>4000</v>
       </c>
       <c r="M31" s="33" t="s">
-        <v>593</v>
+        <v>583</v>
       </c>
       <c r="N31" s="33">
         <v>24</v>
@@ -4490,7 +4490,7 @@
         <v>25504</v>
       </c>
       <c r="T31" s="45" t="s">
-        <v>596</v>
+        <v>586</v>
       </c>
     </row>
     <row r="32" spans="1:20" x14ac:dyDescent="0.2">
@@ -4520,14 +4520,14 @@
         <v>38.421745999999999</v>
       </c>
       <c r="J32" s="44" t="s">
-        <v>589</v>
+        <v>579</v>
       </c>
       <c r="K32" s="29" t="s">
         <v>157</v>
       </c>
       <c r="L32" s="33"/>
       <c r="M32" s="33" t="s">
-        <v>593</v>
+        <v>583</v>
       </c>
       <c r="N32" s="33">
         <v>5</v>
@@ -4548,7 +4548,7 @@
         <v>25703</v>
       </c>
       <c r="T32" s="44" t="s">
-        <v>594</v>
+        <v>584</v>
       </c>
     </row>
     <row r="33" spans="1:20" x14ac:dyDescent="0.2">
@@ -4666,7 +4666,7 @@
         <v>25701</v>
       </c>
       <c r="T34" s="29" t="s">
-        <v>597</v>
+        <v>587</v>
       </c>
     </row>
     <row r="35" spans="1:20" x14ac:dyDescent="0.2">
@@ -4726,7 +4726,7 @@
         <v>25537</v>
       </c>
       <c r="T35" s="29" t="s">
-        <v>598</v>
+        <v>588</v>
       </c>
     </row>
     <row r="36" spans="1:20" x14ac:dyDescent="0.2">
@@ -4756,14 +4756,14 @@
         <v>38.422913110104098</v>
       </c>
       <c r="J36" s="44" t="s">
-        <v>591</v>
+        <v>581</v>
       </c>
       <c r="K36" s="29" t="s">
         <v>157</v>
       </c>
       <c r="L36" s="33"/>
       <c r="M36" s="34" t="s">
-        <v>593</v>
+        <v>583</v>
       </c>
       <c r="N36" s="33">
         <v>5</v>
@@ -4812,14 +4812,14 @@
         <v>38.423076174075902</v>
       </c>
       <c r="J37" s="44" t="s">
-        <v>592</v>
+        <v>582</v>
       </c>
       <c r="K37" s="29" t="s">
         <v>157</v>
       </c>
       <c r="L37" s="33"/>
       <c r="M37" s="34" t="s">
-        <v>593</v>
+        <v>583</v>
       </c>
       <c r="N37" s="33">
         <v>24</v>
@@ -4846,7 +4846,7 @@
         <v>18</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>351</v>
@@ -4906,7 +4906,7 @@
         <v>35</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>351</v>
@@ -4962,7 +4962,7 @@
         <v>0</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>351</v>
@@ -4971,7 +4971,7 @@
         <v>60</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>584</v>
+        <v>574</v>
       </c>
       <c r="F40" s="2" t="s">
         <v>340</v>
@@ -5018,7 +5018,7 @@
         <v>40</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>351</v>
@@ -5074,7 +5074,7 @@
         <v>21</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>351</v>
@@ -5136,7 +5136,7 @@
         <v>25</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>351</v>
@@ -5198,7 +5198,7 @@
         <v>26</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>351</v>
@@ -5260,7 +5260,7 @@
         <v>22</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>351</v>
@@ -5320,7 +5320,7 @@
         <v>27</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>351</v>
@@ -5380,7 +5380,7 @@
         <v>28</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C47" s="2" t="s">
         <v>351</v>
@@ -5440,7 +5440,7 @@
         <v>111</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="C48" s="2" t="s">
         <v>351</v>
@@ -5551,7 +5551,7 @@
         <v>192</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C50" s="2" t="s">
         <v>351</v>
@@ -5613,7 +5613,7 @@
         <v>29</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C51" s="2" t="s">
         <v>351</v>
@@ -5673,7 +5673,7 @@
         <v>30</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C52" s="2" t="s">
         <v>351</v>
@@ -5733,7 +5733,7 @@
         <v>38</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="C53" s="2" t="s">
         <v>351</v>
@@ -5788,7 +5788,7 @@
         <v>39</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="C54" s="2" t="s">
         <v>351</v>
@@ -5843,7 +5843,7 @@
         <v>31</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C55" s="2" t="s">
         <v>351</v>
@@ -5903,7 +5903,7 @@
         <v>36</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C56" s="2" t="s">
         <v>351</v>
@@ -5958,7 +5958,7 @@
         <v>339</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C57" s="2" t="s">
         <v>351</v>
@@ -6018,7 +6018,7 @@
         <v>23</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C58" s="2" t="s">
         <v>351</v>
@@ -6134,7 +6134,7 @@
         <v>184</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C60" s="2" t="s">
         <v>351</v>
@@ -6193,10 +6193,10 @@
     </row>
     <row r="61" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="2" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C61" s="2" t="s">
         <v>351</v>
@@ -6205,7 +6205,7 @@
         <v>60</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="F61" s="2" t="s">
         <v>341</v>
@@ -6251,10 +6251,10 @@
     </row>
     <row r="62" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C62" s="2" t="s">
         <v>351</v>
@@ -6263,7 +6263,7 @@
         <v>103</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="F62" s="2" t="s">
         <v>341</v>
@@ -6305,10 +6305,10 @@
     </row>
     <row r="63" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="2" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C63" s="2" t="s">
         <v>351</v>
@@ -6317,7 +6317,7 @@
         <v>103</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="F63" s="2" t="s">
         <v>341</v>
@@ -6359,10 +6359,10 @@
     </row>
     <row r="64" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="2" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C64" s="2" t="s">
         <v>351</v>
@@ -6371,7 +6371,7 @@
         <v>103</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="F64" s="2" t="s">
         <v>341</v>
@@ -6416,7 +6416,7 @@
         <v>51</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="C65" s="2" t="s">
         <v>351</v>
@@ -6476,7 +6476,7 @@
         <v>58</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="C66" s="2" t="s">
         <v>351</v>
@@ -6532,7 +6532,7 @@
         <v>24</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C67" s="2" t="s">
         <v>351</v>
@@ -6594,7 +6594,7 @@
         <v>37</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="C68" s="2" t="s">
         <v>351</v>
@@ -6650,7 +6650,7 @@
         <v>32</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C69" s="2" t="s">
         <v>351</v>
@@ -6707,10 +6707,10 @@
     </row>
     <row r="70" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="2" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C70" s="2" t="s">
         <v>351</v>
@@ -6719,7 +6719,7 @@
         <v>103</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="F70" s="2" t="s">
         <v>341</v>
@@ -6764,7 +6764,7 @@
         <v>33</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C71" s="2" t="s">
         <v>351</v>
@@ -7102,7 +7102,7 @@
         <v>59</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="C77" s="2" t="s">
         <v>351</v>
@@ -7210,7 +7210,7 @@
         <v>14</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="C79" s="2" t="s">
         <v>351</v>
@@ -7368,10 +7368,10 @@
     </row>
     <row r="82" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A82" s="2" t="s">
-        <v>618</v>
+        <v>606</v>
       </c>
       <c r="B82" t="s">
-        <v>622</v>
+        <v>610</v>
       </c>
       <c r="C82" s="2" t="s">
         <v>351</v>
@@ -7380,7 +7380,7 @@
         <v>181</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>619</v>
+        <v>607</v>
       </c>
       <c r="F82" s="2" t="s">
         <v>340</v>
@@ -7395,7 +7395,7 @@
         <v>39.115929999999999</v>
       </c>
       <c r="J82" s="2" t="s">
-        <v>620</v>
+        <v>608</v>
       </c>
       <c r="K82" s="2" t="s">
         <v>202</v>
@@ -7421,10 +7421,10 @@
     </row>
     <row r="83" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A83" s="2" t="s">
-        <v>629</v>
+        <v>617</v>
       </c>
       <c r="B83" t="s">
-        <v>628</v>
+        <v>616</v>
       </c>
       <c r="C83" s="2" t="s">
         <v>351</v>
@@ -7433,7 +7433,7 @@
         <v>60</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>630</v>
+        <v>618</v>
       </c>
       <c r="F83" s="2" t="s">
         <v>340</v>
@@ -7448,7 +7448,7 @@
         <v>38.301869799999999</v>
       </c>
       <c r="J83" s="2" t="s">
-        <v>631</v>
+        <v>619</v>
       </c>
       <c r="K83" s="2" t="s">
         <v>209</v>
@@ -7509,7 +7509,7 @@
         <v>230</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="C1" s="13" t="s">
         <v>229</v>
@@ -7521,7 +7521,7 @@
         <v>238</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="G1" s="13" t="s">
         <v>240</v>
@@ -7538,7 +7538,7 @@
         <v>275</v>
       </c>
       <c r="B2" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="C2" s="17" t="s">
         <v>64</v>
@@ -7550,7 +7550,7 @@
         <v>63</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="G2" s="31">
         <v>54003906001</v>
@@ -7568,7 +7568,7 @@
         <v>244</v>
       </c>
       <c r="B3" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="C3" s="17" t="s">
         <v>277</v>
@@ -7580,7 +7580,7 @@
         <v>17</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="G3" s="17">
         <v>54002701001</v>
@@ -7605,7 +7605,7 @@
         <v>157</v>
       </c>
       <c r="F4" s="64" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="G4" s="63">
         <v>54000601001</v>
@@ -7632,7 +7632,7 @@
         <v>123</v>
       </c>
       <c r="F5" s="64" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="G5" s="63">
         <v>54000101001</v>
@@ -7659,7 +7659,7 @@
         <v>11</v>
       </c>
       <c r="F6" s="64" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="G6" s="63">
         <v>54003031001</v>
@@ -7686,7 +7686,7 @@
         <v>88</v>
       </c>
       <c r="F7" s="64" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="G7" s="63">
         <v>54001702001</v>
@@ -7711,7 +7711,7 @@
         <v>5</v>
       </c>
       <c r="F8" s="64" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="G8" s="63">
         <v>54002510001</v>
@@ -7728,7 +7728,7 @@
         <v>357</v>
       </c>
       <c r="B9" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="C9" s="17" t="s">
         <v>362</v>
@@ -7738,7 +7738,7 @@
         <v>1</v>
       </c>
       <c r="F9" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="G9" s="31">
         <v>54002003001</v>
@@ -7755,7 +7755,7 @@
         <v>249</v>
       </c>
       <c r="B10" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="C10" s="17" t="s">
         <v>282</v>
@@ -7765,7 +7765,7 @@
         <v>1</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="G10" s="31">
         <v>54002003001</v>
@@ -7782,7 +7782,7 @@
         <v>250</v>
       </c>
       <c r="B11" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="C11" s="17" t="s">
         <v>283</v>
@@ -7792,7 +7792,7 @@
         <v>7</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="G11" s="31">
         <v>54001901001</v>
@@ -7809,7 +7809,7 @@
         <v>251</v>
       </c>
       <c r="B12" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="C12" s="17" t="s">
         <v>306</v>
@@ -7821,7 +7821,7 @@
         <v>11</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="G12" s="31">
         <v>54003045001</v>
@@ -7838,7 +7838,7 @@
         <v>252</v>
       </c>
       <c r="B13" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="C13" s="17" t="s">
         <v>284</v>
@@ -7848,7 +7848,7 @@
         <v>88</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="G13" s="31">
         <v>54001703001</v>
@@ -7865,7 +7865,7 @@
         <v>358</v>
       </c>
       <c r="B14" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="C14" s="17" t="s">
         <v>363</v>
@@ -7875,7 +7875,7 @@
         <v>1</v>
       </c>
       <c r="F14" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="G14" s="31">
         <v>54002007001</v>
@@ -7892,7 +7892,7 @@
         <v>253</v>
       </c>
       <c r="B15" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="C15" s="17" t="s">
         <v>285</v>
@@ -7902,7 +7902,7 @@
         <v>121</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="G15" s="31">
         <v>54004202001</v>
@@ -7927,7 +7927,7 @@
         <v>89</v>
       </c>
       <c r="F16" s="64" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="G16" s="63">
         <v>54002405001</v>
@@ -7944,7 +7944,7 @@
         <v>255</v>
       </c>
       <c r="B17" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="C17" s="17" t="s">
         <v>287</v>
@@ -7954,7 +7954,7 @@
         <v>89</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="G17" s="31">
         <v>54002408001</v>
@@ -7971,7 +7971,7 @@
         <v>256</v>
       </c>
       <c r="B18" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="C18" s="17" t="s">
         <v>288</v>
@@ -7981,7 +7981,7 @@
         <v>122</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="G18" s="17">
         <v>54000504001</v>
@@ -7998,7 +7998,7 @@
         <v>257</v>
       </c>
       <c r="B19" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="C19" s="17" t="s">
         <v>289</v>
@@ -8008,7 +8008,7 @@
         <v>100</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="G19" s="31">
         <v>54004602001</v>
@@ -8045,22 +8045,22 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" s="49" t="s">
-        <v>599</v>
+        <v>589</v>
       </c>
       <c r="B21" s="50" t="s">
-        <v>635</v>
+        <v>623</v>
       </c>
       <c r="C21" s="49" t="s">
-        <v>586</v>
+        <v>576</v>
       </c>
       <c r="D21" s="49" t="s">
-        <v>600</v>
+        <v>590</v>
       </c>
       <c r="E21" s="49" t="s">
         <v>159</v>
       </c>
       <c r="F21" s="49" t="s">
-        <v>601</v>
+        <v>591</v>
       </c>
       <c r="G21" s="49"/>
       <c r="H21" s="49">
@@ -8075,7 +8075,7 @@
         <v>353</v>
       </c>
       <c r="B22" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="C22" s="17" t="s">
         <v>360</v>
@@ -8087,7 +8087,7 @@
         <v>182</v>
       </c>
       <c r="F22" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="G22" s="31">
         <v>54000603001</v>
@@ -8104,7 +8104,7 @@
         <v>258</v>
       </c>
       <c r="B23" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="C23" s="17" t="s">
         <v>291</v>
@@ -8114,7 +8114,7 @@
         <v>121</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="G23" s="31">
         <v>54004215001</v>
@@ -8131,7 +8131,7 @@
         <v>243</v>
       </c>
       <c r="B24" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="C24" s="17" t="s">
         <v>292</v>
@@ -8141,7 +8141,7 @@
         <v>13</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="G24" s="31">
         <v>54002803001</v>
@@ -8158,7 +8158,7 @@
         <v>259</v>
       </c>
       <c r="B25" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="C25" s="17" t="s">
         <v>293</v>
@@ -8168,7 +8168,7 @@
         <v>153</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="G25" s="31">
         <v>54000316001</v>
@@ -8185,7 +8185,7 @@
         <v>260</v>
       </c>
       <c r="B26" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="C26" s="17" t="s">
         <v>294</v>
@@ -8195,7 +8195,7 @@
         <v>89</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="G26" s="31">
         <v>54002415001</v>
@@ -8212,7 +8212,7 @@
         <v>261</v>
       </c>
       <c r="B27" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="C27" s="17" t="s">
         <v>295</v>
@@ -8222,7 +8222,7 @@
         <v>5</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="G27" s="31">
         <v>54002509001</v>
@@ -8239,7 +8239,7 @@
         <v>262</v>
       </c>
       <c r="B28" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="C28" s="17" t="s">
         <v>296</v>
@@ -8249,7 +8249,7 @@
         <v>54</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="G28" s="31">
         <v>54005405001</v>
@@ -8266,7 +8266,7 @@
         <v>355</v>
       </c>
       <c r="B29" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="C29" s="17" t="s">
         <v>365</v>
@@ -8276,7 +8276,7 @@
         <v>157</v>
       </c>
       <c r="F29" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="G29" s="4"/>
       <c r="H29" s="17">
@@ -8341,7 +8341,7 @@
         <v>55</v>
       </c>
       <c r="F32" s="61" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="G32" s="61">
         <v>54001205001</v>
@@ -8358,7 +8358,7 @@
         <v>264</v>
       </c>
       <c r="B33" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C33" s="17" t="s">
         <v>307</v>
@@ -8368,7 +8368,7 @@
         <v>190</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="G33" s="17">
         <v>54002606001</v>
@@ -8385,7 +8385,7 @@
         <v>265</v>
       </c>
       <c r="B34" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="C34" s="17" t="s">
         <v>298</v>
@@ -8395,7 +8395,7 @@
         <v>17</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="G34" s="17">
         <v>54002716001</v>
@@ -8412,7 +8412,7 @@
         <v>266</v>
       </c>
       <c r="B35" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="C35" s="17" t="s">
         <v>299</v>
@@ -8422,7 +8422,7 @@
         <v>88</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="G35" s="31">
         <v>54001710001</v>
@@ -8439,7 +8439,7 @@
         <v>370</v>
       </c>
       <c r="B36" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="C36" s="17" t="s">
         <v>372</v>
@@ -8449,7 +8449,7 @@
         <v>157</v>
       </c>
       <c r="F36" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="G36" s="4"/>
       <c r="H36" s="17">
@@ -8464,7 +8464,7 @@
         <v>371</v>
       </c>
       <c r="B37" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="C37" s="17" t="s">
         <v>373</v>
@@ -8474,7 +8474,7 @@
         <v>157</v>
       </c>
       <c r="F37" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="G37" s="17"/>
       <c r="H37" s="17">
@@ -8497,7 +8497,7 @@
         <v>129</v>
       </c>
       <c r="F38" s="64" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="G38" s="63">
         <v>54004804001</v>
@@ -8514,7 +8514,7 @@
         <v>231</v>
       </c>
       <c r="B39" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="C39" s="17" t="s">
         <v>276</v>
@@ -8526,7 +8526,7 @@
         <v>11</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="G39" s="31">
         <v>54003011001</v>
@@ -8543,7 +8543,7 @@
         <v>268</v>
       </c>
       <c r="B40" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="C40" s="17" t="s">
         <v>308</v>
@@ -8553,7 +8553,7 @@
         <v>56</v>
       </c>
       <c r="F40" s="17" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="G40" s="17">
         <v>54003703001</v>
@@ -8570,7 +8570,7 @@
         <v>269</v>
       </c>
       <c r="B41" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="C41" s="17" t="s">
         <v>301</v>
@@ -8580,7 +8580,7 @@
         <v>15</v>
       </c>
       <c r="F41" s="17" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="G41" s="31">
         <v>54003203001</v>
@@ -8605,7 +8605,7 @@
         <v>122</v>
       </c>
       <c r="F42" s="61" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="G42" s="63">
         <v>54000509001</v>
@@ -8622,7 +8622,7 @@
         <v>271</v>
       </c>
       <c r="B43" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="C43" s="17" t="s">
         <v>303</v>
@@ -8632,7 +8632,7 @@
         <v>9</v>
       </c>
       <c r="F43" s="17" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="G43" s="17">
         <v>54002102001</v>
@@ -8649,7 +8649,7 @@
         <v>272</v>
       </c>
       <c r="B44" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="C44" s="17" t="s">
         <v>309</v>
@@ -8659,7 +8659,7 @@
         <v>57</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="G44" s="31">
         <v>54000901001</v>
@@ -8676,7 +8676,7 @@
         <v>273</v>
       </c>
       <c r="B45" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="C45" s="17" t="s">
         <v>304</v>
@@ -8686,7 +8686,7 @@
         <v>3</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="G45" s="31">
         <v>54003508001</v>
@@ -8700,20 +8700,20 @@
     </row>
     <row r="46" spans="1:26" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A46" s="4" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D46" s="4"/>
       <c r="E46" s="4" t="s">
         <v>197</v>
       </c>
       <c r="F46" s="31" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="G46" s="31">
         <v>54001022001</v>
@@ -8774,22 +8774,22 @@
     </row>
     <row r="48" spans="1:26" s="62" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A48" s="61" t="s">
-        <v>620</v>
+        <v>608</v>
       </c>
       <c r="B48" s="62" t="s">
-        <v>623</v>
+        <v>611</v>
       </c>
       <c r="C48" s="62" t="s">
-        <v>621</v>
+        <v>609</v>
       </c>
       <c r="D48" s="62" t="s">
-        <v>621</v>
+        <v>609</v>
       </c>
       <c r="E48" s="61" t="s">
         <v>202</v>
       </c>
       <c r="F48" s="61" t="s">
-        <v>624</v>
+        <v>612</v>
       </c>
       <c r="G48" s="63">
         <v>54001601001</v>
@@ -8803,22 +8803,22 @@
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A49" s="17" t="s">
-        <v>631</v>
+        <v>619</v>
       </c>
       <c r="B49" s="66" t="s">
-        <v>636</v>
+        <v>624</v>
       </c>
       <c r="C49" s="17" t="s">
-        <v>632</v>
+        <v>620</v>
       </c>
       <c r="D49" t="s">
-        <v>633</v>
+        <v>621</v>
       </c>
       <c r="E49" s="17" t="s">
         <v>209</v>
       </c>
       <c r="F49" s="17" t="s">
-        <v>634</v>
+        <v>622</v>
       </c>
       <c r="G49" s="31">
         <v>54003404001</v>
@@ -8854,10 +8854,10 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="13" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="C1" s="13" t="s">
         <v>239</v>
@@ -9020,7 +9020,7 @@
         <v>197</v>
       </c>
       <c r="B11" s="56" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="C11" s="57">
         <v>54019</v>
@@ -9117,7 +9117,7 @@
         <v>202</v>
       </c>
       <c r="B17" s="56" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="C17" s="57">
         <v>54031</v>
@@ -9419,7 +9419,7 @@
         <v>209</v>
       </c>
       <c r="B35" s="56" t="s">
-        <v>627</v>
+        <v>615</v>
       </c>
       <c r="C35" s="57">
         <v>54067</v>
@@ -9841,7 +9841,7 @@
         <v>380</v>
       </c>
       <c r="C2" s="25" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="D2" s="25" t="s">
         <v>381</v>
@@ -9855,19 +9855,19 @@
     </row>
     <row r="3" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A3" s="42" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="B3" s="25" t="s">
+        <v>407</v>
+      </c>
+      <c r="C3" s="25" t="s">
+        <v>414</v>
+      </c>
+      <c r="D3" s="25" t="s">
+        <v>408</v>
+      </c>
+      <c r="E3" s="25" t="s">
         <v>409</v>
-      </c>
-      <c r="C3" s="25" t="s">
-        <v>416</v>
-      </c>
-      <c r="D3" s="25" t="s">
-        <v>410</v>
-      </c>
-      <c r="E3" s="25" t="s">
-        <v>411</v>
       </c>
       <c r="F3" s="25" t="s">
         <v>315</v>
@@ -9875,13 +9875,13 @@
     </row>
     <row r="4" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A4" s="42" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="B4" s="25" t="s">
-        <v>568</v>
+        <v>558</v>
       </c>
       <c r="C4" s="25" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="D4" s="25"/>
       <c r="E4" s="25" t="s">
@@ -9890,16 +9890,16 @@
     </row>
     <row r="5" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A5" s="42" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="B5" s="25" t="s">
+        <v>412</v>
+      </c>
+      <c r="C5" s="25" t="s">
         <v>414</v>
       </c>
-      <c r="C5" s="25" t="s">
-        <v>416</v>
-      </c>
       <c r="D5" s="25" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="E5" s="25" t="s">
         <v>382</v>
@@ -9907,13 +9907,13 @@
     </row>
     <row r="6" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A6" s="42" t="s">
-        <v>554</v>
+        <v>634</v>
       </c>
       <c r="B6" s="25" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="C6" s="25" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="D6" s="25" t="s">
         <v>381</v>
@@ -9922,235 +9922,235 @@
         <v>382</v>
       </c>
       <c r="F6" s="25" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="G6" s="25"/>
     </row>
     <row r="7" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A7" s="42" t="s">
-        <v>555</v>
+        <v>635</v>
       </c>
       <c r="B7" s="25" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="C7" s="25" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="D7" s="25" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="E7" s="25" t="s">
         <v>382</v>
       </c>
       <c r="F7" s="25" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A8" s="42" t="s">
-        <v>556</v>
+        <v>636</v>
       </c>
       <c r="B8" s="25" t="s">
-        <v>565</v>
+        <v>557</v>
       </c>
       <c r="C8" s="25" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="D8" s="25" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="E8" s="25" t="s">
         <v>382</v>
       </c>
       <c r="F8" s="25" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A9" s="42" t="s">
+        <v>625</v>
+      </c>
+      <c r="B9" s="25" t="s">
         <v>383</v>
       </c>
-      <c r="B9" s="25" t="s">
-        <v>384</v>
-      </c>
       <c r="C9" s="25" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="E9" s="25" t="s">
         <v>382</v>
       </c>
       <c r="F9" s="25" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A10" s="42" t="s">
-        <v>386</v>
+        <v>626</v>
       </c>
       <c r="B10" s="25" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="C10" s="25" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="D10" s="25" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="E10" s="25" t="s">
         <v>382</v>
       </c>
       <c r="F10" s="25" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A11" s="42" t="s">
-        <v>557</v>
+        <v>552</v>
       </c>
       <c r="B11" s="25" t="s">
-        <v>569</v>
+        <v>559</v>
       </c>
       <c r="C11" s="25" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="E11" s="25" t="s">
         <v>382</v>
       </c>
       <c r="F11" s="25" t="s">
-        <v>574</v>
+        <v>564</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A12" s="42" t="s">
-        <v>566</v>
+        <v>627</v>
       </c>
       <c r="B12" s="25" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="C12" s="25" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="D12" s="25" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="E12" s="25" t="s">
         <v>382</v>
       </c>
       <c r="F12" s="25" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A13" s="42" t="s">
-        <v>567</v>
+        <v>628</v>
       </c>
       <c r="B13" s="25" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="C13" s="25" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="D13" s="25" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="E13" s="25" t="s">
         <v>382</v>
       </c>
       <c r="F13" s="25" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="G13" s="25"/>
     </row>
     <row r="14" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A14" s="42" t="s">
-        <v>610</v>
+        <v>629</v>
       </c>
       <c r="B14" s="25" t="s">
-        <v>617</v>
+        <v>605</v>
       </c>
       <c r="C14" s="25" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="D14" s="25" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="E14" s="25" t="s">
         <v>382</v>
       </c>
       <c r="F14" s="25" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A15" s="42" t="s">
-        <v>607</v>
+        <v>630</v>
       </c>
       <c r="B15" s="25" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="C15" s="25" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="D15" s="25" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="E15" s="25" t="s">
         <v>382</v>
       </c>
       <c r="F15" s="25" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A16" s="42" t="s">
-        <v>558</v>
+        <v>631</v>
       </c>
       <c r="B16" s="25" t="s">
+        <v>401</v>
+      </c>
+      <c r="C16" s="25" t="s">
+        <v>414</v>
+      </c>
+      <c r="D16" s="25" t="s">
+        <v>402</v>
+      </c>
+      <c r="E16" s="25" t="s">
         <v>403</v>
       </c>
-      <c r="C16" s="25" t="s">
-        <v>416</v>
-      </c>
-      <c r="D16" s="25" t="s">
+      <c r="F16" s="25" t="s">
         <v>404</v>
-      </c>
-      <c r="E16" s="25" t="s">
-        <v>405</v>
-      </c>
-      <c r="F16" s="25" t="s">
-        <v>406</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A17" s="42" t="s">
-        <v>559</v>
+        <v>632</v>
       </c>
       <c r="B17" s="25" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="D17" s="25" t="s">
         <v>381</v>
       </c>
       <c r="E17" s="25" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="F17" s="25" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="G17" s="25"/>
     </row>
     <row r="18" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A18" s="42" t="s">
-        <v>560</v>
+        <v>633</v>
       </c>
       <c r="B18" s="25" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="D18" s="25" t="s">
         <v>381</v>
@@ -10159,18 +10159,18 @@
         <v>382</v>
       </c>
       <c r="F18" s="25" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A19" s="42" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="B19" s="25" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="D19" s="25" t="s">
         <v>381</v>
@@ -10179,21 +10179,21 @@
         <v>382</v>
       </c>
       <c r="F19" s="25" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A20" s="42" t="s">
-        <v>561</v>
+        <v>553</v>
       </c>
       <c r="B20" s="25" t="s">
-        <v>570</v>
+        <v>560</v>
       </c>
       <c r="C20" s="25" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="D20" s="25" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="E20" s="25" t="s">
         <v>382</v>
@@ -10201,16 +10201,16 @@
     </row>
     <row r="21" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A21" s="42" t="s">
-        <v>562</v>
+        <v>554</v>
       </c>
       <c r="B21" s="25" t="s">
-        <v>573</v>
+        <v>563</v>
       </c>
       <c r="C21" s="25" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="D21" s="25" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="E21" s="25" t="s">
         <v>382</v>
@@ -10218,16 +10218,16 @@
     </row>
     <row r="22" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A22" s="42" t="s">
-        <v>563</v>
+        <v>555</v>
       </c>
       <c r="B22" s="25" t="s">
-        <v>571</v>
+        <v>561</v>
       </c>
       <c r="C22" s="25" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="D22" s="25" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="E22" s="25" t="s">
         <v>382</v>
@@ -10235,16 +10235,16 @@
     </row>
     <row r="23" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A23" s="42" t="s">
-        <v>564</v>
+        <v>556</v>
       </c>
       <c r="B23" s="25" t="s">
-        <v>572</v>
+        <v>562</v>
       </c>
       <c r="C23" s="25" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="D23" s="25" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="E23" s="25" t="s">
         <v>382</v>
@@ -10252,13 +10252,13 @@
     </row>
     <row r="24" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A24" s="42" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="B24" s="25" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="C24" s="25" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="D24" s="25" t="s">
         <v>381</v>
@@ -10267,21 +10267,21 @@
         <v>382</v>
       </c>
       <c r="F24" s="25" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="19" x14ac:dyDescent="0.25">
       <c r="A25" s="42" t="s">
-        <v>602</v>
+        <v>592</v>
       </c>
       <c r="B25" s="25" t="s">
-        <v>602</v>
+        <v>592</v>
       </c>
       <c r="C25" s="25" t="s">
-        <v>626</v>
+        <v>614</v>
       </c>
       <c r="D25" s="25" t="s">
-        <v>626</v>
+        <v>614</v>
       </c>
       <c r="E25" s="25" t="s">
         <v>382</v>
@@ -10312,19 +10312,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="26" t="s">
+        <v>416</v>
+      </c>
+      <c r="B1" s="26" t="s">
+        <v>417</v>
+      </c>
+      <c r="C1" s="26" t="s">
         <v>418</v>
       </c>
-      <c r="B1" s="26" t="s">
+      <c r="D1" s="26" t="s">
         <v>419</v>
       </c>
-      <c r="C1" s="26" t="s">
+      <c r="E1" s="26" t="s">
         <v>420</v>
-      </c>
-      <c r="D1" s="26" t="s">
-        <v>421</v>
-      </c>
-      <c r="E1" s="26" t="s">
-        <v>422</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -10332,16 +10332,16 @@
         <v>351</v>
       </c>
       <c r="B2" t="s">
+        <v>421</v>
+      </c>
+      <c r="C2" t="s">
+        <v>422</v>
+      </c>
+      <c r="D2" t="s">
         <v>423</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>424</v>
-      </c>
-      <c r="D2" t="s">
-        <v>425</v>
-      </c>
-      <c r="E2" t="s">
-        <v>426</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -10349,16 +10349,16 @@
         <v>352</v>
       </c>
       <c r="B3" t="s">
+        <v>425</v>
+      </c>
+      <c r="C3" t="s">
+        <v>426</v>
+      </c>
+      <c r="D3" t="s">
         <v>427</v>
       </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
         <v>428</v>
-      </c>
-      <c r="D3" t="s">
-        <v>429</v>
-      </c>
-      <c r="E3" t="s">
-        <v>430</v>
       </c>
     </row>
   </sheetData>
@@ -10381,28 +10381,28 @@
         <v>374</v>
       </c>
       <c r="B1" s="24" t="s">
-        <v>581</v>
+        <v>571</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="25" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="B2" s="43" t="s">
-        <v>576</v>
+        <v>566</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="25" t="s">
-        <v>602</v>
+        <v>592</v>
       </c>
       <c r="B3" s="43" t="s">
-        <v>579</v>
+        <v>569</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="43" t="s">
-        <v>383</v>
+        <v>625</v>
       </c>
       <c r="B4" s="43" t="s">
         <v>329</v>
@@ -10410,63 +10410,63 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="43" t="s">
-        <v>386</v>
+        <v>626</v>
       </c>
       <c r="B5" s="43" t="s">
-        <v>603</v>
+        <v>593</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="25" t="s">
-        <v>557</v>
+        <v>552</v>
       </c>
       <c r="B6" s="43" t="s">
-        <v>575</v>
+        <v>565</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="43" t="s">
-        <v>566</v>
+        <v>627</v>
       </c>
       <c r="B7" s="43" t="s">
-        <v>577</v>
+        <v>567</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="43" t="s">
-        <v>567</v>
+        <v>628</v>
       </c>
       <c r="B8" s="43" t="s">
-        <v>580</v>
+        <v>570</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="25" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="B9" s="43" t="s">
-        <v>604</v>
+        <v>594</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="25" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="B10" s="43" t="s">
-        <v>605</v>
+        <v>595</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="25" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="B11" s="43" t="s">
-        <v>606</v>
+        <v>596</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="25" t="s">
-        <v>560</v>
+        <v>633</v>
       </c>
       <c r="B12" s="25" t="s">
         <v>323</v>
@@ -10474,42 +10474,42 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="25" t="s">
-        <v>607</v>
+        <v>630</v>
       </c>
       <c r="B13" s="25" t="s">
-        <v>608</v>
+        <v>597</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="52" t="s">
-        <v>559</v>
+        <v>632</v>
       </c>
       <c r="B14" s="25" t="s">
-        <v>609</v>
+        <v>598</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="53" t="s">
-        <v>555</v>
+        <v>635</v>
       </c>
       <c r="B15" s="25" t="s">
-        <v>609</v>
+        <v>598</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="53" t="s">
-        <v>556</v>
+        <v>636</v>
       </c>
       <c r="B16" s="25" t="s">
-        <v>609</v>
+        <v>598</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="52" t="s">
-        <v>610</v>
+        <v>629</v>
       </c>
       <c r="B17" s="25" t="s">
-        <v>578</v>
+        <v>568</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -10543,10 +10543,10 @@
   <sheetData>
     <row r="1" spans="1:2" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" s="54" t="s">
-        <v>611</v>
+        <v>599</v>
       </c>
       <c r="B1" s="54" t="s">
-        <v>612</v>
+        <v>600</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -10554,7 +10554,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="55" t="s">
-        <v>613</v>
+        <v>601</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="51" x14ac:dyDescent="0.2">
@@ -10562,7 +10562,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="55" t="s">
-        <v>614</v>
+        <v>602</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -10582,7 +10582,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="55" t="s">
-        <v>615</v>
+        <v>603</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="51" x14ac:dyDescent="0.2">
@@ -10590,7 +10590,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="55" t="s">
-        <v>616</v>
+        <v>604</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Data update - activate Summersville.
</commit_message>
<xml_diff>
--- a/dashboard/data/watchdb.all_tables.xlsx
+++ b/dashboard/data/watchdb.all_tables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tpd0001/github/watch-wv/patchr/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54462D28-41AC-B142-8D34-1C1C95523423}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27DA4118-05BD-6A44-8EA4-D199C2229565}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="24500" windowHeight="18980" xr2:uid="{ABEE2980-A2EF-284E-9534-8BF6C1D1D8CC}"/>
   </bookViews>
@@ -2216,7 +2216,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2375,6 +2375,16 @@
     </xf>
     <xf numFmtId="0" fontId="26" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="27" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -3538,10 +3548,10 @@
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>436</v>
+        <v>10</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>351</v>
@@ -3550,37 +3560,39 @@
         <v>103</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>437</v>
+        <v>137</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>368</v>
-      </c>
-      <c r="H15" s="10"/>
-      <c r="I15" s="2"/>
+        <v>369</v>
+      </c>
+      <c r="H15" s="2">
+        <v>-79.992055399999998</v>
+      </c>
+      <c r="I15" s="2">
+        <v>39.655174500000001</v>
+      </c>
       <c r="J15" s="2" t="s">
-        <v>10</v>
+        <v>231</v>
       </c>
       <c r="K15" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="L15" s="2"/>
-      <c r="M15" s="33" t="s">
-        <v>337</v>
-      </c>
-      <c r="N15" s="33">
-        <v>12</v>
-      </c>
-      <c r="O15" s="34">
-        <v>25</v>
-      </c>
-      <c r="P15" s="34">
-        <v>30</v>
-      </c>
+      <c r="L15" s="34">
+        <v>48328</v>
+      </c>
+      <c r="M15" s="34" t="s">
+        <v>338</v>
+      </c>
+      <c r="N15" s="34">
+        <v>24</v>
+      </c>
+      <c r="O15" s="34"/>
+      <c r="P15" s="34"/>
       <c r="Q15" s="2" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="R15" s="2" t="s">
         <v>20</v>
@@ -3591,65 +3603,71 @@
       <c r="T15" s="2"/>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A16" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>510</v>
-      </c>
-      <c r="C16" s="2" t="s">
+      <c r="A16" s="70" t="s">
+        <v>617</v>
+      </c>
+      <c r="B16" s="70" t="s">
+        <v>616</v>
+      </c>
+      <c r="C16" s="70" t="s">
         <v>351</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="71" t="s">
         <v>103</v>
       </c>
-      <c r="E16" s="2" t="s">
-        <v>435</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>341</v>
-      </c>
-      <c r="G16" s="2" t="s">
+      <c r="E16" s="70" t="s">
+        <v>618</v>
+      </c>
+      <c r="F16" s="70" t="s">
+        <v>340</v>
+      </c>
+      <c r="G16" s="70" t="s">
         <v>368</v>
       </c>
-      <c r="H16" s="10"/>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="K16" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="L16" s="2"/>
-      <c r="M16" s="33" t="s">
+      <c r="H16" s="70">
+        <v>-80.910900499999997</v>
+      </c>
+      <c r="I16" s="70">
+        <v>38.301869799999999</v>
+      </c>
+      <c r="J16" s="70" t="s">
+        <v>619</v>
+      </c>
+      <c r="K16" s="70" t="s">
+        <v>209</v>
+      </c>
+      <c r="L16" s="72">
+        <v>3791</v>
+      </c>
+      <c r="M16" s="73" t="s">
         <v>337</v>
       </c>
-      <c r="N16" s="33">
-        <v>12</v>
-      </c>
-      <c r="O16" s="34">
+      <c r="N16" s="73">
+        <v>24</v>
+      </c>
+      <c r="O16" s="73">
         <v>25</v>
       </c>
-      <c r="P16" s="34">
+      <c r="P16" s="73">
         <v>30</v>
       </c>
-      <c r="Q16" s="2" t="s">
+      <c r="Q16" s="70" t="s">
         <v>347</v>
       </c>
-      <c r="R16" s="2" t="s">
+      <c r="R16" s="70" t="s">
         <v>20</v>
       </c>
-      <c r="S16" s="4">
-        <v>26505</v>
-      </c>
-      <c r="T16" s="2"/>
+      <c r="S16" s="71">
+        <v>26651</v>
+      </c>
+      <c r="T16" s="70"/>
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>438</v>
+        <v>8</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>510</v>
+        <v>530</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>351</v>
@@ -3658,34 +3676,40 @@
         <v>103</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>439</v>
+        <v>83</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>368</v>
       </c>
-      <c r="H17" s="10"/>
-      <c r="I17" s="2"/>
+      <c r="H17" s="2">
+        <v>-80.459909999999994</v>
+      </c>
+      <c r="I17" s="2">
+        <v>39.062240000000003</v>
+      </c>
       <c r="J17" s="2" t="s">
-        <v>10</v>
+        <v>271</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="L17" s="2"/>
+        <v>9</v>
+      </c>
+      <c r="L17" s="34">
+        <v>10364</v>
+      </c>
       <c r="M17" s="33" t="s">
         <v>337</v>
       </c>
-      <c r="N17" s="33">
-        <v>12</v>
+      <c r="N17" s="34">
+        <v>24</v>
       </c>
       <c r="O17" s="34">
         <v>25</v>
       </c>
       <c r="P17" s="34">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="Q17" s="2" t="s">
         <v>347</v>
@@ -3694,16 +3718,16 @@
         <v>20</v>
       </c>
       <c r="S17" s="4">
-        <v>26505</v>
+        <v>26452</v>
       </c>
       <c r="T17" s="2"/>
     </row>
     <row r="18" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>432</v>
+        <v>52</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>510</v>
+        <v>613</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>351</v>
@@ -3712,34 +3736,40 @@
         <v>103</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>433</v>
+        <v>84</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>368</v>
       </c>
-      <c r="H18" s="10"/>
-      <c r="I18" s="2"/>
+      <c r="H18" s="2">
+        <v>-80.778989999999993</v>
+      </c>
+      <c r="I18" s="32">
+        <v>39.299059999999997</v>
+      </c>
       <c r="J18" s="2" t="s">
-        <v>10</v>
+        <v>272</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="L18" s="2"/>
+        <v>57</v>
+      </c>
+      <c r="L18" s="34">
+        <v>564</v>
+      </c>
       <c r="M18" s="33" t="s">
         <v>337</v>
       </c>
-      <c r="N18" s="33">
-        <v>12</v>
+      <c r="N18" s="34">
+        <v>24</v>
       </c>
       <c r="O18" s="34">
         <v>25</v>
       </c>
       <c r="P18" s="34">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="Q18" s="2" t="s">
         <v>347</v>
@@ -3748,16 +3778,16 @@
         <v>20</v>
       </c>
       <c r="S18" s="4">
-        <v>26505</v>
+        <v>26456</v>
       </c>
       <c r="T18" s="2"/>
     </row>
     <row r="19" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>509</v>
+        <v>531</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>351</v>
@@ -3766,7 +3796,7 @@
         <v>103</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>137</v>
+        <v>85</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>340</v>
@@ -3775,19 +3805,19 @@
         <v>369</v>
       </c>
       <c r="H19" s="2">
-        <v>-79.992055399999998</v>
+        <v>-80.72757</v>
       </c>
       <c r="I19" s="2">
-        <v>39.655174500000001</v>
+        <v>40.055880000000002</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>231</v>
+        <v>273</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="L19" s="34">
-        <v>48328</v>
+        <v>50000</v>
       </c>
       <c r="M19" s="34" t="s">
         <v>338</v>
@@ -3804,76 +3834,76 @@
         <v>20</v>
       </c>
       <c r="S19" s="4">
-        <v>26505</v>
+        <v>26003</v>
       </c>
       <c r="T19" s="2"/>
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A20" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>530</v>
-      </c>
-      <c r="C20" s="2" t="s">
+      <c r="A20" s="10" t="s">
+        <v>442</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>508</v>
+      </c>
+      <c r="C20" s="10" t="s">
         <v>351</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D20" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="E20" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="F20" s="2" t="s">
+      <c r="E20" s="10" t="s">
+        <v>443</v>
+      </c>
+      <c r="F20" s="10" t="s">
         <v>340</v>
       </c>
-      <c r="G20" s="2" t="s">
+      <c r="G20" s="10" t="s">
         <v>368</v>
       </c>
-      <c r="H20" s="2">
-        <v>-80.459909999999994</v>
-      </c>
-      <c r="I20" s="2">
-        <v>39.062240000000003</v>
-      </c>
-      <c r="J20" s="2" t="s">
-        <v>271</v>
-      </c>
-      <c r="K20" s="2" t="s">
-        <v>9</v>
+      <c r="H20" s="10">
+        <v>-81.165005500000007</v>
+      </c>
+      <c r="I20" s="10">
+        <v>37.946770700000002</v>
+      </c>
+      <c r="J20" s="10" t="s">
+        <v>549</v>
+      </c>
+      <c r="K20" s="10" t="s">
+        <v>197</v>
       </c>
       <c r="L20" s="34">
-        <v>10364</v>
+        <v>2626</v>
       </c>
       <c r="M20" s="33" t="s">
         <v>337</v>
       </c>
-      <c r="N20" s="34">
+      <c r="N20" s="35">
         <v>24</v>
       </c>
-      <c r="O20" s="34">
+      <c r="O20" s="35">
         <v>25</v>
       </c>
-      <c r="P20" s="34">
+      <c r="P20" s="35">
+        <v>30</v>
+      </c>
+      <c r="Q20" s="27" t="s">
+        <v>347</v>
+      </c>
+      <c r="R20" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="Q20" s="2" t="s">
-        <v>347</v>
-      </c>
-      <c r="R20" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="S20" s="4">
-        <v>26452</v>
-      </c>
-      <c r="T20" s="2"/>
+      <c r="S20" s="15">
+        <v>25917</v>
+      </c>
+      <c r="T20" s="10"/>
     </row>
     <row r="21" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>52</v>
+        <v>639</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>613</v>
+        <v>510</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>351</v>
@@ -3882,40 +3912,38 @@
         <v>103</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>84</v>
+        <v>640</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>368</v>
       </c>
       <c r="H21" s="2">
-        <v>-80.778989999999993</v>
-      </c>
-      <c r="I21" s="32">
-        <v>39.299059999999997</v>
+        <v>-79.972157499999994</v>
+      </c>
+      <c r="I21" s="2">
+        <v>39.650096900000001</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>272</v>
+        <v>10</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="L21" s="34">
-        <v>564</v>
-      </c>
-      <c r="M21" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="L21" s="34"/>
+      <c r="M21" s="34" t="s">
         <v>337</v>
       </c>
       <c r="N21" s="34">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="O21" s="34">
         <v>25</v>
       </c>
       <c r="P21" s="34">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="Q21" s="2" t="s">
         <v>347</v>
@@ -3924,15 +3952,18 @@
         <v>20</v>
       </c>
       <c r="S21" s="4">
-        <v>26456</v>
+        <v>26505</v>
+      </c>
+      <c r="T21" s="2" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>2</v>
+        <v>436</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>531</v>
+        <v>510</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>351</v>
@@ -3941,51 +3972,49 @@
         <v>103</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>85</v>
+        <v>437</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>369</v>
-      </c>
-      <c r="H22" s="2">
-        <v>-80.72757</v>
-      </c>
-      <c r="I22" s="2">
-        <v>40.055880000000002</v>
-      </c>
+        <v>368</v>
+      </c>
+      <c r="H22" s="10"/>
+      <c r="I22" s="2"/>
       <c r="J22" s="2" t="s">
-        <v>273</v>
+        <v>10</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="L22" s="34">
-        <v>50000</v>
-      </c>
-      <c r="M22" s="34" t="s">
-        <v>338</v>
-      </c>
-      <c r="N22" s="34">
-        <v>24</v>
-      </c>
-      <c r="O22" s="34"/>
-      <c r="P22" s="34"/>
+        <v>11</v>
+      </c>
+      <c r="L22" s="2"/>
+      <c r="M22" s="33" t="s">
+        <v>337</v>
+      </c>
+      <c r="N22" s="33">
+        <v>12</v>
+      </c>
+      <c r="O22" s="34">
+        <v>25</v>
+      </c>
+      <c r="P22" s="34">
+        <v>30</v>
+      </c>
       <c r="Q22" s="2" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="R22" s="2" t="s">
         <v>20</v>
       </c>
       <c r="S22" s="4">
-        <v>26003</v>
+        <v>26505</v>
       </c>
       <c r="T22" s="2"/>
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>639</v>
+        <v>434</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>510</v>
@@ -3997,7 +4026,7 @@
         <v>103</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>640</v>
+        <v>435</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>341</v>
@@ -4005,24 +4034,20 @@
       <c r="G23" s="2" t="s">
         <v>368</v>
       </c>
-      <c r="H23" s="2">
-        <v>-79.972157499999994</v>
-      </c>
-      <c r="I23" s="2">
-        <v>39.650096900000001</v>
-      </c>
+      <c r="H23" s="10"/>
+      <c r="I23" s="2"/>
       <c r="J23" s="2" t="s">
         <v>10</v>
       </c>
       <c r="K23" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="L23" s="34"/>
-      <c r="M23" s="34" t="s">
+      <c r="L23" s="2"/>
+      <c r="M23" s="33" t="s">
         <v>337</v>
       </c>
-      <c r="N23" s="34">
-        <v>48</v>
+      <c r="N23" s="33">
+        <v>12</v>
       </c>
       <c r="O23" s="34">
         <v>25</v>
@@ -4039,13 +4064,11 @@
       <c r="S23" s="4">
         <v>26505</v>
       </c>
-      <c r="T23" s="2" t="s">
-        <v>130</v>
-      </c>
+      <c r="T23" s="2"/>
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>637</v>
+        <v>438</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>510</v>
@@ -4057,15 +4080,15 @@
         <v>103</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>638</v>
+        <v>439</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>19</v>
+        <v>341</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>368</v>
       </c>
-      <c r="H24" s="2"/>
+      <c r="H24" s="10"/>
       <c r="I24" s="2"/>
       <c r="J24" s="2" t="s">
         <v>10</v>
@@ -4073,12 +4096,12 @@
       <c r="K24" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="L24" s="34"/>
-      <c r="M24" s="34" t="s">
+      <c r="L24" s="2"/>
+      <c r="M24" s="33" t="s">
         <v>337</v>
       </c>
-      <c r="N24" s="34">
-        <v>48</v>
+      <c r="N24" s="33">
+        <v>12</v>
       </c>
       <c r="O24" s="34">
         <v>25</v>
@@ -4098,122 +4121,113 @@
       <c r="T24" s="2"/>
     </row>
     <row r="25" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="10" t="s">
-        <v>442</v>
-      </c>
-      <c r="B25" s="10" t="s">
-        <v>508</v>
-      </c>
-      <c r="C25" s="10" t="s">
+      <c r="A25" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>351</v>
       </c>
-      <c r="D25" s="15" t="s">
+      <c r="D25" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="E25" s="10" t="s">
-        <v>443</v>
-      </c>
-      <c r="F25" s="10" t="s">
-        <v>340</v>
-      </c>
-      <c r="G25" s="10" t="s">
+      <c r="E25" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="G25" s="2" t="s">
         <v>368</v>
       </c>
-      <c r="H25" s="10">
-        <v>-81.165005500000007</v>
-      </c>
-      <c r="I25" s="10">
-        <v>37.946770700000002</v>
-      </c>
-      <c r="J25" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="K25" s="10" t="s">
-        <v>197</v>
-      </c>
-      <c r="L25" s="34">
-        <v>2626</v>
+      <c r="H25" s="10"/>
+      <c r="J25" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K25" s="2" t="s">
+        <v>11</v>
       </c>
       <c r="M25" s="33" t="s">
         <v>337</v>
       </c>
-      <c r="N25" s="35">
-        <v>24</v>
-      </c>
-      <c r="O25" s="35">
+      <c r="N25" s="33">
+        <v>12</v>
+      </c>
+      <c r="O25" s="34">
         <v>25</v>
       </c>
-      <c r="P25" s="35">
+      <c r="P25" s="34">
         <v>30</v>
       </c>
-      <c r="Q25" s="27" t="s">
+      <c r="Q25" s="2" t="s">
         <v>347</v>
       </c>
-      <c r="R25" s="10" t="s">
+      <c r="R25" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="S25" s="15">
-        <v>25917</v>
-      </c>
-      <c r="T25" s="10"/>
+      <c r="S25" s="4">
+        <v>26505</v>
+      </c>
     </row>
     <row r="26" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="26" t="s">
-        <v>167</v>
-      </c>
-      <c r="B26" s="26"/>
-      <c r="C26" s="26" t="s">
-        <v>352</v>
-      </c>
-      <c r="D26" s="29" t="s">
+      <c r="A26" s="2" t="s">
+        <v>637</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="D26" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="E26" s="26" t="s">
-        <v>68</v>
-      </c>
-      <c r="F26" s="26" t="s">
-        <v>340</v>
-      </c>
-      <c r="G26" s="26" t="s">
+      <c r="E26" s="2" t="s">
+        <v>638</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G26" s="2" t="s">
         <v>368</v>
       </c>
-      <c r="H26" s="26">
-        <v>-81.679554234298493</v>
-      </c>
-      <c r="I26" s="26">
-        <v>38.373735533484897</v>
-      </c>
-      <c r="J26" s="26" t="s">
-        <v>357</v>
-      </c>
-      <c r="K26" s="26" t="s">
-        <v>1</v>
-      </c>
-      <c r="L26" s="30">
-        <v>49500</v>
-      </c>
-      <c r="M26" s="31" t="s">
-        <v>338</v>
-      </c>
-      <c r="N26" s="31">
-        <v>24</v>
-      </c>
-      <c r="O26" s="31"/>
-      <c r="P26" s="31"/>
-      <c r="Q26" s="26" t="s">
-        <v>348</v>
-      </c>
-      <c r="R26" s="26" t="s">
+      <c r="H26" s="2"/>
+      <c r="I26" s="2"/>
+      <c r="J26" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="L26" s="34"/>
+      <c r="M26" s="34" t="s">
+        <v>337</v>
+      </c>
+      <c r="N26" s="34">
+        <v>48</v>
+      </c>
+      <c r="O26" s="34">
+        <v>25</v>
+      </c>
+      <c r="P26" s="34">
+        <v>30</v>
+      </c>
+      <c r="Q26" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="R26" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="S26" s="36">
-        <v>25387</v>
-      </c>
-      <c r="T26" s="26"/>
+      <c r="S26" s="4">
+        <v>26505</v>
+      </c>
+      <c r="T26" s="2"/>
     </row>
     <row r="27" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A27" s="26" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="B27" s="26"/>
       <c r="C27" s="26" t="s">
@@ -4223,7 +4237,7 @@
         <v>103</v>
       </c>
       <c r="E27" s="26" t="s">
-        <v>162</v>
+        <v>68</v>
       </c>
       <c r="F27" s="26" t="s">
         <v>340</v>
@@ -4232,19 +4246,19 @@
         <v>368</v>
       </c>
       <c r="H27" s="26">
-        <v>-81.758709180509001</v>
+        <v>-81.679554234298493</v>
       </c>
       <c r="I27" s="26">
-        <v>38.368519014596998</v>
+        <v>38.373735533484897</v>
       </c>
       <c r="J27" s="26" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="K27" s="26" t="s">
         <v>1</v>
       </c>
       <c r="L27" s="30">
-        <v>9000</v>
+        <v>49500</v>
       </c>
       <c r="M27" s="31" t="s">
         <v>338</v>
@@ -4252,26 +4266,22 @@
       <c r="N27" s="31">
         <v>24</v>
       </c>
-      <c r="O27" s="31">
-        <v>25</v>
-      </c>
-      <c r="P27" s="31">
-        <v>20</v>
-      </c>
+      <c r="O27" s="31"/>
+      <c r="P27" s="31"/>
       <c r="Q27" s="26" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="R27" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="S27" s="29">
-        <v>25064</v>
+      <c r="S27" s="36">
+        <v>25387</v>
       </c>
       <c r="T27" s="26"/>
     </row>
     <row r="28" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A28" s="26" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="B28" s="26"/>
       <c r="C28" s="26" t="s">
@@ -4281,7 +4291,7 @@
         <v>103</v>
       </c>
       <c r="E28" s="26" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="F28" s="26" t="s">
         <v>340</v>
@@ -4290,19 +4300,19 @@
         <v>368</v>
       </c>
       <c r="H28" s="26">
-        <v>-82.528864034905197</v>
+        <v>-81.758709180509001</v>
       </c>
       <c r="I28" s="26">
-        <v>38.400744931017101</v>
+        <v>38.368519014596998</v>
       </c>
       <c r="J28" s="26" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="K28" s="26" t="s">
-        <v>164</v>
+        <v>1</v>
       </c>
       <c r="L28" s="30">
-        <v>56000</v>
+        <v>9000</v>
       </c>
       <c r="M28" s="31" t="s">
         <v>338</v>
@@ -4322,14 +4332,14 @@
       <c r="R28" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="S28" s="36">
-        <v>25704</v>
+      <c r="S28" s="29">
+        <v>25064</v>
       </c>
       <c r="T28" s="26"/>
     </row>
     <row r="29" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A29" s="26" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="B29" s="26"/>
       <c r="C29" s="26" t="s">
@@ -4339,7 +4349,7 @@
         <v>103</v>
       </c>
       <c r="E29" s="26" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="F29" s="26" t="s">
         <v>340</v>
@@ -4348,22 +4358,22 @@
         <v>368</v>
       </c>
       <c r="H29" s="26">
-        <v>-82.298209254857795</v>
+        <v>-82.528864034905197</v>
       </c>
       <c r="I29" s="26">
-        <v>38.419661908139098</v>
+        <v>38.400744931017101</v>
       </c>
       <c r="J29" s="26" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="K29" s="26" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="L29" s="30">
-        <v>7000</v>
+        <v>56000</v>
       </c>
       <c r="M29" s="31" t="s">
-        <v>583</v>
+        <v>338</v>
       </c>
       <c r="N29" s="31">
         <v>24</v>
@@ -4380,132 +4390,130 @@
       <c r="R29" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="S29" s="29">
+      <c r="S29" s="36">
+        <v>25704</v>
+      </c>
+      <c r="T29" s="26"/>
+    </row>
+    <row r="30" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="26" t="s">
+        <v>171</v>
+      </c>
+      <c r="B30" s="26"/>
+      <c r="C30" s="26" t="s">
+        <v>352</v>
+      </c>
+      <c r="D30" s="29" t="s">
+        <v>103</v>
+      </c>
+      <c r="E30" s="26" t="s">
+        <v>161</v>
+      </c>
+      <c r="F30" s="26" t="s">
+        <v>340</v>
+      </c>
+      <c r="G30" s="26" t="s">
+        <v>368</v>
+      </c>
+      <c r="H30" s="26">
+        <v>-82.298209254857795</v>
+      </c>
+      <c r="I30" s="26">
+        <v>38.419661908139098</v>
+      </c>
+      <c r="J30" s="26" t="s">
+        <v>355</v>
+      </c>
+      <c r="K30" s="26" t="s">
+        <v>157</v>
+      </c>
+      <c r="L30" s="30">
+        <v>7000</v>
+      </c>
+      <c r="M30" s="31" t="s">
+        <v>583</v>
+      </c>
+      <c r="N30" s="31">
+        <v>24</v>
+      </c>
+      <c r="O30" s="31">
+        <v>25</v>
+      </c>
+      <c r="P30" s="31">
+        <v>20</v>
+      </c>
+      <c r="Q30" s="26" t="s">
+        <v>347</v>
+      </c>
+      <c r="R30" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="S30" s="29">
         <v>25705</v>
       </c>
-      <c r="T29" s="26"/>
-    </row>
-    <row r="30" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="39" t="s">
+      <c r="T30" s="26"/>
+    </row>
+    <row r="31" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="39" t="s">
         <v>575</v>
       </c>
-      <c r="B30" s="39"/>
-      <c r="C30" s="39" t="s">
+      <c r="B31" s="39"/>
+      <c r="C31" s="39" t="s">
         <v>352</v>
       </c>
-      <c r="D30" s="40" t="s">
+      <c r="D31" s="40" t="s">
         <v>103</v>
       </c>
-      <c r="E30" s="39" t="s">
+      <c r="E31" s="39" t="s">
         <v>576</v>
       </c>
-      <c r="F30" s="39" t="s">
+      <c r="F31" s="39" t="s">
         <v>340</v>
       </c>
-      <c r="G30" s="39" t="s">
+      <c r="G31" s="39" t="s">
         <v>368</v>
       </c>
-      <c r="H30" s="39">
+      <c r="H31" s="39">
         <v>-81.867118796822695</v>
       </c>
-      <c r="I30" s="39">
+      <c r="I31" s="39">
         <v>38.537901317549398</v>
       </c>
-      <c r="J30" s="39" t="s">
+      <c r="J31" s="39" t="s">
         <v>577</v>
       </c>
-      <c r="K30" s="39" t="s">
+      <c r="K31" s="39" t="s">
         <v>159</v>
       </c>
-      <c r="L30" s="41">
+      <c r="L31" s="41">
         <v>4900</v>
       </c>
-      <c r="M30" s="42" t="s">
+      <c r="M31" s="42" t="s">
         <v>338</v>
       </c>
-      <c r="N30" s="42">
+      <c r="N31" s="42">
         <v>48</v>
       </c>
-      <c r="O30" s="42">
+      <c r="O31" s="42">
         <v>333</v>
       </c>
-      <c r="P30" s="42">
+      <c r="P31" s="42">
         <v>1440</v>
       </c>
-      <c r="Q30" s="39" t="s">
+      <c r="Q31" s="39" t="s">
         <v>347</v>
       </c>
-      <c r="R30" s="39" t="s">
+      <c r="R31" s="39" t="s">
         <v>20</v>
       </c>
-      <c r="S30" s="40">
+      <c r="S31" s="40">
         <v>25168</v>
       </c>
-      <c r="T30" s="39"/>
-    </row>
-    <row r="31" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="26" t="s">
-        <v>580</v>
-      </c>
-      <c r="B31" s="26"/>
-      <c r="C31" s="26" t="s">
-        <v>352</v>
-      </c>
-      <c r="D31" s="29" t="s">
-        <v>103</v>
-      </c>
-      <c r="E31" s="26" t="s">
-        <v>573</v>
-      </c>
-      <c r="F31" s="26" t="s">
-        <v>340</v>
-      </c>
-      <c r="G31" s="26" t="s">
-        <v>368</v>
-      </c>
-      <c r="H31" s="26">
-        <v>-82.105144999999993</v>
-      </c>
-      <c r="I31" s="26">
-        <v>38.425437000000002</v>
-      </c>
-      <c r="J31" s="26" t="s">
-        <v>370</v>
-      </c>
-      <c r="K31" s="26" t="s">
-        <v>157</v>
-      </c>
-      <c r="L31" s="30">
-        <v>7200</v>
-      </c>
-      <c r="M31" s="31" t="s">
-        <v>338</v>
-      </c>
-      <c r="N31" s="31">
-        <v>24</v>
-      </c>
-      <c r="O31" s="31">
-        <v>25</v>
-      </c>
-      <c r="P31" s="31">
-        <v>20</v>
-      </c>
-      <c r="Q31" s="26" t="s">
-        <v>347</v>
-      </c>
-      <c r="R31" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="S31" s="29">
-        <v>25541</v>
-      </c>
-      <c r="T31" s="26" t="s">
-        <v>160</v>
-      </c>
+      <c r="T31" s="39"/>
     </row>
     <row r="32" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A32" s="26" t="s">
-        <v>170</v>
+        <v>580</v>
       </c>
       <c r="B32" s="26"/>
       <c r="C32" s="26" t="s">
@@ -4515,7 +4523,7 @@
         <v>103</v>
       </c>
       <c r="E32" s="26" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="F32" s="26" t="s">
         <v>340</v>
@@ -4524,19 +4532,19 @@
         <v>368</v>
       </c>
       <c r="H32" s="26">
-        <v>-82.244877751268803</v>
+        <v>-82.105144999999993</v>
       </c>
       <c r="I32" s="26">
-        <v>38.372162360135</v>
+        <v>38.425437000000002</v>
       </c>
       <c r="J32" s="26" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="K32" s="26" t="s">
         <v>157</v>
       </c>
       <c r="L32" s="30">
-        <v>4050</v>
+        <v>7200</v>
       </c>
       <c r="M32" s="31" t="s">
         <v>338</v>
@@ -4557,65 +4565,70 @@
         <v>20</v>
       </c>
       <c r="S32" s="29">
-        <v>25545</v>
+        <v>25541</v>
       </c>
       <c r="T32" s="26" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="33" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="61" t="s">
-        <v>35</v>
-      </c>
-      <c r="B33" s="61" t="s">
-        <v>511</v>
-      </c>
-      <c r="C33" s="61" t="s">
-        <v>351</v>
-      </c>
-      <c r="D33" s="62" t="s">
-        <v>60</v>
-      </c>
-      <c r="E33" s="61" t="s">
-        <v>66</v>
-      </c>
-      <c r="F33" s="61" t="s">
-        <v>34</v>
-      </c>
-      <c r="G33" s="61" t="s">
+      <c r="A33" s="26" t="s">
+        <v>170</v>
+      </c>
+      <c r="B33" s="26"/>
+      <c r="C33" s="26" t="s">
+        <v>352</v>
+      </c>
+      <c r="D33" s="29" t="s">
+        <v>103</v>
+      </c>
+      <c r="E33" s="26" t="s">
+        <v>572</v>
+      </c>
+      <c r="F33" s="26" t="s">
+        <v>340</v>
+      </c>
+      <c r="G33" s="26" t="s">
         <v>368</v>
       </c>
-      <c r="H33" s="61">
-        <v>-79.905010000000004</v>
-      </c>
-      <c r="I33" s="61">
-        <v>39.610210000000002</v>
-      </c>
-      <c r="J33" s="61" t="s">
-        <v>231</v>
-      </c>
-      <c r="K33" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="L33" s="63">
-        <v>579</v>
-      </c>
-      <c r="M33" s="63" t="s">
-        <v>337</v>
-      </c>
-      <c r="N33" s="63">
-        <v>8</v>
-      </c>
-      <c r="O33" s="63"/>
-      <c r="P33" s="63"/>
-      <c r="Q33" s="61" t="s">
+      <c r="H33" s="26">
+        <v>-82.244877751268803</v>
+      </c>
+      <c r="I33" s="26">
+        <v>38.372162360135</v>
+      </c>
+      <c r="J33" s="26" t="s">
+        <v>371</v>
+      </c>
+      <c r="K33" s="26" t="s">
+        <v>157</v>
+      </c>
+      <c r="L33" s="30">
+        <v>4050</v>
+      </c>
+      <c r="M33" s="31" t="s">
+        <v>338</v>
+      </c>
+      <c r="N33" s="31">
+        <v>24</v>
+      </c>
+      <c r="O33" s="31">
+        <v>25</v>
+      </c>
+      <c r="P33" s="31">
+        <v>20</v>
+      </c>
+      <c r="Q33" s="26" t="s">
         <v>347</v>
       </c>
-      <c r="R33" s="61" t="s">
+      <c r="R33" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="S33" s="62">
-        <v>26508</v>
+      <c r="S33" s="29">
+        <v>25545</v>
+      </c>
+      <c r="T33" s="26" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="34" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
@@ -4675,10 +4688,10 @@
     </row>
     <row r="35" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A35" s="61" t="s">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="B35" s="61" t="s">
-        <v>511</v>
+        <v>526</v>
       </c>
       <c r="C35" s="61" t="s">
         <v>351</v>
@@ -4687,37 +4700,41 @@
         <v>60</v>
       </c>
       <c r="E35" s="61" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="F35" s="61" t="s">
-        <v>34</v>
+        <v>340</v>
       </c>
       <c r="G35" s="61" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="H35" s="61">
-        <v>-79.867609999999999</v>
+        <v>-81.079930000000004</v>
       </c>
       <c r="I35" s="61">
-        <v>39.652670000000001</v>
+        <v>37.380360000000003</v>
       </c>
       <c r="J35" s="61" t="s">
-        <v>231</v>
+        <v>265</v>
       </c>
       <c r="K35" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="L35" s="63">
-        <v>830</v>
+        <v>17</v>
+      </c>
+      <c r="L35" s="64">
+        <v>36000</v>
       </c>
       <c r="M35" s="63" t="s">
-        <v>337</v>
-      </c>
-      <c r="N35" s="63">
-        <v>8</v>
-      </c>
-      <c r="O35" s="63"/>
-      <c r="P35" s="63"/>
+        <v>342</v>
+      </c>
+      <c r="N35" s="64">
+        <v>24</v>
+      </c>
+      <c r="O35" s="64">
+        <v>25</v>
+      </c>
+      <c r="P35" s="64">
+        <v>20</v>
+      </c>
       <c r="Q35" s="61" t="s">
         <v>347</v>
       </c>
@@ -4725,15 +4742,15 @@
         <v>20</v>
       </c>
       <c r="S35" s="62">
-        <v>26508</v>
+        <v>24740</v>
       </c>
     </row>
     <row r="36" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A36" s="61" t="s">
-        <v>440</v>
+        <v>106</v>
       </c>
       <c r="B36" s="61" t="s">
-        <v>510</v>
+        <v>527</v>
       </c>
       <c r="C36" s="61" t="s">
         <v>351</v>
@@ -4742,38 +4759,40 @@
         <v>60</v>
       </c>
       <c r="E36" s="61" t="s">
-        <v>441</v>
+        <v>107</v>
       </c>
       <c r="F36" s="61" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="G36" s="61" t="s">
         <v>368</v>
       </c>
       <c r="H36" s="61">
-        <v>-79.985057699999999</v>
-      </c>
-      <c r="I36" s="61">
-        <v>39.648165400000003</v>
+        <v>-80.545150000000007</v>
+      </c>
+      <c r="I36" s="65">
+        <v>39.285969999999999</v>
       </c>
       <c r="J36" s="61" t="s">
-        <v>10</v>
+        <v>266</v>
       </c>
       <c r="K36" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="L36" s="63"/>
+        <v>88</v>
+      </c>
+      <c r="L36" s="64">
+        <v>1853</v>
+      </c>
       <c r="M36" s="63" t="s">
         <v>337</v>
       </c>
-      <c r="N36" s="63">
-        <v>8</v>
+      <c r="N36" s="64">
+        <v>24</v>
       </c>
       <c r="O36" s="64">
         <v>25</v>
       </c>
       <c r="P36" s="64">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="Q36" s="61" t="s">
         <v>347</v>
@@ -4782,12 +4801,12 @@
         <v>20</v>
       </c>
       <c r="S36" s="62">
-        <v>26505</v>
+        <v>26426</v>
       </c>
     </row>
     <row r="37" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A37" s="61" t="s">
-        <v>21</v>
+        <v>440</v>
       </c>
       <c r="B37" s="61" t="s">
         <v>510</v>
@@ -4799,39 +4818,37 @@
         <v>60</v>
       </c>
       <c r="E37" s="61" t="s">
-        <v>187</v>
+        <v>441</v>
       </c>
       <c r="F37" s="61" t="s">
-        <v>19</v>
+        <v>341</v>
       </c>
       <c r="G37" s="61" t="s">
         <v>368</v>
       </c>
       <c r="H37" s="61">
-        <v>-79.945801900000006</v>
+        <v>-79.985057699999999</v>
       </c>
       <c r="I37" s="61">
-        <v>39.6362083</v>
+        <v>39.648165400000003</v>
       </c>
       <c r="J37" s="61" t="s">
-        <v>231</v>
+        <v>10</v>
       </c>
       <c r="K37" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="L37" s="63">
-        <v>567</v>
-      </c>
+      <c r="L37" s="63"/>
       <c r="M37" s="63" t="s">
         <v>337</v>
       </c>
       <c r="N37" s="63">
-        <v>48</v>
-      </c>
-      <c r="O37" s="63">
+        <v>8</v>
+      </c>
+      <c r="O37" s="64">
         <v>25</v>
       </c>
-      <c r="P37" s="63">
+      <c r="P37" s="64">
         <v>30</v>
       </c>
       <c r="Q37" s="61" t="s">
@@ -4843,13 +4860,10 @@
       <c r="S37" s="62">
         <v>26505</v>
       </c>
-      <c r="T37" s="61" t="s">
-        <v>131</v>
-      </c>
     </row>
     <row r="38" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A38" s="61" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B38" s="61" t="s">
         <v>510</v>
@@ -4861,19 +4875,19 @@
         <v>60</v>
       </c>
       <c r="E38" s="61" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="F38" s="61" t="s">
-        <v>19</v>
+        <v>341</v>
       </c>
       <c r="G38" s="61" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="H38" s="61">
-        <v>-79.953093199999998</v>
+        <v>-79.972157499999994</v>
       </c>
       <c r="I38" s="61">
-        <v>39.636423100000002</v>
+        <v>39.650096900000001</v>
       </c>
       <c r="J38" s="61" t="s">
         <v>231</v>
@@ -4881,9 +4895,7 @@
       <c r="K38" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="L38" s="63">
-        <v>639</v>
-      </c>
+      <c r="L38" s="63"/>
       <c r="M38" s="63" t="s">
         <v>337</v>
       </c>
@@ -4906,15 +4918,15 @@
         <v>26505</v>
       </c>
       <c r="T38" s="61" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="39" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A39" s="61" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="B39" s="61" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="C39" s="61" t="s">
         <v>351</v>
@@ -4923,19 +4935,19 @@
         <v>60</v>
       </c>
       <c r="E39" s="61" t="s">
-        <v>143</v>
+        <v>66</v>
       </c>
       <c r="F39" s="61" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="G39" s="61" t="s">
         <v>368</v>
       </c>
       <c r="H39" s="61">
-        <v>-80.000420899999995</v>
+        <v>-79.905010000000004</v>
       </c>
       <c r="I39" s="61">
-        <v>39.6535571</v>
+        <v>39.610210000000002</v>
       </c>
       <c r="J39" s="61" t="s">
         <v>231</v>
@@ -4944,20 +4956,16 @@
         <v>11</v>
       </c>
       <c r="L39" s="63">
-        <v>912</v>
+        <v>579</v>
       </c>
       <c r="M39" s="63" t="s">
         <v>337</v>
       </c>
       <c r="N39" s="63">
-        <v>48</v>
-      </c>
-      <c r="O39" s="63">
-        <v>25</v>
-      </c>
-      <c r="P39" s="63">
-        <v>30</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="O39" s="63"/>
+      <c r="P39" s="63"/>
       <c r="Q39" s="61" t="s">
         <v>347</v>
       </c>
@@ -4965,18 +4973,15 @@
         <v>20</v>
       </c>
       <c r="S39" s="62">
-        <v>26505</v>
-      </c>
-      <c r="T39" s="61" t="s">
-        <v>135</v>
+        <v>26508</v>
       </c>
     </row>
     <row r="40" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A40" s="61" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="B40" s="61" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="C40" s="61" t="s">
         <v>351</v>
@@ -4985,19 +4990,19 @@
         <v>60</v>
       </c>
       <c r="E40" s="61" t="s">
-        <v>138</v>
+        <v>70</v>
       </c>
       <c r="F40" s="61" t="s">
-        <v>341</v>
+        <v>34</v>
       </c>
       <c r="G40" s="61" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="H40" s="61">
-        <v>-79.972157499999994</v>
+        <v>-79.867609999999999</v>
       </c>
       <c r="I40" s="61">
-        <v>39.650096900000001</v>
+        <v>39.652670000000001</v>
       </c>
       <c r="J40" s="61" t="s">
         <v>231</v>
@@ -5005,19 +5010,17 @@
       <c r="K40" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="L40" s="63"/>
+      <c r="L40" s="63">
+        <v>830</v>
+      </c>
       <c r="M40" s="63" t="s">
         <v>337</v>
       </c>
       <c r="N40" s="63">
-        <v>48</v>
-      </c>
-      <c r="O40" s="63">
-        <v>25</v>
-      </c>
-      <c r="P40" s="63">
-        <v>30</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="O40" s="63"/>
+      <c r="P40" s="63"/>
       <c r="Q40" s="61" t="s">
         <v>347</v>
       </c>
@@ -5025,18 +5028,15 @@
         <v>20</v>
       </c>
       <c r="S40" s="62">
-        <v>26505</v>
-      </c>
-      <c r="T40" s="61" t="s">
-        <v>130</v>
+        <v>26508</v>
       </c>
     </row>
     <row r="41" spans="1:20" s="61" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="61" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="B41" s="61" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="C41" s="61" t="s">
         <v>351</v>
@@ -5045,19 +5045,19 @@
         <v>60</v>
       </c>
       <c r="E41" s="61" t="s">
-        <v>145</v>
+        <v>72</v>
       </c>
       <c r="F41" s="61" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="G41" s="61" t="s">
         <v>368</v>
       </c>
       <c r="H41" s="61">
-        <v>-79.956234100000003</v>
+        <v>-79.957359999999994</v>
       </c>
       <c r="I41" s="61">
-        <v>39.667909799999997</v>
+        <v>39.625419999999998</v>
       </c>
       <c r="J41" s="61" t="s">
         <v>231</v>
@@ -5065,19 +5065,17 @@
       <c r="K41" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="L41" s="63"/>
+      <c r="L41" s="63">
+        <v>1851</v>
+      </c>
       <c r="M41" s="63" t="s">
         <v>337</v>
       </c>
       <c r="N41" s="63">
-        <v>48</v>
-      </c>
-      <c r="O41" s="63">
-        <v>25</v>
-      </c>
-      <c r="P41" s="63">
-        <v>30</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="O41" s="63"/>
+      <c r="P41" s="63"/>
       <c r="Q41" s="61" t="s">
         <v>347</v>
       </c>
@@ -5085,18 +5083,15 @@
         <v>20</v>
       </c>
       <c r="S41" s="62">
-        <v>26505</v>
-      </c>
-      <c r="T41" s="61" t="s">
-        <v>42</v>
+        <v>26501</v>
       </c>
     </row>
     <row r="42" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A42" s="61" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="B42" s="61" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="C42" s="61" t="s">
         <v>351</v>
@@ -5105,19 +5100,19 @@
         <v>60</v>
       </c>
       <c r="E42" s="61" t="s">
-        <v>144</v>
+        <v>74</v>
       </c>
       <c r="F42" s="61" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="G42" s="61" t="s">
         <v>368</v>
       </c>
       <c r="H42" s="61">
-        <v>-79.956204600000007</v>
+        <v>-79.943309999999997</v>
       </c>
       <c r="I42" s="61">
-        <v>39.668112200000003</v>
+        <v>39.61036</v>
       </c>
       <c r="J42" s="61" t="s">
         <v>231</v>
@@ -5125,19 +5120,17 @@
       <c r="K42" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="L42" s="63"/>
+      <c r="L42" s="63">
+        <v>726</v>
+      </c>
       <c r="M42" s="63" t="s">
         <v>337</v>
       </c>
       <c r="N42" s="63">
-        <v>48</v>
-      </c>
-      <c r="O42" s="63">
-        <v>25</v>
-      </c>
-      <c r="P42" s="63">
-        <v>30</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="O42" s="63"/>
+      <c r="P42" s="63"/>
       <c r="Q42" s="61" t="s">
         <v>347</v>
       </c>
@@ -5145,15 +5138,12 @@
         <v>20</v>
       </c>
       <c r="S42" s="62">
-        <v>26505</v>
-      </c>
-      <c r="T42" s="61" t="s">
-        <v>43</v>
+        <v>26501</v>
       </c>
     </row>
     <row r="43" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A43" s="61" t="s">
-        <v>192</v>
+        <v>36</v>
       </c>
       <c r="B43" s="61" t="s">
         <v>510</v>
@@ -5165,19 +5155,19 @@
         <v>60</v>
       </c>
       <c r="E43" s="61" t="s">
-        <v>139</v>
+        <v>75</v>
       </c>
       <c r="F43" s="61" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="G43" s="61" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="H43" s="61">
-        <v>-79.956762600000005</v>
+        <v>-79.956739999999996</v>
       </c>
       <c r="I43" s="61">
-        <v>39.637875299999997</v>
+        <v>39.660640000000001</v>
       </c>
       <c r="J43" s="61" t="s">
         <v>231</v>
@@ -5186,20 +5176,16 @@
         <v>11</v>
       </c>
       <c r="L43" s="63">
-        <v>874</v>
+        <v>688</v>
       </c>
       <c r="M43" s="63" t="s">
         <v>337</v>
       </c>
       <c r="N43" s="63">
-        <v>48</v>
-      </c>
-      <c r="O43" s="63">
-        <v>25</v>
-      </c>
-      <c r="P43" s="63">
-        <v>30</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="O43" s="63"/>
+      <c r="P43" s="63"/>
       <c r="Q43" s="61" t="s">
         <v>347</v>
       </c>
@@ -5209,16 +5195,13 @@
       <c r="S43" s="62">
         <v>26505</v>
       </c>
-      <c r="T43" s="61" t="s">
-        <v>132</v>
-      </c>
     </row>
     <row r="44" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A44" s="61" t="s">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="B44" s="61" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="C44" s="61" t="s">
         <v>351</v>
@@ -5227,19 +5210,19 @@
         <v>60</v>
       </c>
       <c r="E44" s="61" t="s">
-        <v>146</v>
+        <v>80</v>
       </c>
       <c r="F44" s="61" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="G44" s="61" t="s">
         <v>368</v>
       </c>
       <c r="H44" s="61">
-        <v>-79.955122099999997</v>
+        <v>-79.978250000000003</v>
       </c>
       <c r="I44" s="61">
-        <v>39.669188599999998</v>
+        <v>39.671370000000003</v>
       </c>
       <c r="J44" s="61" t="s">
         <v>231</v>
@@ -5247,19 +5230,17 @@
       <c r="K44" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="L44" s="63"/>
+      <c r="L44" s="63">
+        <v>515</v>
+      </c>
       <c r="M44" s="63" t="s">
         <v>337</v>
       </c>
       <c r="N44" s="63">
-        <v>48</v>
-      </c>
-      <c r="O44" s="63">
-        <v>25</v>
-      </c>
-      <c r="P44" s="63">
-        <v>30</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="O44" s="63"/>
+      <c r="P44" s="63"/>
       <c r="Q44" s="61" t="s">
         <v>347</v>
       </c>
@@ -5269,16 +5250,13 @@
       <c r="S44" s="62">
         <v>26505</v>
       </c>
-      <c r="T44" s="61" t="s">
-        <v>44</v>
-      </c>
     </row>
     <row r="45" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A45" s="61" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="B45" s="61" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="C45" s="61" t="s">
         <v>351</v>
@@ -5287,19 +5265,19 @@
         <v>60</v>
       </c>
       <c r="E45" s="61" t="s">
-        <v>147</v>
+        <v>81</v>
       </c>
       <c r="F45" s="61" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="G45" s="61" t="s">
         <v>368</v>
       </c>
       <c r="H45" s="61">
-        <v>-79.955245399999995</v>
+        <v>-79.926150000000007</v>
       </c>
       <c r="I45" s="61">
-        <v>39.669279500000002</v>
+        <v>39.687820000000002</v>
       </c>
       <c r="J45" s="61" t="s">
         <v>231</v>
@@ -5307,19 +5285,17 @@
       <c r="K45" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="L45" s="63"/>
+      <c r="L45" s="63">
+        <v>1310</v>
+      </c>
       <c r="M45" s="63" t="s">
         <v>337</v>
       </c>
       <c r="N45" s="63">
-        <v>48</v>
-      </c>
-      <c r="O45" s="63">
-        <v>25</v>
-      </c>
-      <c r="P45" s="63">
-        <v>30</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="O45" s="63"/>
+      <c r="P45" s="63"/>
       <c r="Q45" s="61" t="s">
         <v>347</v>
       </c>
@@ -5327,18 +5303,15 @@
         <v>20</v>
       </c>
       <c r="S45" s="62">
-        <v>26505</v>
-      </c>
-      <c r="T45" s="61" t="s">
-        <v>45</v>
+        <v>26508</v>
       </c>
     </row>
     <row r="46" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A46" s="61" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="B46" s="61" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="C46" s="61" t="s">
         <v>351</v>
@@ -5347,19 +5320,19 @@
         <v>60</v>
       </c>
       <c r="E46" s="61" t="s">
-        <v>72</v>
+        <v>187</v>
       </c>
       <c r="F46" s="61" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="G46" s="61" t="s">
         <v>368</v>
       </c>
       <c r="H46" s="61">
-        <v>-79.957359999999994</v>
+        <v>-79.945801900000006</v>
       </c>
       <c r="I46" s="61">
-        <v>39.625419999999998</v>
+        <v>39.6362083</v>
       </c>
       <c r="J46" s="61" t="s">
         <v>231</v>
@@ -5368,16 +5341,20 @@
         <v>11</v>
       </c>
       <c r="L46" s="63">
-        <v>1851</v>
+        <v>567</v>
       </c>
       <c r="M46" s="63" t="s">
         <v>337</v>
       </c>
       <c r="N46" s="63">
-        <v>8</v>
-      </c>
-      <c r="O46" s="63"/>
-      <c r="P46" s="63"/>
+        <v>48</v>
+      </c>
+      <c r="O46" s="63">
+        <v>25</v>
+      </c>
+      <c r="P46" s="63">
+        <v>30</v>
+      </c>
       <c r="Q46" s="61" t="s">
         <v>347</v>
       </c>
@@ -5385,15 +5362,18 @@
         <v>20</v>
       </c>
       <c r="S46" s="62">
-        <v>26501</v>
+        <v>26505</v>
+      </c>
+      <c r="T46" s="61" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="47" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A47" s="61" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="B47" s="61" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="C47" s="61" t="s">
         <v>351</v>
@@ -5402,19 +5382,19 @@
         <v>60</v>
       </c>
       <c r="E47" s="61" t="s">
-        <v>74</v>
+        <v>142</v>
       </c>
       <c r="F47" s="61" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="G47" s="61" t="s">
         <v>368</v>
       </c>
       <c r="H47" s="61">
-        <v>-79.943309999999997</v>
+        <v>-79.953093199999998</v>
       </c>
       <c r="I47" s="61">
-        <v>39.61036</v>
+        <v>39.636423100000002</v>
       </c>
       <c r="J47" s="61" t="s">
         <v>231</v>
@@ -5423,16 +5403,20 @@
         <v>11</v>
       </c>
       <c r="L47" s="63">
-        <v>726</v>
+        <v>639</v>
       </c>
       <c r="M47" s="63" t="s">
         <v>337</v>
       </c>
       <c r="N47" s="63">
-        <v>8</v>
-      </c>
-      <c r="O47" s="63"/>
-      <c r="P47" s="63"/>
+        <v>48</v>
+      </c>
+      <c r="O47" s="63">
+        <v>25</v>
+      </c>
+      <c r="P47" s="63">
+        <v>30</v>
+      </c>
       <c r="Q47" s="61" t="s">
         <v>347</v>
       </c>
@@ -5440,12 +5424,15 @@
         <v>20</v>
       </c>
       <c r="S47" s="62">
-        <v>26501</v>
+        <v>26505</v>
+      </c>
+      <c r="T47" s="61" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="48" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A48" s="61" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B48" s="61" t="s">
         <v>510</v>
@@ -5457,19 +5444,19 @@
         <v>60</v>
       </c>
       <c r="E48" s="61" t="s">
-        <v>183</v>
+        <v>143</v>
       </c>
       <c r="F48" s="61" t="s">
         <v>19</v>
       </c>
       <c r="G48" s="61" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="H48" s="61">
-        <v>-79.965769100000003</v>
+        <v>-80.000420899999995</v>
       </c>
       <c r="I48" s="61">
-        <v>39.672765599999998</v>
+        <v>39.6535571</v>
       </c>
       <c r="J48" s="61" t="s">
         <v>231</v>
@@ -5477,7 +5464,9 @@
       <c r="K48" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="L48" s="63"/>
+      <c r="L48" s="63">
+        <v>912</v>
+      </c>
       <c r="M48" s="63" t="s">
         <v>337</v>
       </c>
@@ -5500,12 +5489,12 @@
         <v>26505</v>
       </c>
       <c r="T48" s="61" t="s">
-        <v>46</v>
+        <v>135</v>
       </c>
     </row>
     <row r="49" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A49" s="61" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="B49" s="61" t="s">
         <v>510</v>
@@ -5517,19 +5506,19 @@
         <v>60</v>
       </c>
       <c r="E49" s="61" t="s">
-        <v>75</v>
+        <v>145</v>
       </c>
       <c r="F49" s="61" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="G49" s="61" t="s">
         <v>368</v>
       </c>
       <c r="H49" s="61">
-        <v>-79.956739999999996</v>
+        <v>-79.956234100000003</v>
       </c>
       <c r="I49" s="61">
-        <v>39.660640000000001</v>
+        <v>39.667909799999997</v>
       </c>
       <c r="J49" s="61" t="s">
         <v>231</v>
@@ -5537,17 +5526,19 @@
       <c r="K49" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="L49" s="63">
-        <v>688</v>
-      </c>
+      <c r="L49" s="63"/>
       <c r="M49" s="63" t="s">
         <v>337</v>
       </c>
       <c r="N49" s="63">
-        <v>8</v>
-      </c>
-      <c r="O49" s="63"/>
-      <c r="P49" s="63"/>
+        <v>48</v>
+      </c>
+      <c r="O49" s="63">
+        <v>25</v>
+      </c>
+      <c r="P49" s="63">
+        <v>30</v>
+      </c>
       <c r="Q49" s="61" t="s">
         <v>347</v>
       </c>
@@ -5557,10 +5548,13 @@
       <c r="S49" s="62">
         <v>26505</v>
       </c>
+      <c r="T49" s="61" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="50" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A50" s="61" t="s">
-        <v>339</v>
+        <v>28</v>
       </c>
       <c r="B50" s="61" t="s">
         <v>510</v>
@@ -5572,19 +5566,19 @@
         <v>60</v>
       </c>
       <c r="E50" s="61" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="F50" s="61" t="s">
         <v>19</v>
       </c>
       <c r="G50" s="61" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="H50" s="61">
-        <v>-79.953202899999994</v>
+        <v>-79.956204600000007</v>
       </c>
       <c r="I50" s="61">
-        <v>39.633116399999999</v>
+        <v>39.668112200000003</v>
       </c>
       <c r="J50" s="61" t="s">
         <v>231</v>
@@ -5615,12 +5609,12 @@
         <v>26505</v>
       </c>
       <c r="T50" s="61" t="s">
-        <v>136</v>
+        <v>43</v>
       </c>
     </row>
     <row r="51" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A51" s="61" t="s">
-        <v>23</v>
+        <v>192</v>
       </c>
       <c r="B51" s="61" t="s">
         <v>510</v>
@@ -5632,7 +5626,7 @@
         <v>60</v>
       </c>
       <c r="E51" s="61" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F51" s="61" t="s">
         <v>19</v>
@@ -5641,10 +5635,10 @@
         <v>369</v>
       </c>
       <c r="H51" s="61">
-        <v>-79.962211800000006</v>
+        <v>-79.956762600000005</v>
       </c>
       <c r="I51" s="61">
-        <v>39.6511596</v>
+        <v>39.637875299999997</v>
       </c>
       <c r="J51" s="61" t="s">
         <v>231</v>
@@ -5653,7 +5647,7 @@
         <v>11</v>
       </c>
       <c r="L51" s="63">
-        <v>862</v>
+        <v>874</v>
       </c>
       <c r="M51" s="63" t="s">
         <v>337</v>
@@ -5677,15 +5671,15 @@
         <v>26505</v>
       </c>
       <c r="T51" s="61" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="52" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A52" s="61" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="B52" s="61" t="s">
-        <v>526</v>
+        <v>510</v>
       </c>
       <c r="C52" s="61" t="s">
         <v>351</v>
@@ -5694,40 +5688,38 @@
         <v>60</v>
       </c>
       <c r="E52" s="61" t="s">
-        <v>78</v>
+        <v>146</v>
       </c>
       <c r="F52" s="61" t="s">
-        <v>340</v>
+        <v>19</v>
       </c>
       <c r="G52" s="61" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="H52" s="61">
-        <v>-81.079930000000004</v>
+        <v>-79.955122099999997</v>
       </c>
       <c r="I52" s="61">
-        <v>37.380360000000003</v>
+        <v>39.669188599999998</v>
       </c>
       <c r="J52" s="61" t="s">
-        <v>265</v>
+        <v>231</v>
       </c>
       <c r="K52" s="61" t="s">
-        <v>17</v>
-      </c>
-      <c r="L52" s="64">
-        <v>36000</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="L52" s="63"/>
       <c r="M52" s="63" t="s">
-        <v>342</v>
-      </c>
-      <c r="N52" s="64">
-        <v>24</v>
-      </c>
-      <c r="O52" s="64">
+        <v>337</v>
+      </c>
+      <c r="N52" s="63">
+        <v>48</v>
+      </c>
+      <c r="O52" s="63">
         <v>25</v>
       </c>
-      <c r="P52" s="64">
-        <v>20</v>
+      <c r="P52" s="63">
+        <v>30</v>
       </c>
       <c r="Q52" s="61" t="s">
         <v>347</v>
@@ -5736,15 +5728,18 @@
         <v>20</v>
       </c>
       <c r="S52" s="62">
-        <v>24740</v>
+        <v>26505</v>
+      </c>
+      <c r="T52" s="61" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="53" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A53" s="61" t="s">
-        <v>106</v>
+        <v>30</v>
       </c>
       <c r="B53" s="61" t="s">
-        <v>527</v>
+        <v>510</v>
       </c>
       <c r="C53" s="61" t="s">
         <v>351</v>
@@ -5753,40 +5748,38 @@
         <v>60</v>
       </c>
       <c r="E53" s="61" t="s">
-        <v>107</v>
+        <v>147</v>
       </c>
       <c r="F53" s="61" t="s">
-        <v>340</v>
+        <v>19</v>
       </c>
       <c r="G53" s="61" t="s">
         <v>368</v>
       </c>
       <c r="H53" s="61">
-        <v>-80.545150000000007</v>
-      </c>
-      <c r="I53" s="65">
-        <v>39.285969999999999</v>
+        <v>-79.955245399999995</v>
+      </c>
+      <c r="I53" s="61">
+        <v>39.669279500000002</v>
       </c>
       <c r="J53" s="61" t="s">
-        <v>266</v>
+        <v>231</v>
       </c>
       <c r="K53" s="61" t="s">
-        <v>88</v>
-      </c>
-      <c r="L53" s="64">
-        <v>1853</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="L53" s="63"/>
       <c r="M53" s="63" t="s">
         <v>337</v>
       </c>
-      <c r="N53" s="64">
-        <v>24</v>
-      </c>
-      <c r="O53" s="64">
+      <c r="N53" s="63">
+        <v>48</v>
+      </c>
+      <c r="O53" s="63">
         <v>25</v>
       </c>
-      <c r="P53" s="64">
-        <v>20</v>
+      <c r="P53" s="63">
+        <v>30</v>
       </c>
       <c r="Q53" s="61" t="s">
         <v>347</v>
@@ -5795,12 +5788,15 @@
         <v>20</v>
       </c>
       <c r="S53" s="62">
-        <v>26426</v>
+        <v>26505</v>
+      </c>
+      <c r="T53" s="61" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="54" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A54" s="61" t="s">
-        <v>184</v>
+        <v>31</v>
       </c>
       <c r="B54" s="61" t="s">
         <v>510</v>
@@ -5812,7 +5808,7 @@
         <v>60</v>
       </c>
       <c r="E54" s="61" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="F54" s="61" t="s">
         <v>19</v>
@@ -5821,10 +5817,10 @@
         <v>369</v>
       </c>
       <c r="H54" s="61">
-        <v>-79.956140000000005</v>
+        <v>-79.965769100000003</v>
       </c>
       <c r="I54" s="61">
-        <v>39.639200000000002</v>
+        <v>39.672765599999998</v>
       </c>
       <c r="J54" s="61" t="s">
         <v>231</v>
@@ -5832,9 +5828,7 @@
       <c r="K54" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="L54" s="63">
-        <v>474</v>
-      </c>
+      <c r="L54" s="63"/>
       <c r="M54" s="63" t="s">
         <v>337</v>
       </c>
@@ -5857,15 +5851,15 @@
         <v>26505</v>
       </c>
       <c r="T54" s="61" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="55" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="55" spans="1:20" s="70" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A55" s="61" t="s">
-        <v>617</v>
+        <v>339</v>
       </c>
       <c r="B55" s="61" t="s">
-        <v>616</v>
+        <v>510</v>
       </c>
       <c r="C55" s="61" t="s">
         <v>351</v>
@@ -5874,34 +5868,32 @@
         <v>60</v>
       </c>
       <c r="E55" s="61" t="s">
-        <v>618</v>
+        <v>140</v>
       </c>
       <c r="F55" s="61" t="s">
-        <v>340</v>
+        <v>19</v>
       </c>
       <c r="G55" s="61" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="H55" s="61">
-        <v>-80.910900499999997</v>
+        <v>-79.953202899999994</v>
       </c>
       <c r="I55" s="61">
-        <v>38.301869799999999</v>
+        <v>39.633116399999999</v>
       </c>
       <c r="J55" s="61" t="s">
-        <v>619</v>
+        <v>231</v>
       </c>
       <c r="K55" s="61" t="s">
-        <v>209</v>
-      </c>
-      <c r="L55" s="64">
-        <v>3791</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="L55" s="63"/>
       <c r="M55" s="63" t="s">
         <v>337</v>
       </c>
       <c r="N55" s="63">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="O55" s="63">
         <v>25</v>
@@ -5916,15 +5908,18 @@
         <v>20</v>
       </c>
       <c r="S55" s="62">
-        <v>26651</v>
+        <v>26505</v>
+      </c>
+      <c r="T55" s="61" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="56" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A56" s="61" t="s">
-        <v>58</v>
+        <v>23</v>
       </c>
       <c r="B56" s="61" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="C56" s="61" t="s">
         <v>351</v>
@@ -5933,19 +5928,19 @@
         <v>60</v>
       </c>
       <c r="E56" s="61" t="s">
-        <v>80</v>
+        <v>141</v>
       </c>
       <c r="F56" s="61" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="G56" s="61" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="H56" s="61">
-        <v>-79.978250000000003</v>
+        <v>-79.962211800000006</v>
       </c>
       <c r="I56" s="61">
-        <v>39.671370000000003</v>
+        <v>39.6511596</v>
       </c>
       <c r="J56" s="61" t="s">
         <v>231</v>
@@ -5954,16 +5949,20 @@
         <v>11</v>
       </c>
       <c r="L56" s="63">
-        <v>515</v>
+        <v>862</v>
       </c>
       <c r="M56" s="63" t="s">
         <v>337</v>
       </c>
       <c r="N56" s="63">
-        <v>8</v>
-      </c>
-      <c r="O56" s="63"/>
-      <c r="P56" s="63"/>
+        <v>48</v>
+      </c>
+      <c r="O56" s="63">
+        <v>25</v>
+      </c>
+      <c r="P56" s="63">
+        <v>30</v>
+      </c>
       <c r="Q56" s="61" t="s">
         <v>347</v>
       </c>
@@ -5973,10 +5972,13 @@
       <c r="S56" s="62">
         <v>26505</v>
       </c>
+      <c r="T56" s="61" t="s">
+        <v>133</v>
+      </c>
     </row>
     <row r="57" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A57" s="61" t="s">
-        <v>24</v>
+        <v>184</v>
       </c>
       <c r="B57" s="61" t="s">
         <v>510</v>
@@ -5988,7 +5990,7 @@
         <v>60</v>
       </c>
       <c r="E57" s="61" t="s">
-        <v>148</v>
+        <v>185</v>
       </c>
       <c r="F57" s="61" t="s">
         <v>19</v>
@@ -5997,10 +5999,10 @@
         <v>369</v>
       </c>
       <c r="H57" s="61">
-        <v>-79.966336100000007</v>
+        <v>-79.956140000000005</v>
       </c>
       <c r="I57" s="61">
-        <v>39.649548899999999</v>
+        <v>39.639200000000002</v>
       </c>
       <c r="J57" s="61" t="s">
         <v>231</v>
@@ -6009,7 +6011,7 @@
         <v>11</v>
       </c>
       <c r="L57" s="63">
-        <v>904</v>
+        <v>474</v>
       </c>
       <c r="M57" s="63" t="s">
         <v>337</v>
@@ -6033,15 +6035,15 @@
         <v>26505</v>
       </c>
       <c r="T57" s="61" t="s">
-        <v>41</v>
+        <v>186</v>
       </c>
     </row>
     <row r="58" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A58" s="61" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="B58" s="61" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="C58" s="61" t="s">
         <v>351</v>
@@ -6050,19 +6052,19 @@
         <v>60</v>
       </c>
       <c r="E58" s="61" t="s">
-        <v>81</v>
+        <v>148</v>
       </c>
       <c r="F58" s="61" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="G58" s="61" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="H58" s="61">
-        <v>-79.926150000000007</v>
+        <v>-79.966336100000007</v>
       </c>
       <c r="I58" s="61">
-        <v>39.687820000000002</v>
+        <v>39.649548899999999</v>
       </c>
       <c r="J58" s="61" t="s">
         <v>231</v>
@@ -6071,16 +6073,20 @@
         <v>11</v>
       </c>
       <c r="L58" s="63">
-        <v>1310</v>
+        <v>904</v>
       </c>
       <c r="M58" s="63" t="s">
         <v>337</v>
       </c>
       <c r="N58" s="63">
-        <v>8</v>
-      </c>
-      <c r="O58" s="63"/>
-      <c r="P58" s="63"/>
+        <v>48</v>
+      </c>
+      <c r="O58" s="63">
+        <v>25</v>
+      </c>
+      <c r="P58" s="63">
+        <v>30</v>
+      </c>
       <c r="Q58" s="61" t="s">
         <v>347</v>
       </c>
@@ -6088,7 +6094,10 @@
         <v>20</v>
       </c>
       <c r="S58" s="62">
-        <v>26508</v>
+        <v>26505</v>
+      </c>
+      <c r="T58" s="61" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="59" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
@@ -6599,7 +6608,10 @@
     </row>
     <row r="68" spans="1:20" s="61" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="61" t="s">
-        <v>235</v>
+        <v>108</v>
+      </c>
+      <c r="B68" s="61" t="s">
+        <v>519</v>
       </c>
       <c r="C68" s="61" t="s">
         <v>351</v>
@@ -6608,28 +6620,28 @@
         <v>181</v>
       </c>
       <c r="E68" s="61" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F68" s="61" t="s">
-        <v>124</v>
+        <v>340</v>
       </c>
       <c r="G68" s="61" t="s">
         <v>368</v>
       </c>
       <c r="H68" s="61">
-        <v>-79.515240000000006</v>
+        <v>-79.978949999999998</v>
       </c>
       <c r="I68" s="65">
-        <v>39.66807</v>
+        <v>38.712879999999998</v>
       </c>
       <c r="J68" s="61" t="s">
-        <v>234</v>
+        <v>258</v>
       </c>
       <c r="K68" s="61" t="s">
-        <v>63</v>
+        <v>121</v>
       </c>
       <c r="L68" s="64">
-        <v>1948</v>
+        <v>2101</v>
       </c>
       <c r="M68" s="63" t="s">
         <v>337</v>
@@ -6637,8 +6649,12 @@
       <c r="N68" s="64">
         <v>24</v>
       </c>
-      <c r="O68" s="64"/>
-      <c r="P68" s="64"/>
+      <c r="O68" s="64">
+        <v>25</v>
+      </c>
+      <c r="P68" s="64">
+        <v>20</v>
+      </c>
       <c r="Q68" s="61" t="s">
         <v>347</v>
       </c>
@@ -6646,15 +6662,15 @@
         <v>20</v>
       </c>
       <c r="S68" s="62">
-        <v>26525</v>
+        <v>26273</v>
       </c>
     </row>
     <row r="69" spans="1:20" s="61" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="61" t="s">
-        <v>108</v>
+        <v>606</v>
       </c>
       <c r="B69" s="61" t="s">
-        <v>519</v>
+        <v>610</v>
       </c>
       <c r="C69" s="61" t="s">
         <v>351</v>
@@ -6663,57 +6679,50 @@
         <v>181</v>
       </c>
       <c r="E69" s="61" t="s">
-        <v>115</v>
+        <v>607</v>
       </c>
       <c r="F69" s="61" t="s">
         <v>340</v>
       </c>
       <c r="G69" s="61" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="H69" s="61">
-        <v>-79.978949999999998</v>
-      </c>
-      <c r="I69" s="65">
-        <v>38.712879999999998</v>
+        <v>-78.955160000000006</v>
+      </c>
+      <c r="I69" s="61">
+        <v>39.115929999999999</v>
       </c>
       <c r="J69" s="61" t="s">
-        <v>258</v>
+        <v>608</v>
       </c>
       <c r="K69" s="61" t="s">
-        <v>121</v>
+        <v>202</v>
       </c>
       <c r="L69" s="64">
-        <v>2101</v>
-      </c>
-      <c r="M69" s="63" t="s">
-        <v>337</v>
+        <v>3510</v>
+      </c>
+      <c r="M69" s="64" t="s">
+        <v>338</v>
       </c>
       <c r="N69" s="64">
         <v>24</v>
       </c>
-      <c r="O69" s="64">
-        <v>25</v>
-      </c>
-      <c r="P69" s="64">
-        <v>20</v>
-      </c>
+      <c r="O69" s="63"/>
+      <c r="P69" s="63"/>
       <c r="Q69" s="61" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="R69" s="61" t="s">
         <v>20</v>
       </c>
       <c r="S69" s="62">
-        <v>26273</v>
+        <v>26836</v>
       </c>
     </row>
     <row r="70" spans="1:20" s="61" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="61" t="s">
-        <v>606</v>
-      </c>
-      <c r="B70" s="61" t="s">
-        <v>610</v>
+        <v>50</v>
       </c>
       <c r="C70" s="61" t="s">
         <v>351</v>
@@ -6722,28 +6731,28 @@
         <v>181</v>
       </c>
       <c r="E70" s="61" t="s">
-        <v>607</v>
+        <v>77</v>
       </c>
       <c r="F70" s="61" t="s">
         <v>340</v>
       </c>
       <c r="G70" s="61" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="H70" s="61">
-        <v>-78.955160000000006</v>
-      </c>
-      <c r="I70" s="61">
-        <v>39.115929999999999</v>
+        <v>-79.127250000000004</v>
+      </c>
+      <c r="I70" s="65">
+        <v>38.99091</v>
       </c>
       <c r="J70" s="61" t="s">
-        <v>608</v>
+        <v>263</v>
       </c>
       <c r="K70" s="61" t="s">
-        <v>202</v>
+        <v>55</v>
       </c>
       <c r="L70" s="64">
-        <v>3510</v>
+        <v>2700</v>
       </c>
       <c r="M70" s="64" t="s">
         <v>338</v>
@@ -6751,8 +6760,8 @@
       <c r="N70" s="64">
         <v>24</v>
       </c>
-      <c r="O70" s="63"/>
-      <c r="P70" s="63"/>
+      <c r="O70" s="64"/>
+      <c r="P70" s="64"/>
       <c r="Q70" s="61" t="s">
         <v>348</v>
       </c>
@@ -6760,12 +6769,12 @@
         <v>20</v>
       </c>
       <c r="S70" s="62">
-        <v>26836</v>
+        <v>26847</v>
       </c>
     </row>
     <row r="71" spans="1:20" s="61" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="61" t="s">
-        <v>50</v>
+        <v>125</v>
       </c>
       <c r="C71" s="61" t="s">
         <v>351</v>
@@ -6774,7 +6783,7 @@
         <v>181</v>
       </c>
       <c r="E71" s="61" t="s">
-        <v>77</v>
+        <v>128</v>
       </c>
       <c r="F71" s="61" t="s">
         <v>340</v>
@@ -6782,20 +6791,14 @@
       <c r="G71" s="61" t="s">
         <v>368</v>
       </c>
-      <c r="H71" s="61">
-        <v>-79.127250000000004</v>
-      </c>
-      <c r="I71" s="65">
-        <v>38.99091</v>
-      </c>
       <c r="J71" s="61" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="K71" s="61" t="s">
-        <v>55</v>
+        <v>129</v>
       </c>
       <c r="L71" s="64">
-        <v>2700</v>
+        <v>1800</v>
       </c>
       <c r="M71" s="64" t="s">
         <v>338</v>
@@ -6811,16 +6814,14 @@
       <c r="R71" s="61" t="s">
         <v>20</v>
       </c>
-      <c r="S71" s="62">
-        <v>26847</v>
-      </c>
+      <c r="S71" s="62"/>
     </row>
     <row r="72" spans="1:20" s="61" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="61" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="B72" s="61" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="C72" s="61" t="s">
         <v>351</v>
@@ -6829,40 +6830,40 @@
         <v>181</v>
       </c>
       <c r="E72" s="61" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="F72" s="61" t="s">
-        <v>19</v>
+        <v>340</v>
       </c>
       <c r="G72" s="61" t="s">
         <v>368</v>
       </c>
       <c r="H72" s="61">
-        <v>-78.98272</v>
+        <v>-81.205110000000005</v>
       </c>
       <c r="I72" s="65">
-        <v>39.438070000000003</v>
+        <v>39.391249999999999</v>
       </c>
       <c r="J72" s="61" t="s">
-        <v>243</v>
+        <v>268</v>
       </c>
       <c r="K72" s="61" t="s">
-        <v>13</v>
-      </c>
-      <c r="L72" s="63">
-        <v>1193</v>
+        <v>56</v>
+      </c>
+      <c r="L72" s="64">
+        <v>2892</v>
       </c>
       <c r="M72" s="63" t="s">
         <v>337</v>
       </c>
-      <c r="N72" s="63">
-        <v>48</v>
+      <c r="N72" s="64">
+        <v>24</v>
       </c>
       <c r="O72" s="64">
         <v>25</v>
       </c>
       <c r="P72" s="64">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="Q72" s="61" t="s">
         <v>347</v>
@@ -6871,12 +6872,15 @@
         <v>20</v>
       </c>
       <c r="S72" s="62">
-        <v>26726</v>
+        <v>26170</v>
       </c>
     </row>
     <row r="73" spans="1:20" s="61" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="61" t="s">
-        <v>125</v>
+        <v>14</v>
+      </c>
+      <c r="B73" s="61" t="s">
+        <v>529</v>
       </c>
       <c r="C73" s="61" t="s">
         <v>351</v>
@@ -6885,7 +6889,7 @@
         <v>181</v>
       </c>
       <c r="E73" s="61" t="s">
-        <v>128</v>
+        <v>82</v>
       </c>
       <c r="F73" s="61" t="s">
         <v>340</v>
@@ -6893,14 +6897,20 @@
       <c r="G73" s="61" t="s">
         <v>368</v>
       </c>
+      <c r="H73" s="61">
+        <v>-78.226619999999997</v>
+      </c>
+      <c r="I73" s="61">
+        <v>39.628019999999999</v>
+      </c>
       <c r="J73" s="61" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="K73" s="61" t="s">
-        <v>129</v>
+        <v>15</v>
       </c>
       <c r="L73" s="64">
-        <v>1800</v>
+        <v>3255</v>
       </c>
       <c r="M73" s="64" t="s">
         <v>338</v>
@@ -6916,14 +6926,13 @@
       <c r="R73" s="61" t="s">
         <v>20</v>
       </c>
-      <c r="S73" s="62"/>
+      <c r="S73" s="62">
+        <v>25411</v>
+      </c>
     </row>
     <row r="74" spans="1:20" s="61" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="61" t="s">
-        <v>51</v>
-      </c>
-      <c r="B74" s="61" t="s">
-        <v>528</v>
+        <v>126</v>
       </c>
       <c r="C74" s="61" t="s">
         <v>351</v>
@@ -6932,7 +6941,7 @@
         <v>181</v>
       </c>
       <c r="E74" s="61" t="s">
-        <v>79</v>
+        <v>127</v>
       </c>
       <c r="F74" s="61" t="s">
         <v>340</v>
@@ -6940,49 +6949,34 @@
       <c r="G74" s="61" t="s">
         <v>368</v>
       </c>
-      <c r="H74" s="61">
-        <v>-81.205110000000005</v>
-      </c>
-      <c r="I74" s="65">
-        <v>39.391249999999999</v>
-      </c>
       <c r="J74" s="61" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="K74" s="61" t="s">
-        <v>56</v>
+        <v>122</v>
       </c>
       <c r="L74" s="64">
-        <v>2892</v>
-      </c>
-      <c r="M74" s="63" t="s">
-        <v>337</v>
+        <v>20411</v>
+      </c>
+      <c r="M74" s="64" t="s">
+        <v>338</v>
       </c>
       <c r="N74" s="64">
         <v>24</v>
       </c>
-      <c r="O74" s="64">
-        <v>25</v>
-      </c>
-      <c r="P74" s="64">
-        <v>20</v>
-      </c>
+      <c r="O74" s="64"/>
+      <c r="P74" s="64"/>
       <c r="Q74" s="61" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="R74" s="61" t="s">
         <v>20</v>
       </c>
-      <c r="S74" s="62">
-        <v>26170</v>
-      </c>
+      <c r="S74" s="62"/>
     </row>
     <row r="75" spans="1:20" s="61" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="61" t="s">
-        <v>14</v>
-      </c>
-      <c r="B75" s="61" t="s">
-        <v>529</v>
+        <v>90</v>
       </c>
       <c r="C75" s="61" t="s">
         <v>351</v>
@@ -6991,7 +6985,7 @@
         <v>181</v>
       </c>
       <c r="E75" s="61" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="F75" s="61" t="s">
         <v>340</v>
@@ -7000,41 +6994,48 @@
         <v>368</v>
       </c>
       <c r="H75" s="61">
-        <v>-78.226619999999997</v>
-      </c>
-      <c r="I75" s="61">
-        <v>39.628019999999999</v>
+        <v>-80.260360000000006</v>
+      </c>
+      <c r="I75" s="65">
+        <v>39.452579999999998</v>
       </c>
       <c r="J75" s="61" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="K75" s="61" t="s">
-        <v>15</v>
+        <v>89</v>
       </c>
       <c r="L75" s="64">
-        <v>3255</v>
-      </c>
-      <c r="M75" s="64" t="s">
-        <v>338</v>
+        <v>2742</v>
+      </c>
+      <c r="M75" s="63" t="s">
+        <v>337</v>
       </c>
       <c r="N75" s="64">
         <v>24</v>
       </c>
-      <c r="O75" s="64"/>
-      <c r="P75" s="64"/>
+      <c r="O75" s="64">
+        <v>25</v>
+      </c>
+      <c r="P75" s="64">
+        <v>30</v>
+      </c>
       <c r="Q75" s="61" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="R75" s="61" t="s">
         <v>20</v>
       </c>
       <c r="S75" s="62">
-        <v>25411</v>
+        <v>26591</v>
       </c>
     </row>
     <row r="76" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A76" s="61" t="s">
-        <v>126</v>
+        <v>59</v>
+      </c>
+      <c r="B76" s="61" t="s">
+        <v>525</v>
       </c>
       <c r="C76" s="61" t="s">
         <v>351</v>
@@ -7043,42 +7044,54 @@
         <v>181</v>
       </c>
       <c r="E76" s="61" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
       <c r="F76" s="61" t="s">
-        <v>340</v>
+        <v>19</v>
       </c>
       <c r="G76" s="61" t="s">
         <v>368</v>
       </c>
+      <c r="H76" s="61">
+        <v>-78.98272</v>
+      </c>
+      <c r="I76" s="65">
+        <v>39.438070000000003</v>
+      </c>
       <c r="J76" s="61" t="s">
-        <v>270</v>
+        <v>243</v>
       </c>
       <c r="K76" s="61" t="s">
-        <v>122</v>
-      </c>
-      <c r="L76" s="64">
-        <v>20411</v>
-      </c>
-      <c r="M76" s="64" t="s">
-        <v>338</v>
-      </c>
-      <c r="N76" s="64">
-        <v>24</v>
-      </c>
-      <c r="O76" s="64"/>
-      <c r="P76" s="64"/>
+        <v>13</v>
+      </c>
+      <c r="L76" s="63">
+        <v>1193</v>
+      </c>
+      <c r="M76" s="63" t="s">
+        <v>337</v>
+      </c>
+      <c r="N76" s="63">
+        <v>48</v>
+      </c>
+      <c r="O76" s="64">
+        <v>25</v>
+      </c>
+      <c r="P76" s="64">
+        <v>30</v>
+      </c>
       <c r="Q76" s="61" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="R76" s="61" t="s">
         <v>20</v>
       </c>
-      <c r="S76" s="62"/>
+      <c r="S76" s="62">
+        <v>26726</v>
+      </c>
     </row>
     <row r="77" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A77" s="61" t="s">
-        <v>90</v>
+        <v>235</v>
       </c>
       <c r="C77" s="61" t="s">
         <v>351</v>
@@ -7087,28 +7100,28 @@
         <v>181</v>
       </c>
       <c r="E77" s="61" t="s">
-        <v>96</v>
+        <v>114</v>
       </c>
       <c r="F77" s="61" t="s">
-        <v>340</v>
+        <v>124</v>
       </c>
       <c r="G77" s="61" t="s">
         <v>368</v>
       </c>
       <c r="H77" s="61">
-        <v>-80.260360000000006</v>
+        <v>-79.515240000000006</v>
       </c>
       <c r="I77" s="65">
-        <v>39.452579999999998</v>
+        <v>39.66807</v>
       </c>
       <c r="J77" s="61" t="s">
-        <v>274</v>
+        <v>234</v>
       </c>
       <c r="K77" s="61" t="s">
-        <v>89</v>
+        <v>63</v>
       </c>
       <c r="L77" s="64">
-        <v>2742</v>
+        <v>1948</v>
       </c>
       <c r="M77" s="63" t="s">
         <v>337</v>
@@ -7116,12 +7129,8 @@
       <c r="N77" s="64">
         <v>24</v>
       </c>
-      <c r="O77" s="64">
-        <v>25</v>
-      </c>
-      <c r="P77" s="64">
-        <v>30</v>
-      </c>
+      <c r="O77" s="64"/>
+      <c r="P77" s="64"/>
       <c r="Q77" s="61" t="s">
         <v>347</v>
       </c>
@@ -7129,12 +7138,12 @@
         <v>20</v>
       </c>
       <c r="S77" s="62">
-        <v>26591</v>
+        <v>26525</v>
       </c>
     </row>
     <row r="78" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A78" s="61" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="C78" s="61" t="s">
         <v>352</v>
@@ -7143,35 +7152,37 @@
         <v>181</v>
       </c>
       <c r="E78" s="61" t="s">
-        <v>174</v>
+        <v>156</v>
       </c>
       <c r="F78" s="61" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="G78" s="61" t="s">
         <v>368</v>
       </c>
-      <c r="H78" s="66">
-        <v>-82.430654000000004</v>
-      </c>
-      <c r="I78" s="66">
-        <v>38.424089000000002</v>
-      </c>
-      <c r="J78" s="66" t="s">
-        <v>578</v>
+      <c r="H78" s="61">
+        <v>-82.285698770801503</v>
+      </c>
+      <c r="I78" s="61">
+        <v>38.414946823509098</v>
+      </c>
+      <c r="J78" s="61" t="s">
+        <v>356</v>
       </c>
       <c r="K78" s="61" t="s">
         <v>157</v>
       </c>
-      <c r="L78" s="63"/>
+      <c r="L78" s="63">
+        <v>4000</v>
+      </c>
       <c r="M78" s="63" t="s">
         <v>583</v>
       </c>
       <c r="N78" s="63">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="O78" s="63">
-        <v>35</v>
+        <v>250</v>
       </c>
       <c r="P78" s="63">
         <v>30</v>
@@ -7182,16 +7193,16 @@
       <c r="R78" s="61" t="s">
         <v>20</v>
       </c>
-      <c r="S78" s="62">
-        <v>25703</v>
-      </c>
-      <c r="T78" s="66" t="s">
-        <v>585</v>
+      <c r="S78" s="67">
+        <v>25504</v>
+      </c>
+      <c r="T78" s="68" t="s">
+        <v>586</v>
       </c>
     </row>
     <row r="79" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A79" s="61" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C79" s="61" t="s">
         <v>352</v>
@@ -7200,7 +7211,7 @@
         <v>181</v>
       </c>
       <c r="E79" s="61" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="F79" s="61" t="s">
         <v>340</v>
@@ -7209,31 +7220,31 @@
         <v>368</v>
       </c>
       <c r="H79" s="61">
-        <v>-82.285698770801503</v>
+        <v>-82.006959612418996</v>
       </c>
       <c r="I79" s="61">
-        <v>38.414946823509098</v>
+        <v>38.446524084559897</v>
       </c>
       <c r="J79" s="61" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="K79" s="61" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="L79" s="63">
-        <v>4000</v>
-      </c>
-      <c r="M79" s="63" t="s">
-        <v>583</v>
-      </c>
-      <c r="N79" s="63">
-        <v>24</v>
-      </c>
-      <c r="O79" s="63">
-        <v>250</v>
-      </c>
-      <c r="P79" s="63">
-        <v>30</v>
+        <v>28759</v>
+      </c>
+      <c r="M79" s="64" t="s">
+        <v>338</v>
+      </c>
+      <c r="N79" s="64">
+        <v>72</v>
+      </c>
+      <c r="O79" s="64">
+        <v>25</v>
+      </c>
+      <c r="P79" s="64">
+        <v>20</v>
       </c>
       <c r="Q79" s="61" t="s">
         <v>347</v>
@@ -7241,16 +7252,13 @@
       <c r="R79" s="61" t="s">
         <v>20</v>
       </c>
-      <c r="S79" s="67">
-        <v>25504</v>
-      </c>
-      <c r="T79" s="68" t="s">
-        <v>586</v>
+      <c r="S79" s="62">
+        <v>25526</v>
       </c>
     </row>
     <row r="80" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A80" s="61" t="s">
-        <v>179</v>
+        <v>163</v>
       </c>
       <c r="C80" s="61" t="s">
         <v>352</v>
@@ -7259,38 +7267,40 @@
         <v>181</v>
       </c>
       <c r="E80" s="61" t="s">
-        <v>180</v>
+        <v>163</v>
       </c>
       <c r="F80" s="61" t="s">
-        <v>19</v>
+        <v>340</v>
       </c>
       <c r="G80" s="61" t="s">
         <v>368</v>
       </c>
-      <c r="H80" s="66">
-        <v>-82.425917999999996</v>
-      </c>
-      <c r="I80" s="66">
-        <v>38.421745999999999</v>
-      </c>
-      <c r="J80" s="66" t="s">
-        <v>579</v>
+      <c r="H80" s="61">
+        <v>-82.451303840583293</v>
+      </c>
+      <c r="I80" s="61">
+        <v>38.343336164586603</v>
+      </c>
+      <c r="J80" s="61" t="s">
+        <v>353</v>
       </c>
       <c r="K80" s="61" t="s">
-        <v>157</v>
-      </c>
-      <c r="L80" s="63"/>
-      <c r="M80" s="63" t="s">
-        <v>583</v>
-      </c>
-      <c r="N80" s="63">
-        <v>5</v>
-      </c>
-      <c r="O80" s="63">
-        <v>100</v>
-      </c>
-      <c r="P80" s="63">
-        <v>30</v>
+        <v>164</v>
+      </c>
+      <c r="L80" s="63">
+        <v>1600</v>
+      </c>
+      <c r="M80" s="64" t="s">
+        <v>338</v>
+      </c>
+      <c r="N80" s="64">
+        <v>24</v>
+      </c>
+      <c r="O80" s="64">
+        <v>25</v>
+      </c>
+      <c r="P80" s="64">
+        <v>20</v>
       </c>
       <c r="Q80" s="61" t="s">
         <v>347</v>
@@ -7299,15 +7309,15 @@
         <v>20</v>
       </c>
       <c r="S80" s="62">
-        <v>25703</v>
-      </c>
-      <c r="T80" s="66" t="s">
-        <v>584</v>
+        <v>25701</v>
+      </c>
+      <c r="T80" s="61" t="s">
+        <v>587</v>
       </c>
     </row>
     <row r="81" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A81" s="61" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="C81" s="61" t="s">
         <v>352</v>
@@ -7316,7 +7326,7 @@
         <v>181</v>
       </c>
       <c r="E81" s="61" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="F81" s="61" t="s">
         <v>340</v>
@@ -7325,25 +7335,25 @@
         <v>368</v>
       </c>
       <c r="H81" s="61">
-        <v>-82.006959612418996</v>
+        <v>-82.287563960345196</v>
       </c>
       <c r="I81" s="61">
-        <v>38.446524084559897</v>
+        <v>38.572623654172197</v>
       </c>
       <c r="J81" s="61" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="K81" s="61" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="L81" s="63">
-        <v>28759</v>
+        <v>1000</v>
       </c>
       <c r="M81" s="64" t="s">
         <v>338</v>
       </c>
       <c r="N81" s="64">
-        <v>72</v>
+        <v>24</v>
       </c>
       <c r="O81" s="64">
         <v>25</v>
@@ -7358,12 +7368,15 @@
         <v>20</v>
       </c>
       <c r="S81" s="62">
-        <v>25526</v>
+        <v>25537</v>
+      </c>
+      <c r="T81" s="61" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="82" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A82" s="61" t="s">
-        <v>163</v>
+        <v>173</v>
       </c>
       <c r="C82" s="61" t="s">
         <v>352</v>
@@ -7372,40 +7385,38 @@
         <v>181</v>
       </c>
       <c r="E82" s="61" t="s">
-        <v>163</v>
+        <v>174</v>
       </c>
       <c r="F82" s="61" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="G82" s="61" t="s">
         <v>368</v>
       </c>
-      <c r="H82" s="61">
-        <v>-82.451303840583293</v>
-      </c>
-      <c r="I82" s="61">
-        <v>38.343336164586603</v>
-      </c>
-      <c r="J82" s="61" t="s">
-        <v>353</v>
+      <c r="H82" s="66">
+        <v>-82.430654000000004</v>
+      </c>
+      <c r="I82" s="66">
+        <v>38.424089000000002</v>
+      </c>
+      <c r="J82" s="66" t="s">
+        <v>578</v>
       </c>
       <c r="K82" s="61" t="s">
-        <v>164</v>
-      </c>
-      <c r="L82" s="63">
-        <v>1600</v>
-      </c>
-      <c r="M82" s="64" t="s">
-        <v>338</v>
-      </c>
-      <c r="N82" s="64">
-        <v>24</v>
-      </c>
-      <c r="O82" s="64">
-        <v>25</v>
-      </c>
-      <c r="P82" s="64">
-        <v>20</v>
+        <v>157</v>
+      </c>
+      <c r="L82" s="63"/>
+      <c r="M82" s="63" t="s">
+        <v>583</v>
+      </c>
+      <c r="N82" s="63">
+        <v>5</v>
+      </c>
+      <c r="O82" s="63">
+        <v>35</v>
+      </c>
+      <c r="P82" s="63">
+        <v>30</v>
       </c>
       <c r="Q82" s="61" t="s">
         <v>347</v>
@@ -7414,15 +7425,15 @@
         <v>20</v>
       </c>
       <c r="S82" s="62">
-        <v>25701</v>
-      </c>
-      <c r="T82" s="61" t="s">
-        <v>587</v>
+        <v>25703</v>
+      </c>
+      <c r="T82" s="66" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="83" spans="1:20" s="69" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A83" s="61" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="B83" s="61"/>
       <c r="C83" s="61" t="s">
@@ -7432,40 +7443,38 @@
         <v>181</v>
       </c>
       <c r="E83" s="61" t="s">
-        <v>165</v>
+        <v>180</v>
       </c>
       <c r="F83" s="61" t="s">
-        <v>340</v>
+        <v>19</v>
       </c>
       <c r="G83" s="61" t="s">
         <v>368</v>
       </c>
-      <c r="H83" s="61">
-        <v>-82.287563960345196</v>
-      </c>
-      <c r="I83" s="61">
-        <v>38.572623654172197</v>
-      </c>
-      <c r="J83" s="61" t="s">
-        <v>354</v>
+      <c r="H83" s="66">
+        <v>-82.425917999999996</v>
+      </c>
+      <c r="I83" s="66">
+        <v>38.421745999999999</v>
+      </c>
+      <c r="J83" s="66" t="s">
+        <v>579</v>
       </c>
       <c r="K83" s="61" t="s">
         <v>157</v>
       </c>
-      <c r="L83" s="63">
-        <v>1000</v>
-      </c>
-      <c r="M83" s="64" t="s">
-        <v>338</v>
-      </c>
-      <c r="N83" s="64">
-        <v>24</v>
-      </c>
-      <c r="O83" s="64">
-        <v>25</v>
-      </c>
-      <c r="P83" s="64">
-        <v>20</v>
+      <c r="L83" s="63"/>
+      <c r="M83" s="63" t="s">
+        <v>583</v>
+      </c>
+      <c r="N83" s="63">
+        <v>5</v>
+      </c>
+      <c r="O83" s="63">
+        <v>100</v>
+      </c>
+      <c r="P83" s="63">
+        <v>30</v>
       </c>
       <c r="Q83" s="61" t="s">
         <v>347</v>
@@ -7474,10 +7483,10 @@
         <v>20</v>
       </c>
       <c r="S83" s="62">
-        <v>25537</v>
-      </c>
-      <c r="T83" s="61" t="s">
-        <v>588</v>
+        <v>25703</v>
+      </c>
+      <c r="T83" s="66" t="s">
+        <v>584</v>
       </c>
     </row>
     <row r="84" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
@@ -7593,6 +7602,7 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:T85">
     <sortCondition ref="D2:D85"/>
     <sortCondition descending="1" ref="C2:C85"/>
+    <sortCondition descending="1" ref="F2:F85"/>
     <sortCondition ref="A2:A85"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Data update from 8/21, and added citation info.
</commit_message>
<xml_diff>
--- a/dashboard/data/watchdb.all_tables.xlsx
+++ b/dashboard/data/watchdb.all_tables.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tpd0001/github/watch-wv/patchr/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13269A63-E9F3-264F-8CF3-597B4A05EFE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59C40D4E-BBF4-3241-BBEC-514678477A64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11260" yWindow="1600" windowWidth="30240" windowHeight="18980" xr2:uid="{ABEE2980-A2EF-284E-9534-8BF6C1D1D8CC}"/>
   </bookViews>
@@ -22,7 +22,7 @@
     <sheet name="methods" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">location!$A$1:$T$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">location!$A$1:$T$88</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1639" uniqueCount="660">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1675" uniqueCount="665">
   <si>
     <t>CharlestonWWTP-01</t>
   </si>
@@ -2023,6 +2023,21 @@
   </si>
   <si>
     <t>54045-001-01-00-00</t>
+  </si>
+  <si>
+    <t>FacManWVU-01</t>
+  </si>
+  <si>
+    <t>OaklandWVU-01</t>
+  </si>
+  <si>
+    <t>ReynoldsWVU-01</t>
+  </si>
+  <si>
+    <t>WVU Reynolds Hall</t>
+  </si>
+  <si>
+    <t>WVU Facility Maintenance</t>
   </si>
 </sst>
 </file>
@@ -2769,7 +2784,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0856F7A-D0C0-3942-9027-9FB2F3C2C3E0}">
-  <dimension ref="A1:T87"/>
+  <dimension ref="A1:T90"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="31.33203125" customWidth="1"/>
@@ -4349,179 +4364,171 @@
       </c>
       <c r="T27" s="2"/>
     </row>
-    <row r="28" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="26" t="s">
+    <row r="28" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
+        <v>660</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>664</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="H28" s="2"/>
+      <c r="I28" s="2"/>
+      <c r="J28" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K28" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="L28" s="34"/>
+      <c r="M28" s="34" t="s">
+        <v>337</v>
+      </c>
+      <c r="N28" s="34">
+        <v>48</v>
+      </c>
+      <c r="O28" s="34">
+        <v>25</v>
+      </c>
+      <c r="P28" s="34">
+        <v>30</v>
+      </c>
+      <c r="Q28" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="R28" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="S28" s="4">
+        <v>26505</v>
+      </c>
+      <c r="T28" s="2"/>
+    </row>
+    <row r="29" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
+        <v>661</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="H29" s="2"/>
+      <c r="I29" s="2"/>
+      <c r="J29" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K29" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="L29" s="34"/>
+      <c r="M29" s="34" t="s">
+        <v>337</v>
+      </c>
+      <c r="N29" s="34">
+        <v>48</v>
+      </c>
+      <c r="O29" s="34">
+        <v>25</v>
+      </c>
+      <c r="P29" s="34">
+        <v>30</v>
+      </c>
+      <c r="Q29" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="R29" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="S29" s="4">
+        <v>26505</v>
+      </c>
+      <c r="T29" s="2"/>
+    </row>
+    <row r="30" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="2" t="s">
+        <v>662</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>663</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="H30" s="2"/>
+      <c r="I30" s="2"/>
+      <c r="J30" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K30" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="L30" s="34"/>
+      <c r="M30" s="34" t="s">
+        <v>337</v>
+      </c>
+      <c r="N30" s="34">
+        <v>48</v>
+      </c>
+      <c r="O30" s="34">
+        <v>25</v>
+      </c>
+      <c r="P30" s="34">
+        <v>30</v>
+      </c>
+      <c r="Q30" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="R30" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="S30" s="4">
+        <v>26505</v>
+      </c>
+      <c r="T30" s="2"/>
+    </row>
+    <row r="31" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="26" t="s">
         <v>167</v>
-      </c>
-      <c r="B28" s="26"/>
-      <c r="C28" s="26" t="s">
-        <v>352</v>
-      </c>
-      <c r="D28" s="29" t="s">
-        <v>103</v>
-      </c>
-      <c r="E28" s="26" t="s">
-        <v>68</v>
-      </c>
-      <c r="F28" s="26" t="s">
-        <v>340</v>
-      </c>
-      <c r="G28" s="26" t="s">
-        <v>368</v>
-      </c>
-      <c r="H28" s="26">
-        <v>-81.679554234298493</v>
-      </c>
-      <c r="I28" s="26">
-        <v>38.373735533484897</v>
-      </c>
-      <c r="J28" s="26" t="s">
-        <v>357</v>
-      </c>
-      <c r="K28" s="26" t="s">
-        <v>1</v>
-      </c>
-      <c r="L28" s="30">
-        <v>49500</v>
-      </c>
-      <c r="M28" s="31" t="s">
-        <v>338</v>
-      </c>
-      <c r="N28" s="31">
-        <v>24</v>
-      </c>
-      <c r="O28" s="31"/>
-      <c r="P28" s="31"/>
-      <c r="Q28" s="26" t="s">
-        <v>348</v>
-      </c>
-      <c r="R28" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="S28" s="36">
-        <v>25387</v>
-      </c>
-      <c r="T28" s="26"/>
-    </row>
-    <row r="29" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="26" t="s">
-        <v>172</v>
-      </c>
-      <c r="B29" s="26"/>
-      <c r="C29" s="26" t="s">
-        <v>352</v>
-      </c>
-      <c r="D29" s="29" t="s">
-        <v>103</v>
-      </c>
-      <c r="E29" s="26" t="s">
-        <v>162</v>
-      </c>
-      <c r="F29" s="26" t="s">
-        <v>340</v>
-      </c>
-      <c r="G29" s="26" t="s">
-        <v>368</v>
-      </c>
-      <c r="H29" s="26">
-        <v>-81.758709180509001</v>
-      </c>
-      <c r="I29" s="26">
-        <v>38.368519014596998</v>
-      </c>
-      <c r="J29" s="26" t="s">
-        <v>358</v>
-      </c>
-      <c r="K29" s="26" t="s">
-        <v>1</v>
-      </c>
-      <c r="L29" s="30">
-        <v>9000</v>
-      </c>
-      <c r="M29" s="31" t="s">
-        <v>338</v>
-      </c>
-      <c r="N29" s="31">
-        <v>24</v>
-      </c>
-      <c r="O29" s="31">
-        <v>25</v>
-      </c>
-      <c r="P29" s="31">
-        <v>20</v>
-      </c>
-      <c r="Q29" s="26" t="s">
-        <v>347</v>
-      </c>
-      <c r="R29" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="S29" s="29">
-        <v>25064</v>
-      </c>
-      <c r="T29" s="26"/>
-    </row>
-    <row r="30" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="26" t="s">
-        <v>166</v>
-      </c>
-      <c r="B30" s="26"/>
-      <c r="C30" s="26" t="s">
-        <v>352</v>
-      </c>
-      <c r="D30" s="29" t="s">
-        <v>103</v>
-      </c>
-      <c r="E30" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="F30" s="26" t="s">
-        <v>340</v>
-      </c>
-      <c r="G30" s="26" t="s">
-        <v>368</v>
-      </c>
-      <c r="H30" s="26">
-        <v>-82.528864034905197</v>
-      </c>
-      <c r="I30" s="26">
-        <v>38.400744931017101</v>
-      </c>
-      <c r="J30" s="26" t="s">
-        <v>353</v>
-      </c>
-      <c r="K30" s="26" t="s">
-        <v>164</v>
-      </c>
-      <c r="L30" s="30">
-        <v>56000</v>
-      </c>
-      <c r="M30" s="31" t="s">
-        <v>338</v>
-      </c>
-      <c r="N30" s="31">
-        <v>24</v>
-      </c>
-      <c r="O30" s="31">
-        <v>25</v>
-      </c>
-      <c r="P30" s="31">
-        <v>20</v>
-      </c>
-      <c r="Q30" s="26" t="s">
-        <v>347</v>
-      </c>
-      <c r="R30" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="S30" s="36">
-        <v>25704</v>
-      </c>
-      <c r="T30" s="26"/>
-    </row>
-    <row r="31" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="26" t="s">
-        <v>171</v>
       </c>
       <c r="B31" s="26"/>
       <c r="C31" s="26" t="s">
@@ -4531,7 +4538,7 @@
         <v>103</v>
       </c>
       <c r="E31" s="26" t="s">
-        <v>161</v>
+        <v>68</v>
       </c>
       <c r="F31" s="26" t="s">
         <v>340</v>
@@ -4540,104 +4547,100 @@
         <v>368</v>
       </c>
       <c r="H31" s="26">
-        <v>-82.298209254857795</v>
+        <v>-81.679554234298493</v>
       </c>
       <c r="I31" s="26">
-        <v>38.419661908139098</v>
+        <v>38.373735533484897</v>
       </c>
       <c r="J31" s="26" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="K31" s="26" t="s">
-        <v>157</v>
+        <v>1</v>
       </c>
       <c r="L31" s="30">
-        <v>7000</v>
+        <v>49500</v>
       </c>
       <c r="M31" s="31" t="s">
-        <v>583</v>
+        <v>338</v>
       </c>
       <c r="N31" s="31">
         <v>24</v>
       </c>
-      <c r="O31" s="31">
+      <c r="O31" s="31"/>
+      <c r="P31" s="31"/>
+      <c r="Q31" s="26" t="s">
+        <v>348</v>
+      </c>
+      <c r="R31" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="S31" s="36">
+        <v>25387</v>
+      </c>
+      <c r="T31" s="26"/>
+    </row>
+    <row r="32" spans="1:20" s="6" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="26" t="s">
+        <v>172</v>
+      </c>
+      <c r="B32" s="26"/>
+      <c r="C32" s="26" t="s">
+        <v>352</v>
+      </c>
+      <c r="D32" s="29" t="s">
+        <v>103</v>
+      </c>
+      <c r="E32" s="26" t="s">
+        <v>162</v>
+      </c>
+      <c r="F32" s="26" t="s">
+        <v>340</v>
+      </c>
+      <c r="G32" s="26" t="s">
+        <v>368</v>
+      </c>
+      <c r="H32" s="26">
+        <v>-81.758709180509001</v>
+      </c>
+      <c r="I32" s="26">
+        <v>38.368519014596998</v>
+      </c>
+      <c r="J32" s="26" t="s">
+        <v>358</v>
+      </c>
+      <c r="K32" s="26" t="s">
+        <v>1</v>
+      </c>
+      <c r="L32" s="30">
+        <v>9000</v>
+      </c>
+      <c r="M32" s="31" t="s">
+        <v>338</v>
+      </c>
+      <c r="N32" s="31">
+        <v>24</v>
+      </c>
+      <c r="O32" s="31">
         <v>25</v>
       </c>
-      <c r="P31" s="31">
-        <v>20</v>
-      </c>
-      <c r="Q31" s="26" t="s">
+      <c r="P32" s="31">
+        <v>20</v>
+      </c>
+      <c r="Q32" s="26" t="s">
         <v>347</v>
       </c>
-      <c r="R31" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="S31" s="29">
-        <v>25705</v>
-      </c>
-      <c r="T31" s="26"/>
-    </row>
-    <row r="32" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="39" t="s">
-        <v>575</v>
-      </c>
-      <c r="B32" s="39"/>
-      <c r="C32" s="39" t="s">
-        <v>352</v>
-      </c>
-      <c r="D32" s="40" t="s">
-        <v>103</v>
-      </c>
-      <c r="E32" s="39" t="s">
-        <v>576</v>
-      </c>
-      <c r="F32" s="39" t="s">
-        <v>340</v>
-      </c>
-      <c r="G32" s="39" t="s">
-        <v>368</v>
-      </c>
-      <c r="H32" s="39">
-        <v>-81.867118796822695</v>
-      </c>
-      <c r="I32" s="39">
-        <v>38.537901317549398</v>
-      </c>
-      <c r="J32" s="39" t="s">
-        <v>577</v>
-      </c>
-      <c r="K32" s="39" t="s">
-        <v>159</v>
-      </c>
-      <c r="L32" s="41">
-        <v>4900</v>
-      </c>
-      <c r="M32" s="42" t="s">
-        <v>338</v>
-      </c>
-      <c r="N32" s="42">
-        <v>48</v>
-      </c>
-      <c r="O32" s="42">
-        <v>333</v>
-      </c>
-      <c r="P32" s="42">
-        <v>1440</v>
-      </c>
-      <c r="Q32" s="39" t="s">
-        <v>347</v>
-      </c>
-      <c r="R32" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="S32" s="40">
-        <v>25168</v>
-      </c>
-      <c r="T32" s="39"/>
+      <c r="R32" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="S32" s="29">
+        <v>25064</v>
+      </c>
+      <c r="T32" s="26"/>
     </row>
     <row r="33" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A33" s="26" t="s">
-        <v>580</v>
+        <v>166</v>
       </c>
       <c r="B33" s="26"/>
       <c r="C33" s="26" t="s">
@@ -4647,7 +4650,7 @@
         <v>103</v>
       </c>
       <c r="E33" s="26" t="s">
-        <v>573</v>
+        <v>155</v>
       </c>
       <c r="F33" s="26" t="s">
         <v>340</v>
@@ -4656,19 +4659,19 @@
         <v>368</v>
       </c>
       <c r="H33" s="26">
-        <v>-82.105144999999993</v>
+        <v>-82.528864034905197</v>
       </c>
       <c r="I33" s="26">
-        <v>38.425437000000002</v>
+        <v>38.400744931017101</v>
       </c>
       <c r="J33" s="26" t="s">
-        <v>370</v>
+        <v>353</v>
       </c>
       <c r="K33" s="26" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="L33" s="30">
-        <v>7200</v>
+        <v>56000</v>
       </c>
       <c r="M33" s="31" t="s">
         <v>338</v>
@@ -4688,16 +4691,14 @@
       <c r="R33" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="S33" s="29">
-        <v>25541</v>
-      </c>
-      <c r="T33" s="26" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="34" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="S33" s="36">
+        <v>25704</v>
+      </c>
+      <c r="T33" s="26"/>
+    </row>
+    <row r="34" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A34" s="26" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B34" s="26"/>
       <c r="C34" s="26" t="s">
@@ -4707,7 +4708,7 @@
         <v>103</v>
       </c>
       <c r="E34" s="26" t="s">
-        <v>572</v>
+        <v>161</v>
       </c>
       <c r="F34" s="26" t="s">
         <v>340</v>
@@ -4716,22 +4717,22 @@
         <v>368</v>
       </c>
       <c r="H34" s="26">
-        <v>-82.244877751268803</v>
+        <v>-82.298209254857795</v>
       </c>
       <c r="I34" s="26">
-        <v>38.372162360135</v>
+        <v>38.419661908139098</v>
       </c>
       <c r="J34" s="26" t="s">
-        <v>371</v>
+        <v>355</v>
       </c>
       <c r="K34" s="26" t="s">
         <v>157</v>
       </c>
       <c r="L34" s="30">
-        <v>4050</v>
+        <v>7000</v>
       </c>
       <c r="M34" s="31" t="s">
-        <v>338</v>
+        <v>583</v>
       </c>
       <c r="N34" s="31">
         <v>24</v>
@@ -4749,191 +4750,194 @@
         <v>20</v>
       </c>
       <c r="S34" s="29">
+        <v>25705</v>
+      </c>
+      <c r="T34" s="26"/>
+    </row>
+    <row r="35" spans="1:20" s="9" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="39" t="s">
+        <v>575</v>
+      </c>
+      <c r="B35" s="39"/>
+      <c r="C35" s="39" t="s">
+        <v>352</v>
+      </c>
+      <c r="D35" s="40" t="s">
+        <v>103</v>
+      </c>
+      <c r="E35" s="39" t="s">
+        <v>576</v>
+      </c>
+      <c r="F35" s="39" t="s">
+        <v>340</v>
+      </c>
+      <c r="G35" s="39" t="s">
+        <v>368</v>
+      </c>
+      <c r="H35" s="39">
+        <v>-81.867118796822695</v>
+      </c>
+      <c r="I35" s="39">
+        <v>38.537901317549398</v>
+      </c>
+      <c r="J35" s="39" t="s">
+        <v>577</v>
+      </c>
+      <c r="K35" s="39" t="s">
+        <v>159</v>
+      </c>
+      <c r="L35" s="41">
+        <v>4900</v>
+      </c>
+      <c r="M35" s="42" t="s">
+        <v>338</v>
+      </c>
+      <c r="N35" s="42">
+        <v>48</v>
+      </c>
+      <c r="O35" s="42">
+        <v>333</v>
+      </c>
+      <c r="P35" s="42">
+        <v>1440</v>
+      </c>
+      <c r="Q35" s="39" t="s">
+        <v>347</v>
+      </c>
+      <c r="R35" s="39" t="s">
+        <v>20</v>
+      </c>
+      <c r="S35" s="40">
+        <v>25168</v>
+      </c>
+      <c r="T35" s="39"/>
+    </row>
+    <row r="36" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="26" t="s">
+        <v>580</v>
+      </c>
+      <c r="B36" s="26"/>
+      <c r="C36" s="26" t="s">
+        <v>352</v>
+      </c>
+      <c r="D36" s="29" t="s">
+        <v>103</v>
+      </c>
+      <c r="E36" s="26" t="s">
+        <v>573</v>
+      </c>
+      <c r="F36" s="26" t="s">
+        <v>340</v>
+      </c>
+      <c r="G36" s="26" t="s">
+        <v>368</v>
+      </c>
+      <c r="H36" s="26">
+        <v>-82.105144999999993</v>
+      </c>
+      <c r="I36" s="26">
+        <v>38.425437000000002</v>
+      </c>
+      <c r="J36" s="26" t="s">
+        <v>370</v>
+      </c>
+      <c r="K36" s="26" t="s">
+        <v>157</v>
+      </c>
+      <c r="L36" s="30">
+        <v>7200</v>
+      </c>
+      <c r="M36" s="31" t="s">
+        <v>338</v>
+      </c>
+      <c r="N36" s="31">
+        <v>24</v>
+      </c>
+      <c r="O36" s="31">
+        <v>25</v>
+      </c>
+      <c r="P36" s="31">
+        <v>20</v>
+      </c>
+      <c r="Q36" s="26" t="s">
+        <v>347</v>
+      </c>
+      <c r="R36" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="S36" s="29">
+        <v>25541</v>
+      </c>
+      <c r="T36" s="26" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="37" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="26" t="s">
+        <v>170</v>
+      </c>
+      <c r="B37" s="26"/>
+      <c r="C37" s="26" t="s">
+        <v>352</v>
+      </c>
+      <c r="D37" s="29" t="s">
+        <v>103</v>
+      </c>
+      <c r="E37" s="26" t="s">
+        <v>572</v>
+      </c>
+      <c r="F37" s="26" t="s">
+        <v>340</v>
+      </c>
+      <c r="G37" s="26" t="s">
+        <v>368</v>
+      </c>
+      <c r="H37" s="26">
+        <v>-82.244877751268803</v>
+      </c>
+      <c r="I37" s="26">
+        <v>38.372162360135</v>
+      </c>
+      <c r="J37" s="26" t="s">
+        <v>371</v>
+      </c>
+      <c r="K37" s="26" t="s">
+        <v>157</v>
+      </c>
+      <c r="L37" s="30">
+        <v>4050</v>
+      </c>
+      <c r="M37" s="31" t="s">
+        <v>338</v>
+      </c>
+      <c r="N37" s="31">
+        <v>24</v>
+      </c>
+      <c r="O37" s="31">
+        <v>25</v>
+      </c>
+      <c r="P37" s="31">
+        <v>20</v>
+      </c>
+      <c r="Q37" s="26" t="s">
+        <v>347</v>
+      </c>
+      <c r="R37" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="S37" s="29">
         <v>25545</v>
       </c>
-      <c r="T34" s="26" t="s">
+      <c r="T37" s="26" t="s">
         <v>160</v>
-      </c>
-    </row>
-    <row r="35" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="60" t="s">
-        <v>0</v>
-      </c>
-      <c r="B35" s="60" t="s">
-        <v>513</v>
-      </c>
-      <c r="C35" s="60" t="s">
-        <v>351</v>
-      </c>
-      <c r="D35" s="61" t="s">
-        <v>60</v>
-      </c>
-      <c r="E35" s="60" t="s">
-        <v>574</v>
-      </c>
-      <c r="F35" s="60" t="s">
-        <v>340</v>
-      </c>
-      <c r="G35" s="60" t="s">
-        <v>368</v>
-      </c>
-      <c r="H35" s="60">
-        <v>-81.677679999999995</v>
-      </c>
-      <c r="I35" s="60">
-        <v>38.372869999999999</v>
-      </c>
-      <c r="J35" s="60" t="s">
-        <v>249</v>
-      </c>
-      <c r="K35" s="60" t="s">
-        <v>1</v>
-      </c>
-      <c r="L35" s="63">
-        <v>50000</v>
-      </c>
-      <c r="M35" s="63" t="s">
-        <v>338</v>
-      </c>
-      <c r="N35" s="63">
-        <v>24</v>
-      </c>
-      <c r="O35" s="63"/>
-      <c r="P35" s="63"/>
-      <c r="Q35" s="60" t="s">
-        <v>348</v>
-      </c>
-      <c r="R35" s="60" t="s">
-        <v>20</v>
-      </c>
-      <c r="S35" s="61">
-        <v>25312</v>
-      </c>
-    </row>
-    <row r="36" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="60" t="s">
-        <v>16</v>
-      </c>
-      <c r="B36" s="60" t="s">
-        <v>526</v>
-      </c>
-      <c r="C36" s="60" t="s">
-        <v>351</v>
-      </c>
-      <c r="D36" s="61" t="s">
-        <v>60</v>
-      </c>
-      <c r="E36" s="60" t="s">
-        <v>78</v>
-      </c>
-      <c r="F36" s="60" t="s">
-        <v>340</v>
-      </c>
-      <c r="G36" s="60" t="s">
-        <v>369</v>
-      </c>
-      <c r="H36" s="60">
-        <v>-81.079930000000004</v>
-      </c>
-      <c r="I36" s="60">
-        <v>37.380360000000003</v>
-      </c>
-      <c r="J36" s="60" t="s">
-        <v>265</v>
-      </c>
-      <c r="K36" s="60" t="s">
-        <v>17</v>
-      </c>
-      <c r="L36" s="63">
-        <v>36000</v>
-      </c>
-      <c r="M36" s="62" t="s">
-        <v>342</v>
-      </c>
-      <c r="N36" s="63">
-        <v>24</v>
-      </c>
-      <c r="O36" s="63">
-        <v>25</v>
-      </c>
-      <c r="P36" s="63">
-        <v>20</v>
-      </c>
-      <c r="Q36" s="60" t="s">
-        <v>347</v>
-      </c>
-      <c r="R36" s="60" t="s">
-        <v>20</v>
-      </c>
-      <c r="S36" s="61">
-        <v>24740</v>
-      </c>
-    </row>
-    <row r="37" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="60" t="s">
-        <v>106</v>
-      </c>
-      <c r="B37" s="60" t="s">
-        <v>527</v>
-      </c>
-      <c r="C37" s="60" t="s">
-        <v>351</v>
-      </c>
-      <c r="D37" s="61" t="s">
-        <v>60</v>
-      </c>
-      <c r="E37" s="60" t="s">
-        <v>107</v>
-      </c>
-      <c r="F37" s="60" t="s">
-        <v>340</v>
-      </c>
-      <c r="G37" s="60" t="s">
-        <v>368</v>
-      </c>
-      <c r="H37" s="60">
-        <v>-80.545150000000007</v>
-      </c>
-      <c r="I37" s="64">
-        <v>39.285969999999999</v>
-      </c>
-      <c r="J37" s="60" t="s">
-        <v>266</v>
-      </c>
-      <c r="K37" s="60" t="s">
-        <v>88</v>
-      </c>
-      <c r="L37" s="63">
-        <v>1853</v>
-      </c>
-      <c r="M37" s="62" t="s">
-        <v>337</v>
-      </c>
-      <c r="N37" s="63">
-        <v>24</v>
-      </c>
-      <c r="O37" s="63">
-        <v>25</v>
-      </c>
-      <c r="P37" s="63">
-        <v>20</v>
-      </c>
-      <c r="Q37" s="60" t="s">
-        <v>347</v>
-      </c>
-      <c r="R37" s="60" t="s">
-        <v>20</v>
-      </c>
-      <c r="S37" s="61">
-        <v>26426</v>
       </c>
     </row>
     <row r="38" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A38" s="60" t="s">
-        <v>440</v>
+        <v>0</v>
       </c>
       <c r="B38" s="60" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="C38" s="60" t="s">
         <v>351</v>
@@ -4942,55 +4946,53 @@
         <v>60</v>
       </c>
       <c r="E38" s="60" t="s">
-        <v>441</v>
+        <v>574</v>
       </c>
       <c r="F38" s="60" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="G38" s="60" t="s">
         <v>368</v>
       </c>
       <c r="H38" s="60">
-        <v>-79.985057699999999</v>
+        <v>-81.677679999999995</v>
       </c>
       <c r="I38" s="60">
-        <v>39.648165400000003</v>
+        <v>38.372869999999999</v>
       </c>
       <c r="J38" s="60" t="s">
-        <v>10</v>
+        <v>249</v>
       </c>
       <c r="K38" s="60" t="s">
-        <v>11</v>
-      </c>
-      <c r="L38" s="62"/>
-      <c r="M38" s="62" t="s">
-        <v>337</v>
-      </c>
-      <c r="N38" s="62">
-        <v>8</v>
-      </c>
-      <c r="O38" s="63">
-        <v>25</v>
-      </c>
-      <c r="P38" s="63">
-        <v>30</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="L38" s="63">
+        <v>50000</v>
+      </c>
+      <c r="M38" s="63" t="s">
+        <v>338</v>
+      </c>
+      <c r="N38" s="63">
+        <v>24</v>
+      </c>
+      <c r="O38" s="63"/>
+      <c r="P38" s="63"/>
       <c r="Q38" s="60" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="R38" s="60" t="s">
         <v>20</v>
       </c>
       <c r="S38" s="61">
-        <v>26505</v>
+        <v>25312</v>
       </c>
     </row>
     <row r="39" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A39" s="60" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="B39" s="60" t="s">
-        <v>510</v>
+        <v>526</v>
       </c>
       <c r="C39" s="60" t="s">
         <v>351</v>
@@ -4999,38 +5001,40 @@
         <v>60</v>
       </c>
       <c r="E39" s="60" t="s">
-        <v>138</v>
+        <v>78</v>
       </c>
       <c r="F39" s="60" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="G39" s="60" t="s">
         <v>369</v>
       </c>
       <c r="H39" s="60">
-        <v>-79.972157499999994</v>
+        <v>-81.079930000000004</v>
       </c>
       <c r="I39" s="60">
-        <v>39.650096900000001</v>
+        <v>37.380360000000003</v>
       </c>
       <c r="J39" s="60" t="s">
-        <v>231</v>
+        <v>265</v>
       </c>
       <c r="K39" s="60" t="s">
-        <v>11</v>
-      </c>
-      <c r="L39" s="62"/>
+        <v>17</v>
+      </c>
+      <c r="L39" s="63">
+        <v>36000</v>
+      </c>
       <c r="M39" s="62" t="s">
-        <v>337</v>
-      </c>
-      <c r="N39" s="62">
-        <v>48</v>
-      </c>
-      <c r="O39" s="62">
+        <v>342</v>
+      </c>
+      <c r="N39" s="63">
+        <v>24</v>
+      </c>
+      <c r="O39" s="63">
         <v>25</v>
       </c>
-      <c r="P39" s="62">
-        <v>30</v>
+      <c r="P39" s="63">
+        <v>20</v>
       </c>
       <c r="Q39" s="60" t="s">
         <v>347</v>
@@ -5039,18 +5043,15 @@
         <v>20</v>
       </c>
       <c r="S39" s="61">
-        <v>26505</v>
-      </c>
-      <c r="T39" s="60" t="s">
-        <v>130</v>
+        <v>24740</v>
       </c>
     </row>
     <row r="40" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A40" s="60" t="s">
-        <v>35</v>
+        <v>106</v>
       </c>
       <c r="B40" s="60" t="s">
-        <v>511</v>
+        <v>527</v>
       </c>
       <c r="C40" s="60" t="s">
         <v>351</v>
@@ -5059,37 +5060,41 @@
         <v>60</v>
       </c>
       <c r="E40" s="60" t="s">
-        <v>66</v>
+        <v>107</v>
       </c>
       <c r="F40" s="60" t="s">
-        <v>34</v>
+        <v>340</v>
       </c>
       <c r="G40" s="60" t="s">
         <v>368</v>
       </c>
       <c r="H40" s="60">
-        <v>-79.905010000000004</v>
-      </c>
-      <c r="I40" s="60">
-        <v>39.610210000000002</v>
+        <v>-80.545150000000007</v>
+      </c>
+      <c r="I40" s="64">
+        <v>39.285969999999999</v>
       </c>
       <c r="J40" s="60" t="s">
-        <v>231</v>
+        <v>266</v>
       </c>
       <c r="K40" s="60" t="s">
-        <v>11</v>
-      </c>
-      <c r="L40" s="62">
-        <v>579</v>
+        <v>88</v>
+      </c>
+      <c r="L40" s="63">
+        <v>1853</v>
       </c>
       <c r="M40" s="62" t="s">
         <v>337</v>
       </c>
-      <c r="N40" s="62">
-        <v>8</v>
-      </c>
-      <c r="O40" s="62"/>
-      <c r="P40" s="62"/>
+      <c r="N40" s="63">
+        <v>24</v>
+      </c>
+      <c r="O40" s="63">
+        <v>25</v>
+      </c>
+      <c r="P40" s="63">
+        <v>20</v>
+      </c>
       <c r="Q40" s="60" t="s">
         <v>347</v>
       </c>
@@ -5097,15 +5102,15 @@
         <v>20</v>
       </c>
       <c r="S40" s="61">
-        <v>26508</v>
+        <v>26426</v>
       </c>
     </row>
     <row r="41" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A41" s="60" t="s">
-        <v>40</v>
+        <v>440</v>
       </c>
       <c r="B41" s="60" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="C41" s="60" t="s">
         <v>351</v>
@@ -5114,37 +5119,39 @@
         <v>60</v>
       </c>
       <c r="E41" s="60" t="s">
-        <v>70</v>
+        <v>441</v>
       </c>
       <c r="F41" s="60" t="s">
-        <v>34</v>
+        <v>341</v>
       </c>
       <c r="G41" s="60" t="s">
         <v>368</v>
       </c>
       <c r="H41" s="60">
-        <v>-79.867609999999999</v>
+        <v>-79.985057699999999</v>
       </c>
       <c r="I41" s="60">
-        <v>39.652670000000001</v>
+        <v>39.648165400000003</v>
       </c>
       <c r="J41" s="60" t="s">
-        <v>231</v>
+        <v>10</v>
       </c>
       <c r="K41" s="60" t="s">
         <v>11</v>
       </c>
-      <c r="L41" s="62">
-        <v>830</v>
-      </c>
+      <c r="L41" s="62"/>
       <c r="M41" s="62" t="s">
         <v>337</v>
       </c>
       <c r="N41" s="62">
         <v>8</v>
       </c>
-      <c r="O41" s="62"/>
-      <c r="P41" s="62"/>
+      <c r="O41" s="63">
+        <v>25</v>
+      </c>
+      <c r="P41" s="63">
+        <v>30</v>
+      </c>
       <c r="Q41" s="60" t="s">
         <v>347</v>
       </c>
@@ -5152,15 +5159,15 @@
         <v>20</v>
       </c>
       <c r="S41" s="61">
-        <v>26508</v>
-      </c>
-    </row>
-    <row r="42" spans="1:20" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>26505</v>
+      </c>
+    </row>
+    <row r="42" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A42" s="60" t="s">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="B42" s="60" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="C42" s="60" t="s">
         <v>351</v>
@@ -5169,19 +5176,19 @@
         <v>60</v>
       </c>
       <c r="E42" s="60" t="s">
-        <v>72</v>
+        <v>138</v>
       </c>
       <c r="F42" s="60" t="s">
-        <v>34</v>
+        <v>341</v>
       </c>
       <c r="G42" s="60" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="H42" s="60">
-        <v>-79.957359999999994</v>
+        <v>-79.972157499999994</v>
       </c>
       <c r="I42" s="60">
-        <v>39.625419999999998</v>
+        <v>39.650096900000001</v>
       </c>
       <c r="J42" s="60" t="s">
         <v>231</v>
@@ -5189,17 +5196,19 @@
       <c r="K42" s="60" t="s">
         <v>11</v>
       </c>
-      <c r="L42" s="62">
-        <v>1851</v>
-      </c>
+      <c r="L42" s="62"/>
       <c r="M42" s="62" t="s">
         <v>337</v>
       </c>
       <c r="N42" s="62">
-        <v>8</v>
-      </c>
-      <c r="O42" s="62"/>
-      <c r="P42" s="62"/>
+        <v>48</v>
+      </c>
+      <c r="O42" s="62">
+        <v>25</v>
+      </c>
+      <c r="P42" s="62">
+        <v>30</v>
+      </c>
       <c r="Q42" s="60" t="s">
         <v>347</v>
       </c>
@@ -5207,12 +5216,15 @@
         <v>20</v>
       </c>
       <c r="S42" s="61">
-        <v>26501</v>
+        <v>26505</v>
+      </c>
+      <c r="T42" s="60" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="43" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A43" s="60" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="B43" s="60" t="s">
         <v>511</v>
@@ -5224,7 +5236,7 @@
         <v>60</v>
       </c>
       <c r="E43" s="60" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="F43" s="60" t="s">
         <v>34</v>
@@ -5233,10 +5245,10 @@
         <v>368</v>
       </c>
       <c r="H43" s="60">
-        <v>-79.943309999999997</v>
+        <v>-79.905010000000004</v>
       </c>
       <c r="I43" s="60">
-        <v>39.61036</v>
+        <v>39.610210000000002</v>
       </c>
       <c r="J43" s="60" t="s">
         <v>231</v>
@@ -5245,7 +5257,7 @@
         <v>11</v>
       </c>
       <c r="L43" s="62">
-        <v>726</v>
+        <v>579</v>
       </c>
       <c r="M43" s="62" t="s">
         <v>337</v>
@@ -5262,15 +5274,15 @@
         <v>20</v>
       </c>
       <c r="S43" s="61">
-        <v>26501</v>
+        <v>26508</v>
       </c>
     </row>
     <row r="44" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A44" s="60" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B44" s="60" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="C44" s="60" t="s">
         <v>351</v>
@@ -5279,7 +5291,7 @@
         <v>60</v>
       </c>
       <c r="E44" s="60" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="F44" s="60" t="s">
         <v>34</v>
@@ -5288,10 +5300,10 @@
         <v>368</v>
       </c>
       <c r="H44" s="60">
-        <v>-79.956739999999996</v>
+        <v>-79.867609999999999</v>
       </c>
       <c r="I44" s="60">
-        <v>39.660640000000001</v>
+        <v>39.652670000000001</v>
       </c>
       <c r="J44" s="60" t="s">
         <v>231</v>
@@ -5300,7 +5312,7 @@
         <v>11</v>
       </c>
       <c r="L44" s="62">
-        <v>688</v>
+        <v>830</v>
       </c>
       <c r="M44" s="62" t="s">
         <v>337</v>
@@ -5317,12 +5329,12 @@
         <v>20</v>
       </c>
       <c r="S44" s="61">
-        <v>26505</v>
-      </c>
-    </row>
-    <row r="45" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
+        <v>26508</v>
+      </c>
+    </row>
+    <row r="45" spans="1:20" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="60" t="s">
-        <v>58</v>
+        <v>38</v>
       </c>
       <c r="B45" s="60" t="s">
         <v>511</v>
@@ -5334,7 +5346,7 @@
         <v>60</v>
       </c>
       <c r="E45" s="60" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="F45" s="60" t="s">
         <v>34</v>
@@ -5343,10 +5355,10 @@
         <v>368</v>
       </c>
       <c r="H45" s="60">
-        <v>-79.978250000000003</v>
+        <v>-79.957359999999994</v>
       </c>
       <c r="I45" s="60">
-        <v>39.671370000000003</v>
+        <v>39.625419999999998</v>
       </c>
       <c r="J45" s="60" t="s">
         <v>231</v>
@@ -5355,7 +5367,7 @@
         <v>11</v>
       </c>
       <c r="L45" s="62">
-        <v>515</v>
+        <v>1851</v>
       </c>
       <c r="M45" s="62" t="s">
         <v>337</v>
@@ -5372,12 +5384,12 @@
         <v>20</v>
       </c>
       <c r="S45" s="61">
-        <v>26505</v>
+        <v>26501</v>
       </c>
     </row>
     <row r="46" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A46" s="60" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B46" s="60" t="s">
         <v>511</v>
@@ -5389,7 +5401,7 @@
         <v>60</v>
       </c>
       <c r="E46" s="60" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="F46" s="60" t="s">
         <v>34</v>
@@ -5398,10 +5410,10 @@
         <v>368</v>
       </c>
       <c r="H46" s="60">
-        <v>-79.926150000000007</v>
+        <v>-79.943309999999997</v>
       </c>
       <c r="I46" s="60">
-        <v>39.687820000000002</v>
+        <v>39.61036</v>
       </c>
       <c r="J46" s="60" t="s">
         <v>231</v>
@@ -5410,7 +5422,7 @@
         <v>11</v>
       </c>
       <c r="L46" s="62">
-        <v>1310</v>
+        <v>726</v>
       </c>
       <c r="M46" s="62" t="s">
         <v>337</v>
@@ -5427,12 +5439,12 @@
         <v>20</v>
       </c>
       <c r="S46" s="61">
-        <v>26508</v>
+        <v>26501</v>
       </c>
     </row>
     <row r="47" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A47" s="60" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="B47" s="60" t="s">
         <v>510</v>
@@ -5444,19 +5456,19 @@
         <v>60</v>
       </c>
       <c r="E47" s="60" t="s">
-        <v>187</v>
+        <v>75</v>
       </c>
       <c r="F47" s="60" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="G47" s="60" t="s">
         <v>368</v>
       </c>
       <c r="H47" s="60">
-        <v>-79.945801900000006</v>
+        <v>-79.956739999999996</v>
       </c>
       <c r="I47" s="60">
-        <v>39.6362083</v>
+        <v>39.660640000000001</v>
       </c>
       <c r="J47" s="60" t="s">
         <v>231</v>
@@ -5465,20 +5477,16 @@
         <v>11</v>
       </c>
       <c r="L47" s="62">
-        <v>567</v>
+        <v>688</v>
       </c>
       <c r="M47" s="62" t="s">
         <v>337</v>
       </c>
       <c r="N47" s="62">
-        <v>48</v>
-      </c>
-      <c r="O47" s="62">
-        <v>25</v>
-      </c>
-      <c r="P47" s="62">
-        <v>30</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="O47" s="62"/>
+      <c r="P47" s="62"/>
       <c r="Q47" s="60" t="s">
         <v>347</v>
       </c>
@@ -5488,16 +5496,13 @@
       <c r="S47" s="61">
         <v>26505</v>
       </c>
-      <c r="T47" s="60" t="s">
-        <v>131</v>
-      </c>
     </row>
     <row r="48" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A48" s="60" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="B48" s="60" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="C48" s="60" t="s">
         <v>351</v>
@@ -5506,19 +5511,19 @@
         <v>60</v>
       </c>
       <c r="E48" s="60" t="s">
-        <v>142</v>
+        <v>80</v>
       </c>
       <c r="F48" s="60" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="G48" s="60" t="s">
         <v>368</v>
       </c>
       <c r="H48" s="60">
-        <v>-79.953093199999998</v>
+        <v>-79.978250000000003</v>
       </c>
       <c r="I48" s="60">
-        <v>39.636423100000002</v>
+        <v>39.671370000000003</v>
       </c>
       <c r="J48" s="60" t="s">
         <v>231</v>
@@ -5527,20 +5532,16 @@
         <v>11</v>
       </c>
       <c r="L48" s="62">
-        <v>639</v>
+        <v>515</v>
       </c>
       <c r="M48" s="62" t="s">
         <v>337</v>
       </c>
       <c r="N48" s="62">
-        <v>48</v>
-      </c>
-      <c r="O48" s="62">
-        <v>25</v>
-      </c>
-      <c r="P48" s="62">
-        <v>30</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="O48" s="62"/>
+      <c r="P48" s="62"/>
       <c r="Q48" s="60" t="s">
         <v>347</v>
       </c>
@@ -5550,16 +5551,13 @@
       <c r="S48" s="61">
         <v>26505</v>
       </c>
-      <c r="T48" s="60" t="s">
-        <v>134</v>
-      </c>
     </row>
     <row r="49" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A49" s="60" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="B49" s="60" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="C49" s="60" t="s">
         <v>351</v>
@@ -5568,19 +5566,19 @@
         <v>60</v>
       </c>
       <c r="E49" s="60" t="s">
-        <v>143</v>
+        <v>81</v>
       </c>
       <c r="F49" s="60" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="G49" s="60" t="s">
         <v>368</v>
       </c>
       <c r="H49" s="60">
-        <v>-80.000420899999995</v>
+        <v>-79.926150000000007</v>
       </c>
       <c r="I49" s="60">
-        <v>39.6535571</v>
+        <v>39.687820000000002</v>
       </c>
       <c r="J49" s="60" t="s">
         <v>231</v>
@@ -5589,20 +5587,16 @@
         <v>11</v>
       </c>
       <c r="L49" s="62">
-        <v>912</v>
+        <v>1310</v>
       </c>
       <c r="M49" s="62" t="s">
         <v>337</v>
       </c>
       <c r="N49" s="62">
-        <v>48</v>
-      </c>
-      <c r="O49" s="62">
-        <v>25</v>
-      </c>
-      <c r="P49" s="62">
-        <v>30</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="O49" s="62"/>
+      <c r="P49" s="62"/>
       <c r="Q49" s="60" t="s">
         <v>347</v>
       </c>
@@ -5610,15 +5604,12 @@
         <v>20</v>
       </c>
       <c r="S49" s="61">
-        <v>26505</v>
-      </c>
-      <c r="T49" s="60" t="s">
-        <v>135</v>
+        <v>26508</v>
       </c>
     </row>
     <row r="50" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A50" s="60" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="B50" s="60" t="s">
         <v>510</v>
@@ -5630,7 +5621,7 @@
         <v>60</v>
       </c>
       <c r="E50" s="60" t="s">
-        <v>145</v>
+        <v>187</v>
       </c>
       <c r="F50" s="60" t="s">
         <v>19</v>
@@ -5639,10 +5630,10 @@
         <v>368</v>
       </c>
       <c r="H50" s="60">
-        <v>-79.956234100000003</v>
+        <v>-79.945801900000006</v>
       </c>
       <c r="I50" s="60">
-        <v>39.667909799999997</v>
+        <v>39.6362083</v>
       </c>
       <c r="J50" s="60" t="s">
         <v>231</v>
@@ -5650,7 +5641,9 @@
       <c r="K50" s="60" t="s">
         <v>11</v>
       </c>
-      <c r="L50" s="62"/>
+      <c r="L50" s="62">
+        <v>567</v>
+      </c>
       <c r="M50" s="62" t="s">
         <v>337</v>
       </c>
@@ -5673,12 +5666,12 @@
         <v>26505</v>
       </c>
       <c r="T50" s="60" t="s">
-        <v>42</v>
+        <v>131</v>
       </c>
     </row>
     <row r="51" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A51" s="60" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B51" s="60" t="s">
         <v>510</v>
@@ -5690,7 +5683,7 @@
         <v>60</v>
       </c>
       <c r="E51" s="60" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="F51" s="60" t="s">
         <v>19</v>
@@ -5699,10 +5692,10 @@
         <v>368</v>
       </c>
       <c r="H51" s="60">
-        <v>-79.956204600000007</v>
+        <v>-79.953093199999998</v>
       </c>
       <c r="I51" s="60">
-        <v>39.668112200000003</v>
+        <v>39.636423100000002</v>
       </c>
       <c r="J51" s="60" t="s">
         <v>231</v>
@@ -5710,7 +5703,9 @@
       <c r="K51" s="60" t="s">
         <v>11</v>
       </c>
-      <c r="L51" s="62"/>
+      <c r="L51" s="62">
+        <v>639</v>
+      </c>
       <c r="M51" s="62" t="s">
         <v>337</v>
       </c>
@@ -5733,12 +5728,12 @@
         <v>26505</v>
       </c>
       <c r="T51" s="60" t="s">
-        <v>43</v>
+        <v>134</v>
       </c>
     </row>
     <row r="52" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A52" s="60" t="s">
-        <v>192</v>
+        <v>26</v>
       </c>
       <c r="B52" s="60" t="s">
         <v>510</v>
@@ -5750,19 +5745,19 @@
         <v>60</v>
       </c>
       <c r="E52" s="60" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="F52" s="60" t="s">
         <v>19</v>
       </c>
       <c r="G52" s="60" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="H52" s="60">
-        <v>-79.956762600000005</v>
+        <v>-80.000420899999995</v>
       </c>
       <c r="I52" s="60">
-        <v>39.637875299999997</v>
+        <v>39.6535571</v>
       </c>
       <c r="J52" s="60" t="s">
         <v>231</v>
@@ -5771,7 +5766,7 @@
         <v>11</v>
       </c>
       <c r="L52" s="62">
-        <v>874</v>
+        <v>912</v>
       </c>
       <c r="M52" s="62" t="s">
         <v>337</v>
@@ -5795,12 +5790,12 @@
         <v>26505</v>
       </c>
       <c r="T52" s="60" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
     </row>
     <row r="53" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A53" s="60" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B53" s="60" t="s">
         <v>510</v>
@@ -5812,7 +5807,7 @@
         <v>60</v>
       </c>
       <c r="E53" s="60" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F53" s="60" t="s">
         <v>19</v>
@@ -5821,10 +5816,10 @@
         <v>368</v>
       </c>
       <c r="H53" s="60">
-        <v>-79.955122099999997</v>
+        <v>-79.956234100000003</v>
       </c>
       <c r="I53" s="60">
-        <v>39.669188599999998</v>
+        <v>39.667909799999997</v>
       </c>
       <c r="J53" s="60" t="s">
         <v>231</v>
@@ -5855,12 +5850,12 @@
         <v>26505</v>
       </c>
       <c r="T53" s="60" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="54" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A54" s="60" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B54" s="60" t="s">
         <v>510</v>
@@ -5872,7 +5867,7 @@
         <v>60</v>
       </c>
       <c r="E54" s="60" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="F54" s="60" t="s">
         <v>19</v>
@@ -5881,10 +5876,10 @@
         <v>368</v>
       </c>
       <c r="H54" s="60">
-        <v>-79.955245399999995</v>
+        <v>-79.956204600000007</v>
       </c>
       <c r="I54" s="60">
-        <v>39.669279500000002</v>
+        <v>39.668112200000003</v>
       </c>
       <c r="J54" s="60" t="s">
         <v>231</v>
@@ -5915,12 +5910,12 @@
         <v>26505</v>
       </c>
       <c r="T54" s="60" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="55" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A55" s="60" t="s">
-        <v>31</v>
+        <v>192</v>
       </c>
       <c r="B55" s="60" t="s">
         <v>510</v>
@@ -5932,7 +5927,7 @@
         <v>60</v>
       </c>
       <c r="E55" s="60" t="s">
-        <v>183</v>
+        <v>139</v>
       </c>
       <c r="F55" s="60" t="s">
         <v>19</v>
@@ -5941,10 +5936,10 @@
         <v>369</v>
       </c>
       <c r="H55" s="60">
-        <v>-79.965769100000003</v>
+        <v>-79.956762600000005</v>
       </c>
       <c r="I55" s="60">
-        <v>39.672765599999998</v>
+        <v>39.637875299999997</v>
       </c>
       <c r="J55" s="60" t="s">
         <v>231</v>
@@ -5952,7 +5947,9 @@
       <c r="K55" s="60" t="s">
         <v>11</v>
       </c>
-      <c r="L55" s="62"/>
+      <c r="L55" s="62">
+        <v>874</v>
+      </c>
       <c r="M55" s="62" t="s">
         <v>337</v>
       </c>
@@ -5975,12 +5972,12 @@
         <v>26505</v>
       </c>
       <c r="T55" s="60" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="56" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.2">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="56" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A56" s="60" t="s">
-        <v>339</v>
+        <v>29</v>
       </c>
       <c r="B56" s="60" t="s">
         <v>510</v>
@@ -5992,19 +5989,19 @@
         <v>60</v>
       </c>
       <c r="E56" s="60" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F56" s="60" t="s">
         <v>19</v>
       </c>
       <c r="G56" s="60" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="H56" s="60">
-        <v>-79.953202899999994</v>
+        <v>-79.955122099999997</v>
       </c>
       <c r="I56" s="60">
-        <v>39.633116399999999</v>
+        <v>39.669188599999998</v>
       </c>
       <c r="J56" s="60" t="s">
         <v>231</v>
@@ -6035,12 +6032,12 @@
         <v>26505</v>
       </c>
       <c r="T56" s="60" t="s">
-        <v>136</v>
+        <v>44</v>
       </c>
     </row>
     <row r="57" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A57" s="60" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="B57" s="60" t="s">
         <v>510</v>
@@ -6052,19 +6049,19 @@
         <v>60</v>
       </c>
       <c r="E57" s="60" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="F57" s="60" t="s">
         <v>19</v>
       </c>
       <c r="G57" s="60" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="H57" s="60">
-        <v>-79.962211800000006</v>
+        <v>-79.955245399999995</v>
       </c>
       <c r="I57" s="60">
-        <v>39.6511596</v>
+        <v>39.669279500000002</v>
       </c>
       <c r="J57" s="60" t="s">
         <v>231</v>
@@ -6072,9 +6069,7 @@
       <c r="K57" s="60" t="s">
         <v>11</v>
       </c>
-      <c r="L57" s="62">
-        <v>862</v>
-      </c>
+      <c r="L57" s="62"/>
       <c r="M57" s="62" t="s">
         <v>337</v>
       </c>
@@ -6097,12 +6092,12 @@
         <v>26505</v>
       </c>
       <c r="T57" s="60" t="s">
-        <v>133</v>
+        <v>45</v>
       </c>
     </row>
     <row r="58" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A58" s="60" t="s">
-        <v>184</v>
+        <v>31</v>
       </c>
       <c r="B58" s="60" t="s">
         <v>510</v>
@@ -6114,7 +6109,7 @@
         <v>60</v>
       </c>
       <c r="E58" s="60" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="F58" s="60" t="s">
         <v>19</v>
@@ -6123,10 +6118,10 @@
         <v>369</v>
       </c>
       <c r="H58" s="60">
-        <v>-79.956140000000005</v>
+        <v>-79.965769100000003</v>
       </c>
       <c r="I58" s="60">
-        <v>39.639200000000002</v>
+        <v>39.672765599999998</v>
       </c>
       <c r="J58" s="60" t="s">
         <v>231</v>
@@ -6134,9 +6129,7 @@
       <c r="K58" s="60" t="s">
         <v>11</v>
       </c>
-      <c r="L58" s="62">
-        <v>474</v>
-      </c>
+      <c r="L58" s="62"/>
       <c r="M58" s="62" t="s">
         <v>337</v>
       </c>
@@ -6159,12 +6152,12 @@
         <v>26505</v>
       </c>
       <c r="T58" s="60" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="59" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="59" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A59" s="60" t="s">
-        <v>24</v>
+        <v>339</v>
       </c>
       <c r="B59" s="60" t="s">
         <v>510</v>
@@ -6176,7 +6169,7 @@
         <v>60</v>
       </c>
       <c r="E59" s="60" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="F59" s="60" t="s">
         <v>19</v>
@@ -6185,10 +6178,10 @@
         <v>369</v>
       </c>
       <c r="H59" s="60">
-        <v>-79.966336100000007</v>
+        <v>-79.953202899999994</v>
       </c>
       <c r="I59" s="60">
-        <v>39.649548899999999</v>
+        <v>39.633116399999999</v>
       </c>
       <c r="J59" s="60" t="s">
         <v>231</v>
@@ -6196,9 +6189,7 @@
       <c r="K59" s="60" t="s">
         <v>11</v>
       </c>
-      <c r="L59" s="62">
-        <v>904</v>
-      </c>
+      <c r="L59" s="62"/>
       <c r="M59" s="62" t="s">
         <v>337</v>
       </c>
@@ -6221,12 +6212,12 @@
         <v>26505</v>
       </c>
       <c r="T59" s="60" t="s">
-        <v>41</v>
+        <v>136</v>
       </c>
     </row>
     <row r="60" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A60" s="60" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="B60" s="60" t="s">
         <v>510</v>
@@ -6238,7 +6229,7 @@
         <v>60</v>
       </c>
       <c r="E60" s="60" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="F60" s="60" t="s">
         <v>19</v>
@@ -6247,10 +6238,10 @@
         <v>369</v>
       </c>
       <c r="H60" s="60">
-        <v>-79.956755900000005</v>
+        <v>-79.962211800000006</v>
       </c>
       <c r="I60" s="60">
-        <v>39.640189999999997</v>
+        <v>39.6511596</v>
       </c>
       <c r="J60" s="60" t="s">
         <v>231</v>
@@ -6258,7 +6249,9 @@
       <c r="K60" s="60" t="s">
         <v>11</v>
       </c>
-      <c r="L60" s="62"/>
+      <c r="L60" s="62">
+        <v>862</v>
+      </c>
       <c r="M60" s="62" t="s">
         <v>337</v>
       </c>
@@ -6281,12 +6274,12 @@
         <v>26505</v>
       </c>
       <c r="T60" s="60" t="s">
-        <v>47</v>
+        <v>133</v>
       </c>
     </row>
     <row r="61" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A61" s="60" t="s">
-        <v>33</v>
+        <v>184</v>
       </c>
       <c r="B61" s="60" t="s">
         <v>510</v>
@@ -6298,19 +6291,19 @@
         <v>60</v>
       </c>
       <c r="E61" s="60" t="s">
-        <v>150</v>
+        <v>185</v>
       </c>
       <c r="F61" s="60" t="s">
         <v>19</v>
       </c>
       <c r="G61" s="60" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="H61" s="60">
-        <v>-79.925397000000004</v>
+        <v>-79.956140000000005</v>
       </c>
       <c r="I61" s="60">
-        <v>39.6565887</v>
+        <v>39.639200000000002</v>
       </c>
       <c r="J61" s="60" t="s">
         <v>231</v>
@@ -6318,7 +6311,9 @@
       <c r="K61" s="60" t="s">
         <v>11</v>
       </c>
-      <c r="L61" s="62"/>
+      <c r="L61" s="62">
+        <v>474</v>
+      </c>
       <c r="M61" s="62" t="s">
         <v>337</v>
       </c>
@@ -6341,57 +6336,57 @@
         <v>26505</v>
       </c>
       <c r="T61" s="60" t="s">
-        <v>48</v>
+        <v>186</v>
       </c>
     </row>
     <row r="62" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A62" s="60" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="B62" s="60" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C62" s="60" t="s">
         <v>351</v>
       </c>
       <c r="D62" s="61" t="s">
-        <v>181</v>
+        <v>60</v>
       </c>
       <c r="E62" s="60" t="s">
-        <v>65</v>
+        <v>148</v>
       </c>
       <c r="F62" s="60" t="s">
-        <v>340</v>
+        <v>19</v>
       </c>
       <c r="G62" s="60" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="H62" s="60">
-        <v>-81.015979999999999</v>
+        <v>-79.966336100000007</v>
       </c>
       <c r="I62" s="60">
-        <v>37.42163</v>
+        <v>39.649548899999999</v>
       </c>
       <c r="J62" s="60" t="s">
-        <v>244</v>
+        <v>231</v>
       </c>
       <c r="K62" s="60" t="s">
-        <v>17</v>
-      </c>
-      <c r="L62" s="63">
-        <v>2391</v>
+        <v>11</v>
+      </c>
+      <c r="L62" s="62">
+        <v>904</v>
       </c>
       <c r="M62" s="62" t="s">
-        <v>342</v>
-      </c>
-      <c r="N62" s="63">
-        <v>24</v>
-      </c>
-      <c r="O62" s="63">
+        <v>337</v>
+      </c>
+      <c r="N62" s="62">
+        <v>48</v>
+      </c>
+      <c r="O62" s="62">
         <v>25</v>
       </c>
-      <c r="P62" s="63">
-        <v>20</v>
+      <c r="P62" s="62">
+        <v>30</v>
       </c>
       <c r="Q62" s="60" t="s">
         <v>347</v>
@@ -6400,116 +6395,138 @@
         <v>20</v>
       </c>
       <c r="S62" s="61">
-        <v>24740</v>
-      </c>
-    </row>
-    <row r="63" spans="1:20" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>26505</v>
+      </c>
+      <c r="T62" s="60" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="63" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A63" s="60" t="s">
-        <v>112</v>
+        <v>32</v>
+      </c>
+      <c r="B63" s="60" t="s">
+        <v>510</v>
       </c>
       <c r="C63" s="60" t="s">
         <v>351</v>
       </c>
       <c r="D63" s="61" t="s">
-        <v>181</v>
+        <v>60</v>
       </c>
       <c r="E63" s="60" t="s">
-        <v>119</v>
+        <v>149</v>
       </c>
       <c r="F63" s="60" t="s">
-        <v>340</v>
+        <v>19</v>
       </c>
       <c r="G63" s="60" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="H63" s="60">
-        <v>-79.936940000000007</v>
-      </c>
-      <c r="I63" s="64">
-        <v>39.022010000000002</v>
+        <v>-79.956755900000005</v>
+      </c>
+      <c r="I63" s="60">
+        <v>39.640189999999997</v>
       </c>
       <c r="J63" s="60" t="s">
-        <v>245</v>
+        <v>231</v>
       </c>
       <c r="K63" s="60" t="s">
-        <v>123</v>
-      </c>
-      <c r="L63" s="63">
-        <v>1974</v>
-      </c>
-      <c r="M63" s="63" t="s">
-        <v>338</v>
-      </c>
-      <c r="N63" s="63">
-        <v>24</v>
-      </c>
-      <c r="O63" s="63"/>
-      <c r="P63" s="63"/>
+        <v>11</v>
+      </c>
+      <c r="L63" s="62"/>
+      <c r="M63" s="62" t="s">
+        <v>337</v>
+      </c>
+      <c r="N63" s="62">
+        <v>48</v>
+      </c>
+      <c r="O63" s="62">
+        <v>25</v>
+      </c>
+      <c r="P63" s="62">
+        <v>30</v>
+      </c>
       <c r="Q63" s="60" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="R63" s="60" t="s">
         <v>20</v>
       </c>
       <c r="S63" s="61">
-        <v>26250</v>
-      </c>
-    </row>
-    <row r="64" spans="1:20" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>26505</v>
+      </c>
+      <c r="T63" s="60" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="64" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A64" s="60" t="s">
-        <v>110</v>
+        <v>33</v>
+      </c>
+      <c r="B64" s="60" t="s">
+        <v>510</v>
       </c>
       <c r="C64" s="60" t="s">
         <v>351</v>
       </c>
       <c r="D64" s="61" t="s">
-        <v>181</v>
+        <v>60</v>
       </c>
       <c r="E64" s="60" t="s">
-        <v>117</v>
+        <v>150</v>
       </c>
       <c r="F64" s="60" t="s">
-        <v>340</v>
+        <v>19</v>
       </c>
       <c r="G64" s="60" t="s">
         <v>368</v>
       </c>
       <c r="H64" s="60">
-        <v>-80.212010000000006</v>
-      </c>
-      <c r="I64" s="64">
-        <v>39.72007</v>
+        <v>-79.925397000000004</v>
+      </c>
+      <c r="I64" s="60">
+        <v>39.6565887</v>
       </c>
       <c r="J64" s="60" t="s">
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="K64" s="60" t="s">
         <v>11</v>
       </c>
-      <c r="L64" s="62">
-        <v>400</v>
-      </c>
-      <c r="M64" s="63" t="s">
-        <v>338</v>
-      </c>
-      <c r="N64" s="63">
-        <v>24</v>
-      </c>
-      <c r="O64" s="63"/>
-      <c r="P64" s="63"/>
+      <c r="L64" s="62"/>
+      <c r="M64" s="62" t="s">
+        <v>337</v>
+      </c>
+      <c r="N64" s="62">
+        <v>48</v>
+      </c>
+      <c r="O64" s="62">
+        <v>25</v>
+      </c>
+      <c r="P64" s="62">
+        <v>30</v>
+      </c>
       <c r="Q64" s="60" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="R64" s="60" t="s">
         <v>20</v>
       </c>
       <c r="S64" s="61">
-        <v>26521</v>
-      </c>
-    </row>
-    <row r="65" spans="1:20" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>26505</v>
+      </c>
+      <c r="T64" s="60" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="65" spans="1:19" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A65" s="60" t="s">
-        <v>92</v>
+        <v>18</v>
+      </c>
+      <c r="B65" s="60" t="s">
+        <v>512</v>
       </c>
       <c r="C65" s="60" t="s">
         <v>351</v>
@@ -6518,7 +6535,7 @@
         <v>181</v>
       </c>
       <c r="E65" s="60" t="s">
-        <v>94</v>
+        <v>65</v>
       </c>
       <c r="F65" s="60" t="s">
         <v>340</v>
@@ -6527,41 +6544,45 @@
         <v>368</v>
       </c>
       <c r="H65" s="60">
-        <v>-80.258989999999997</v>
-      </c>
-      <c r="I65" s="64">
-        <v>39.280479999999997</v>
+        <v>-81.015979999999999</v>
+      </c>
+      <c r="I65" s="60">
+        <v>37.42163</v>
       </c>
       <c r="J65" s="60" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="K65" s="60" t="s">
-        <v>88</v>
+        <v>17</v>
       </c>
       <c r="L65" s="63">
-        <v>6984</v>
-      </c>
-      <c r="M65" s="63" t="s">
-        <v>338</v>
+        <v>2391</v>
+      </c>
+      <c r="M65" s="62" t="s">
+        <v>342</v>
       </c>
       <c r="N65" s="63">
         <v>24</v>
       </c>
-      <c r="O65" s="63"/>
-      <c r="P65" s="63"/>
+      <c r="O65" s="63">
+        <v>25</v>
+      </c>
+      <c r="P65" s="63">
+        <v>20</v>
+      </c>
       <c r="Q65" s="60" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="R65" s="60" t="s">
         <v>20</v>
       </c>
       <c r="S65" s="61">
-        <v>26330</v>
-      </c>
-    </row>
-    <row r="66" spans="1:20" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>24740</v>
+      </c>
+    </row>
+    <row r="66" spans="1:19" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="60" t="s">
-        <v>53</v>
+        <v>112</v>
       </c>
       <c r="C66" s="60" t="s">
         <v>351</v>
@@ -6570,7 +6591,7 @@
         <v>181</v>
       </c>
       <c r="E66" s="60" t="s">
-        <v>67</v>
+        <v>119</v>
       </c>
       <c r="F66" s="60" t="s">
         <v>340</v>
@@ -6579,45 +6600,41 @@
         <v>368</v>
       </c>
       <c r="H66" s="60">
-        <v>-80.567440000000005</v>
+        <v>-79.936940000000007</v>
       </c>
       <c r="I66" s="64">
-        <v>39.826610000000002</v>
+        <v>39.022010000000002</v>
       </c>
       <c r="J66" s="60" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="K66" s="60" t="s">
-        <v>5</v>
+        <v>123</v>
       </c>
       <c r="L66" s="63">
-        <v>1340</v>
-      </c>
-      <c r="M66" s="62" t="s">
-        <v>337</v>
+        <v>1974</v>
+      </c>
+      <c r="M66" s="63" t="s">
+        <v>338</v>
       </c>
       <c r="N66" s="63">
         <v>24</v>
       </c>
-      <c r="O66" s="63">
-        <v>25</v>
-      </c>
-      <c r="P66" s="63">
-        <v>30</v>
-      </c>
+      <c r="O66" s="63"/>
+      <c r="P66" s="63"/>
       <c r="Q66" s="60" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="R66" s="60" t="s">
         <v>20</v>
       </c>
       <c r="S66" s="61">
-        <v>26033</v>
-      </c>
-    </row>
-    <row r="67" spans="1:20" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>26250</v>
+      </c>
+    </row>
+    <row r="67" spans="1:19" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="60" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="C67" s="60" t="s">
         <v>351</v>
@@ -6626,7 +6643,7 @@
         <v>181</v>
       </c>
       <c r="E67" s="60" t="s">
-        <v>97</v>
+        <v>117</v>
       </c>
       <c r="F67" s="60" t="s">
         <v>340</v>
@@ -6635,48 +6652,41 @@
         <v>368</v>
       </c>
       <c r="H67" s="60">
-        <v>-80.124449999999996</v>
+        <v>-80.212010000000006</v>
       </c>
       <c r="I67" s="64">
-        <v>39.493949999999998</v>
+        <v>39.72007</v>
       </c>
       <c r="J67" s="60" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
       <c r="K67" s="60" t="s">
-        <v>89</v>
-      </c>
-      <c r="L67" s="63">
-        <v>25525</v>
-      </c>
-      <c r="M67" s="62" t="s">
-        <v>337</v>
+        <v>11</v>
+      </c>
+      <c r="L67" s="62">
+        <v>400</v>
+      </c>
+      <c r="M67" s="63" t="s">
+        <v>338</v>
       </c>
       <c r="N67" s="63">
         <v>24</v>
       </c>
-      <c r="O67" s="63">
-        <v>25</v>
-      </c>
-      <c r="P67" s="63">
-        <v>30</v>
-      </c>
+      <c r="O67" s="63"/>
+      <c r="P67" s="63"/>
       <c r="Q67" s="60" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="R67" s="60" t="s">
         <v>20</v>
       </c>
       <c r="S67" s="61">
-        <v>26554</v>
-      </c>
-    </row>
-    <row r="68" spans="1:20" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>26521</v>
+      </c>
+    </row>
+    <row r="68" spans="1:19" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="60" t="s">
-        <v>111</v>
-      </c>
-      <c r="B68" s="60" t="s">
-        <v>517</v>
+        <v>92</v>
       </c>
       <c r="C68" s="60" t="s">
         <v>351</v>
@@ -6685,7 +6695,7 @@
         <v>181</v>
       </c>
       <c r="E68" s="60" t="s">
-        <v>118</v>
+        <v>94</v>
       </c>
       <c r="F68" s="60" t="s">
         <v>340</v>
@@ -6694,48 +6704,41 @@
         <v>368</v>
       </c>
       <c r="H68" s="60">
-        <v>-80.598290000000006</v>
+        <v>-80.258989999999997</v>
       </c>
       <c r="I68" s="64">
-        <v>40.325800000000001</v>
+        <v>39.280479999999997</v>
       </c>
       <c r="J68" s="60" t="s">
-        <v>256</v>
+        <v>247</v>
       </c>
       <c r="K68" s="60" t="s">
-        <v>122</v>
+        <v>88</v>
       </c>
       <c r="L68" s="63">
-        <v>6468</v>
-      </c>
-      <c r="M68" s="62" t="s">
-        <v>337</v>
+        <v>6984</v>
+      </c>
+      <c r="M68" s="63" t="s">
+        <v>338</v>
       </c>
       <c r="N68" s="63">
         <v>24</v>
       </c>
-      <c r="O68" s="63">
-        <v>25</v>
-      </c>
-      <c r="P68" s="63">
-        <v>20</v>
-      </c>
+      <c r="O68" s="63"/>
+      <c r="P68" s="63"/>
       <c r="Q68" s="60" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="R68" s="60" t="s">
         <v>20</v>
       </c>
       <c r="S68" s="61">
-        <v>26037</v>
-      </c>
-    </row>
-    <row r="69" spans="1:20" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>26330</v>
+      </c>
+    </row>
+    <row r="69" spans="1:19" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="60" t="s">
-        <v>108</v>
-      </c>
-      <c r="B69" s="60" t="s">
-        <v>519</v>
+        <v>53</v>
       </c>
       <c r="C69" s="60" t="s">
         <v>351</v>
@@ -6744,7 +6747,7 @@
         <v>181</v>
       </c>
       <c r="E69" s="60" t="s">
-        <v>115</v>
+        <v>67</v>
       </c>
       <c r="F69" s="60" t="s">
         <v>340</v>
@@ -6753,19 +6756,19 @@
         <v>368</v>
       </c>
       <c r="H69" s="60">
-        <v>-79.978949999999998</v>
+        <v>-80.567440000000005</v>
       </c>
       <c r="I69" s="64">
-        <v>38.712879999999998</v>
+        <v>39.826610000000002</v>
       </c>
       <c r="J69" s="60" t="s">
-        <v>258</v>
+        <v>248</v>
       </c>
       <c r="K69" s="60" t="s">
-        <v>121</v>
+        <v>5</v>
       </c>
       <c r="L69" s="63">
-        <v>2101</v>
+        <v>1340</v>
       </c>
       <c r="M69" s="62" t="s">
         <v>337</v>
@@ -6777,7 +6780,7 @@
         <v>25</v>
       </c>
       <c r="P69" s="63">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="Q69" s="60" t="s">
         <v>347</v>
@@ -6786,15 +6789,12 @@
         <v>20</v>
       </c>
       <c r="S69" s="61">
-        <v>26273</v>
-      </c>
-    </row>
-    <row r="70" spans="1:20" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>26033</v>
+      </c>
+    </row>
+    <row r="70" spans="1:19" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="60" t="s">
-        <v>606</v>
-      </c>
-      <c r="B70" s="60" t="s">
-        <v>610</v>
+        <v>91</v>
       </c>
       <c r="C70" s="60" t="s">
         <v>351</v>
@@ -6803,50 +6803,57 @@
         <v>181</v>
       </c>
       <c r="E70" s="60" t="s">
-        <v>607</v>
+        <v>97</v>
       </c>
       <c r="F70" s="60" t="s">
         <v>340</v>
       </c>
       <c r="G70" s="60" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="H70" s="60">
-        <v>-78.955160000000006</v>
-      </c>
-      <c r="I70" s="60">
-        <v>39.115929999999999</v>
+        <v>-80.124449999999996</v>
+      </c>
+      <c r="I70" s="64">
+        <v>39.493949999999998</v>
       </c>
       <c r="J70" s="60" t="s">
-        <v>608</v>
+        <v>254</v>
       </c>
       <c r="K70" s="60" t="s">
-        <v>202</v>
+        <v>89</v>
       </c>
       <c r="L70" s="63">
-        <v>3510</v>
-      </c>
-      <c r="M70" s="63" t="s">
-        <v>338</v>
+        <v>25525</v>
+      </c>
+      <c r="M70" s="62" t="s">
+        <v>337</v>
       </c>
       <c r="N70" s="63">
         <v>24</v>
       </c>
-      <c r="O70" s="62"/>
-      <c r="P70" s="62"/>
+      <c r="O70" s="63">
+        <v>25</v>
+      </c>
+      <c r="P70" s="63">
+        <v>30</v>
+      </c>
       <c r="Q70" s="60" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="R70" s="60" t="s">
         <v>20</v>
       </c>
       <c r="S70" s="61">
-        <v>26836</v>
-      </c>
-    </row>
-    <row r="71" spans="1:20" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>26554</v>
+      </c>
+    </row>
+    <row r="71" spans="1:19" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="60" t="s">
-        <v>50</v>
+        <v>111</v>
+      </c>
+      <c r="B71" s="60" t="s">
+        <v>517</v>
       </c>
       <c r="C71" s="60" t="s">
         <v>351</v>
@@ -6855,7 +6862,7 @@
         <v>181</v>
       </c>
       <c r="E71" s="60" t="s">
-        <v>77</v>
+        <v>118</v>
       </c>
       <c r="F71" s="60" t="s">
         <v>340</v>
@@ -6864,41 +6871,48 @@
         <v>368</v>
       </c>
       <c r="H71" s="60">
-        <v>-79.127250000000004</v>
+        <v>-80.598290000000006</v>
       </c>
       <c r="I71" s="64">
-        <v>38.99091</v>
+        <v>40.325800000000001</v>
       </c>
       <c r="J71" s="60" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="K71" s="60" t="s">
-        <v>55</v>
+        <v>122</v>
       </c>
       <c r="L71" s="63">
-        <v>2700</v>
-      </c>
-      <c r="M71" s="63" t="s">
-        <v>338</v>
+        <v>6468</v>
+      </c>
+      <c r="M71" s="62" t="s">
+        <v>337</v>
       </c>
       <c r="N71" s="63">
         <v>24</v>
       </c>
-      <c r="O71" s="63"/>
-      <c r="P71" s="63"/>
+      <c r="O71" s="63">
+        <v>25</v>
+      </c>
+      <c r="P71" s="63">
+        <v>20</v>
+      </c>
       <c r="Q71" s="60" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="R71" s="60" t="s">
         <v>20</v>
       </c>
       <c r="S71" s="61">
-        <v>26847</v>
-      </c>
-    </row>
-    <row r="72" spans="1:20" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>26037</v>
+      </c>
+    </row>
+    <row r="72" spans="1:19" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="60" t="s">
-        <v>125</v>
+        <v>108</v>
+      </c>
+      <c r="B72" s="60" t="s">
+        <v>519</v>
       </c>
       <c r="C72" s="60" t="s">
         <v>351</v>
@@ -6907,7 +6921,7 @@
         <v>181</v>
       </c>
       <c r="E72" s="60" t="s">
-        <v>128</v>
+        <v>115</v>
       </c>
       <c r="F72" s="60" t="s">
         <v>340</v>
@@ -6915,37 +6929,49 @@
       <c r="G72" s="60" t="s">
         <v>368</v>
       </c>
+      <c r="H72" s="60">
+        <v>-79.978949999999998</v>
+      </c>
+      <c r="I72" s="64">
+        <v>38.712879999999998</v>
+      </c>
       <c r="J72" s="60" t="s">
-        <v>267</v>
+        <v>258</v>
       </c>
       <c r="K72" s="60" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="L72" s="63">
-        <v>1800</v>
-      </c>
-      <c r="M72" s="63" t="s">
-        <v>338</v>
+        <v>2101</v>
+      </c>
+      <c r="M72" s="62" t="s">
+        <v>337</v>
       </c>
       <c r="N72" s="63">
         <v>24</v>
       </c>
-      <c r="O72" s="63"/>
-      <c r="P72" s="63"/>
+      <c r="O72" s="63">
+        <v>25</v>
+      </c>
+      <c r="P72" s="63">
+        <v>20</v>
+      </c>
       <c r="Q72" s="60" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="R72" s="60" t="s">
         <v>20</v>
       </c>
-      <c r="S72" s="61"/>
-    </row>
-    <row r="73" spans="1:20" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="S72" s="61">
+        <v>26273</v>
+      </c>
+    </row>
+    <row r="73" spans="1:19" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="60" t="s">
-        <v>51</v>
+        <v>606</v>
       </c>
       <c r="B73" s="60" t="s">
-        <v>528</v>
+        <v>610</v>
       </c>
       <c r="C73" s="60" t="s">
         <v>351</v>
@@ -6954,57 +6980,50 @@
         <v>181</v>
       </c>
       <c r="E73" s="60" t="s">
-        <v>79</v>
+        <v>607</v>
       </c>
       <c r="F73" s="60" t="s">
         <v>340</v>
       </c>
       <c r="G73" s="60" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="H73" s="60">
-        <v>-81.205110000000005</v>
-      </c>
-      <c r="I73" s="64">
-        <v>39.391249999999999</v>
+        <v>-78.955160000000006</v>
+      </c>
+      <c r="I73" s="60">
+        <v>39.115929999999999</v>
       </c>
       <c r="J73" s="60" t="s">
-        <v>268</v>
+        <v>608</v>
       </c>
       <c r="K73" s="60" t="s">
-        <v>56</v>
+        <v>202</v>
       </c>
       <c r="L73" s="63">
-        <v>2892</v>
-      </c>
-      <c r="M73" s="62" t="s">
-        <v>337</v>
+        <v>3510</v>
+      </c>
+      <c r="M73" s="63" t="s">
+        <v>338</v>
       </c>
       <c r="N73" s="63">
         <v>24</v>
       </c>
-      <c r="O73" s="63">
-        <v>25</v>
-      </c>
-      <c r="P73" s="63">
-        <v>20</v>
-      </c>
+      <c r="O73" s="62"/>
+      <c r="P73" s="62"/>
       <c r="Q73" s="60" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="R73" s="60" t="s">
         <v>20</v>
       </c>
       <c r="S73" s="61">
-        <v>26170</v>
-      </c>
-    </row>
-    <row r="74" spans="1:20" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>26836</v>
+      </c>
+    </row>
+    <row r="74" spans="1:19" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="60" t="s">
-        <v>14</v>
-      </c>
-      <c r="B74" s="60" t="s">
-        <v>529</v>
+        <v>50</v>
       </c>
       <c r="C74" s="60" t="s">
         <v>351</v>
@@ -7013,7 +7032,7 @@
         <v>181</v>
       </c>
       <c r="E74" s="60" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="F74" s="60" t="s">
         <v>340</v>
@@ -7022,19 +7041,19 @@
         <v>368</v>
       </c>
       <c r="H74" s="60">
-        <v>-78.226619999999997</v>
-      </c>
-      <c r="I74" s="60">
-        <v>39.628019999999999</v>
+        <v>-79.127250000000004</v>
+      </c>
+      <c r="I74" s="64">
+        <v>38.99091</v>
       </c>
       <c r="J74" s="60" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="K74" s="60" t="s">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="L74" s="63">
-        <v>3255</v>
+        <v>2700</v>
       </c>
       <c r="M74" s="63" t="s">
         <v>338</v>
@@ -7051,12 +7070,12 @@
         <v>20</v>
       </c>
       <c r="S74" s="61">
-        <v>25411</v>
-      </c>
-    </row>
-    <row r="75" spans="1:20" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>26847</v>
+      </c>
+    </row>
+    <row r="75" spans="1:19" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="60" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C75" s="60" t="s">
         <v>351</v>
@@ -7065,7 +7084,7 @@
         <v>181</v>
       </c>
       <c r="E75" s="60" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F75" s="60" t="s">
         <v>340</v>
@@ -7074,13 +7093,13 @@
         <v>368</v>
       </c>
       <c r="J75" s="60" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="K75" s="60" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="L75" s="63">
-        <v>20411</v>
+        <v>1800</v>
       </c>
       <c r="M75" s="63" t="s">
         <v>338</v>
@@ -7098,9 +7117,12 @@
       </c>
       <c r="S75" s="61"/>
     </row>
-    <row r="76" spans="1:20" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:19" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="60" t="s">
-        <v>90</v>
+        <v>51</v>
+      </c>
+      <c r="B76" s="60" t="s">
+        <v>528</v>
       </c>
       <c r="C76" s="60" t="s">
         <v>351</v>
@@ -7109,7 +7131,7 @@
         <v>181</v>
       </c>
       <c r="E76" s="60" t="s">
-        <v>96</v>
+        <v>79</v>
       </c>
       <c r="F76" s="60" t="s">
         <v>340</v>
@@ -7118,19 +7140,19 @@
         <v>368</v>
       </c>
       <c r="H76" s="60">
-        <v>-80.260360000000006</v>
+        <v>-81.205110000000005</v>
       </c>
       <c r="I76" s="64">
-        <v>39.452579999999998</v>
+        <v>39.391249999999999</v>
       </c>
       <c r="J76" s="60" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="K76" s="60" t="s">
-        <v>89</v>
+        <v>56</v>
       </c>
       <c r="L76" s="63">
-        <v>2742</v>
+        <v>2892</v>
       </c>
       <c r="M76" s="62" t="s">
         <v>337</v>
@@ -7142,7 +7164,7 @@
         <v>25</v>
       </c>
       <c r="P76" s="63">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="Q76" s="60" t="s">
         <v>347</v>
@@ -7151,15 +7173,15 @@
         <v>20</v>
       </c>
       <c r="S76" s="61">
-        <v>26591</v>
-      </c>
-    </row>
-    <row r="77" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
+        <v>26170</v>
+      </c>
+    </row>
+    <row r="77" spans="1:19" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="60" t="s">
-        <v>59</v>
+        <v>14</v>
       </c>
       <c r="B77" s="60" t="s">
-        <v>525</v>
+        <v>529</v>
       </c>
       <c r="C77" s="60" t="s">
         <v>351</v>
@@ -7168,54 +7190,50 @@
         <v>181</v>
       </c>
       <c r="E77" s="60" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="F77" s="60" t="s">
-        <v>19</v>
+        <v>340</v>
       </c>
       <c r="G77" s="60" t="s">
         <v>368</v>
       </c>
       <c r="H77" s="60">
-        <v>-78.98272</v>
-      </c>
-      <c r="I77" s="64">
-        <v>39.438070000000003</v>
+        <v>-78.226619999999997</v>
+      </c>
+      <c r="I77" s="60">
+        <v>39.628019999999999</v>
       </c>
       <c r="J77" s="60" t="s">
-        <v>243</v>
+        <v>269</v>
       </c>
       <c r="K77" s="60" t="s">
-        <v>13</v>
-      </c>
-      <c r="L77" s="62">
-        <v>1193</v>
-      </c>
-      <c r="M77" s="62" t="s">
-        <v>337</v>
-      </c>
-      <c r="N77" s="62">
-        <v>48</v>
-      </c>
-      <c r="O77" s="63">
-        <v>25</v>
-      </c>
-      <c r="P77" s="63">
-        <v>30</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="L77" s="63">
+        <v>3255</v>
+      </c>
+      <c r="M77" s="63" t="s">
+        <v>338</v>
+      </c>
+      <c r="N77" s="63">
+        <v>24</v>
+      </c>
+      <c r="O77" s="63"/>
+      <c r="P77" s="63"/>
       <c r="Q77" s="60" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="R77" s="60" t="s">
         <v>20</v>
       </c>
       <c r="S77" s="61">
-        <v>26726</v>
-      </c>
-    </row>
-    <row r="78" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
+        <v>25411</v>
+      </c>
+    </row>
+    <row r="78" spans="1:19" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="60" t="s">
-        <v>235</v>
+        <v>126</v>
       </c>
       <c r="C78" s="60" t="s">
         <v>351</v>
@@ -7224,31 +7242,25 @@
         <v>181</v>
       </c>
       <c r="E78" s="60" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="F78" s="60" t="s">
-        <v>124</v>
+        <v>340</v>
       </c>
       <c r="G78" s="60" t="s">
         <v>368</v>
       </c>
-      <c r="H78" s="60">
-        <v>-79.515240000000006</v>
-      </c>
-      <c r="I78" s="64">
-        <v>39.66807</v>
-      </c>
       <c r="J78" s="60" t="s">
-        <v>234</v>
+        <v>270</v>
       </c>
       <c r="K78" s="60" t="s">
-        <v>63</v>
+        <v>122</v>
       </c>
       <c r="L78" s="63">
-        <v>1948</v>
-      </c>
-      <c r="M78" s="62" t="s">
-        <v>337</v>
+        <v>20411</v>
+      </c>
+      <c r="M78" s="63" t="s">
+        <v>338</v>
       </c>
       <c r="N78" s="63">
         <v>24</v>
@@ -7256,27 +7268,25 @@
       <c r="O78" s="63"/>
       <c r="P78" s="63"/>
       <c r="Q78" s="60" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="R78" s="60" t="s">
         <v>20</v>
       </c>
-      <c r="S78" s="61">
-        <v>26525</v>
-      </c>
-    </row>
-    <row r="79" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="S78" s="61"/>
+    </row>
+    <row r="79" spans="1:19" s="60" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="60" t="s">
-        <v>168</v>
+        <v>90</v>
       </c>
       <c r="C79" s="60" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="D79" s="61" t="s">
         <v>181</v>
       </c>
       <c r="E79" s="60" t="s">
-        <v>156</v>
+        <v>96</v>
       </c>
       <c r="F79" s="60" t="s">
         <v>340</v>
@@ -7285,30 +7295,30 @@
         <v>368</v>
       </c>
       <c r="H79" s="60">
-        <v>-82.285698770801503</v>
-      </c>
-      <c r="I79" s="60">
-        <v>38.414946823509098</v>
+        <v>-80.260360000000006</v>
+      </c>
+      <c r="I79" s="64">
+        <v>39.452579999999998</v>
       </c>
       <c r="J79" s="60" t="s">
-        <v>356</v>
+        <v>274</v>
       </c>
       <c r="K79" s="60" t="s">
-        <v>157</v>
-      </c>
-      <c r="L79" s="62">
-        <v>4000</v>
+        <v>89</v>
+      </c>
+      <c r="L79" s="63">
+        <v>2742</v>
       </c>
       <c r="M79" s="62" t="s">
-        <v>583</v>
-      </c>
-      <c r="N79" s="62">
+        <v>337</v>
+      </c>
+      <c r="N79" s="63">
         <v>24</v>
       </c>
-      <c r="O79" s="62">
-        <v>250</v>
-      </c>
-      <c r="P79" s="62">
+      <c r="O79" s="63">
+        <v>25</v>
+      </c>
+      <c r="P79" s="63">
         <v>30</v>
       </c>
       <c r="Q79" s="60" t="s">
@@ -7317,58 +7327,58 @@
       <c r="R79" s="60" t="s">
         <v>20</v>
       </c>
-      <c r="S79" s="66">
-        <v>25504</v>
-      </c>
-      <c r="T79" s="67" t="s">
-        <v>586</v>
-      </c>
-    </row>
-    <row r="80" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="S79" s="61">
+        <v>26591</v>
+      </c>
+    </row>
+    <row r="80" spans="1:19" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A80" s="60" t="s">
-        <v>169</v>
+        <v>59</v>
+      </c>
+      <c r="B80" s="60" t="s">
+        <v>525</v>
       </c>
       <c r="C80" s="60" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="D80" s="61" t="s">
         <v>181</v>
       </c>
       <c r="E80" s="60" t="s">
-        <v>158</v>
+        <v>87</v>
       </c>
       <c r="F80" s="60" t="s">
-        <v>340</v>
+        <v>19</v>
       </c>
       <c r="G80" s="60" t="s">
         <v>368</v>
       </c>
       <c r="H80" s="60">
-        <v>-82.006959612418996</v>
-      </c>
-      <c r="I80" s="60">
-        <v>38.446524084559897</v>
+        <v>-78.98272</v>
+      </c>
+      <c r="I80" s="64">
+        <v>39.438070000000003</v>
       </c>
       <c r="J80" s="60" t="s">
-        <v>359</v>
+        <v>243</v>
       </c>
       <c r="K80" s="60" t="s">
-        <v>159</v>
+        <v>13</v>
       </c>
       <c r="L80" s="62">
-        <v>28759</v>
-      </c>
-      <c r="M80" s="63" t="s">
-        <v>338</v>
-      </c>
-      <c r="N80" s="63">
-        <v>72</v>
+        <v>1193</v>
+      </c>
+      <c r="M80" s="62" t="s">
+        <v>337</v>
+      </c>
+      <c r="N80" s="62">
+        <v>48</v>
       </c>
       <c r="O80" s="63">
         <v>25</v>
       </c>
       <c r="P80" s="63">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="Q80" s="60" t="s">
         <v>347</v>
@@ -7377,55 +7387,51 @@
         <v>20</v>
       </c>
       <c r="S80" s="61">
-        <v>25526</v>
+        <v>26726</v>
       </c>
     </row>
     <row r="81" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A81" s="60" t="s">
-        <v>163</v>
+        <v>235</v>
       </c>
       <c r="C81" s="60" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="D81" s="61" t="s">
         <v>181</v>
       </c>
       <c r="E81" s="60" t="s">
-        <v>163</v>
+        <v>114</v>
       </c>
       <c r="F81" s="60" t="s">
-        <v>340</v>
+        <v>124</v>
       </c>
       <c r="G81" s="60" t="s">
         <v>368</v>
       </c>
       <c r="H81" s="60">
-        <v>-82.451303840583293</v>
-      </c>
-      <c r="I81" s="60">
-        <v>38.343336164586603</v>
+        <v>-79.515240000000006</v>
+      </c>
+      <c r="I81" s="64">
+        <v>39.66807</v>
       </c>
       <c r="J81" s="60" t="s">
-        <v>353</v>
+        <v>234</v>
       </c>
       <c r="K81" s="60" t="s">
-        <v>164</v>
-      </c>
-      <c r="L81" s="62">
-        <v>1600</v>
-      </c>
-      <c r="M81" s="63" t="s">
-        <v>338</v>
+        <v>63</v>
+      </c>
+      <c r="L81" s="63">
+        <v>1948</v>
+      </c>
+      <c r="M81" s="62" t="s">
+        <v>337</v>
       </c>
       <c r="N81" s="63">
         <v>24</v>
       </c>
-      <c r="O81" s="63">
-        <v>25</v>
-      </c>
-      <c r="P81" s="63">
-        <v>20</v>
-      </c>
+      <c r="O81" s="63"/>
+      <c r="P81" s="63"/>
       <c r="Q81" s="60" t="s">
         <v>347</v>
       </c>
@@ -7433,15 +7439,12 @@
         <v>20</v>
       </c>
       <c r="S81" s="61">
-        <v>25701</v>
-      </c>
-      <c r="T81" s="60" t="s">
-        <v>587</v>
+        <v>26525</v>
       </c>
     </row>
     <row r="82" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A82" s="60" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="C82" s="60" t="s">
         <v>352</v>
@@ -7450,7 +7453,7 @@
         <v>181</v>
       </c>
       <c r="E82" s="60" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="F82" s="60" t="s">
         <v>340</v>
@@ -7459,31 +7462,31 @@
         <v>368</v>
       </c>
       <c r="H82" s="60">
-        <v>-82.287563960345196</v>
+        <v>-82.285698770801503</v>
       </c>
       <c r="I82" s="60">
-        <v>38.572623654172197</v>
+        <v>38.414946823509098</v>
       </c>
       <c r="J82" s="60" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="K82" s="60" t="s">
         <v>157</v>
       </c>
       <c r="L82" s="62">
-        <v>1000</v>
-      </c>
-      <c r="M82" s="63" t="s">
-        <v>338</v>
-      </c>
-      <c r="N82" s="63">
+        <v>4000</v>
+      </c>
+      <c r="M82" s="62" t="s">
+        <v>583</v>
+      </c>
+      <c r="N82" s="62">
         <v>24</v>
       </c>
-      <c r="O82" s="63">
-        <v>25</v>
-      </c>
-      <c r="P82" s="63">
-        <v>20</v>
+      <c r="O82" s="62">
+        <v>250</v>
+      </c>
+      <c r="P82" s="62">
+        <v>30</v>
       </c>
       <c r="Q82" s="60" t="s">
         <v>347</v>
@@ -7491,16 +7494,16 @@
       <c r="R82" s="60" t="s">
         <v>20</v>
       </c>
-      <c r="S82" s="61">
-        <v>25537</v>
-      </c>
-      <c r="T82" s="60" t="s">
-        <v>588</v>
+      <c r="S82" s="66">
+        <v>25504</v>
+      </c>
+      <c r="T82" s="67" t="s">
+        <v>586</v>
       </c>
     </row>
     <row r="83" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A83" s="60" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C83" s="60" t="s">
         <v>352</v>
@@ -7509,38 +7512,40 @@
         <v>181</v>
       </c>
       <c r="E83" s="60" t="s">
-        <v>174</v>
+        <v>158</v>
       </c>
       <c r="F83" s="60" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="G83" s="60" t="s">
         <v>368</v>
       </c>
-      <c r="H83" s="65">
-        <v>-82.430654000000004</v>
-      </c>
-      <c r="I83" s="65">
-        <v>38.424089000000002</v>
-      </c>
-      <c r="J83" s="65" t="s">
-        <v>578</v>
+      <c r="H83" s="60">
+        <v>-82.006959612418996</v>
+      </c>
+      <c r="I83" s="60">
+        <v>38.446524084559897</v>
+      </c>
+      <c r="J83" s="60" t="s">
+        <v>359</v>
       </c>
       <c r="K83" s="60" t="s">
-        <v>157</v>
-      </c>
-      <c r="L83" s="62"/>
-      <c r="M83" s="62" t="s">
-        <v>583</v>
-      </c>
-      <c r="N83" s="62">
-        <v>5</v>
-      </c>
-      <c r="O83" s="62">
-        <v>35</v>
-      </c>
-      <c r="P83" s="62">
-        <v>30</v>
+        <v>159</v>
+      </c>
+      <c r="L83" s="62">
+        <v>28759</v>
+      </c>
+      <c r="M83" s="63" t="s">
+        <v>338</v>
+      </c>
+      <c r="N83" s="63">
+        <v>72</v>
+      </c>
+      <c r="O83" s="63">
+        <v>25</v>
+      </c>
+      <c r="P83" s="63">
+        <v>20</v>
       </c>
       <c r="Q83" s="60" t="s">
         <v>347</v>
@@ -7549,17 +7554,13 @@
         <v>20</v>
       </c>
       <c r="S83" s="61">
-        <v>25703</v>
-      </c>
-      <c r="T83" s="65" t="s">
-        <v>585</v>
-      </c>
-    </row>
-    <row r="84" spans="1:20" s="68" customFormat="1" x14ac:dyDescent="0.2">
+        <v>25526</v>
+      </c>
+    </row>
+    <row r="84" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A84" s="60" t="s">
-        <v>179</v>
-      </c>
-      <c r="B84" s="60"/>
+        <v>163</v>
+      </c>
       <c r="C84" s="60" t="s">
         <v>352</v>
       </c>
@@ -7567,38 +7568,40 @@
         <v>181</v>
       </c>
       <c r="E84" s="60" t="s">
-        <v>180</v>
+        <v>163</v>
       </c>
       <c r="F84" s="60" t="s">
-        <v>19</v>
+        <v>340</v>
       </c>
       <c r="G84" s="60" t="s">
         <v>368</v>
       </c>
-      <c r="H84" s="65">
-        <v>-82.425917999999996</v>
-      </c>
-      <c r="I84" s="65">
-        <v>38.421745999999999</v>
-      </c>
-      <c r="J84" s="65" t="s">
-        <v>579</v>
+      <c r="H84" s="60">
+        <v>-82.451303840583293</v>
+      </c>
+      <c r="I84" s="60">
+        <v>38.343336164586603</v>
+      </c>
+      <c r="J84" s="60" t="s">
+        <v>353</v>
       </c>
       <c r="K84" s="60" t="s">
-        <v>157</v>
-      </c>
-      <c r="L84" s="62"/>
-      <c r="M84" s="62" t="s">
-        <v>583</v>
-      </c>
-      <c r="N84" s="62">
-        <v>5</v>
-      </c>
-      <c r="O84" s="62">
-        <v>100</v>
-      </c>
-      <c r="P84" s="62">
-        <v>30</v>
+        <v>164</v>
+      </c>
+      <c r="L84" s="62">
+        <v>1600</v>
+      </c>
+      <c r="M84" s="63" t="s">
+        <v>338</v>
+      </c>
+      <c r="N84" s="63">
+        <v>24</v>
+      </c>
+      <c r="O84" s="63">
+        <v>25</v>
+      </c>
+      <c r="P84" s="63">
+        <v>20</v>
       </c>
       <c r="Q84" s="60" t="s">
         <v>347</v>
@@ -7607,15 +7610,15 @@
         <v>20</v>
       </c>
       <c r="S84" s="61">
-        <v>25703</v>
-      </c>
-      <c r="T84" s="65" t="s">
-        <v>584</v>
+        <v>25701</v>
+      </c>
+      <c r="T84" s="60" t="s">
+        <v>587</v>
       </c>
     </row>
     <row r="85" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A85" s="60" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="C85" s="60" t="s">
         <v>352</v>
@@ -7624,38 +7627,40 @@
         <v>181</v>
       </c>
       <c r="E85" s="60" t="s">
-        <v>176</v>
+        <v>165</v>
       </c>
       <c r="F85" s="60" t="s">
-        <v>19</v>
+        <v>340</v>
       </c>
       <c r="G85" s="60" t="s">
         <v>368</v>
       </c>
-      <c r="H85" s="65">
-        <v>-82.425557700629597</v>
-      </c>
-      <c r="I85" s="65">
-        <v>38.422913110104098</v>
-      </c>
-      <c r="J85" s="65" t="s">
-        <v>581</v>
+      <c r="H85" s="60">
+        <v>-82.287563960345196</v>
+      </c>
+      <c r="I85" s="60">
+        <v>38.572623654172197</v>
+      </c>
+      <c r="J85" s="60" t="s">
+        <v>354</v>
       </c>
       <c r="K85" s="60" t="s">
         <v>157</v>
       </c>
-      <c r="L85" s="62"/>
+      <c r="L85" s="62">
+        <v>1000</v>
+      </c>
       <c r="M85" s="63" t="s">
-        <v>583</v>
-      </c>
-      <c r="N85" s="62">
-        <v>5</v>
-      </c>
-      <c r="O85" s="62">
-        <v>35</v>
-      </c>
-      <c r="P85" s="62">
-        <v>30</v>
+        <v>338</v>
+      </c>
+      <c r="N85" s="63">
+        <v>24</v>
+      </c>
+      <c r="O85" s="63">
+        <v>25</v>
+      </c>
+      <c r="P85" s="63">
+        <v>20</v>
       </c>
       <c r="Q85" s="60" t="s">
         <v>347</v>
@@ -7664,12 +7669,15 @@
         <v>20</v>
       </c>
       <c r="S85" s="61">
-        <v>25703</v>
+        <v>25537</v>
+      </c>
+      <c r="T85" s="60" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="86" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A86" s="60" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="C86" s="60" t="s">
         <v>352</v>
@@ -7678,35 +7686,35 @@
         <v>181</v>
       </c>
       <c r="E86" s="60" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="F86" s="60" t="s">
-        <v>19</v>
+        <v>341</v>
       </c>
       <c r="G86" s="60" t="s">
         <v>368</v>
       </c>
       <c r="H86" s="65">
-        <v>-82.424907815220195</v>
+        <v>-82.430654000000004</v>
       </c>
       <c r="I86" s="65">
-        <v>38.423076174075902</v>
+        <v>38.424089000000002</v>
       </c>
       <c r="J86" s="65" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="K86" s="60" t="s">
         <v>157</v>
       </c>
       <c r="L86" s="62"/>
-      <c r="M86" s="63" t="s">
+      <c r="M86" s="62" t="s">
         <v>583</v>
       </c>
       <c r="N86" s="62">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="O86" s="62">
-        <v>100</v>
+        <v>35</v>
       </c>
       <c r="P86" s="62">
         <v>30</v>
@@ -7720,74 +7728,243 @@
       <c r="S86" s="61">
         <v>25703</v>
       </c>
-    </row>
-    <row r="87" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A87" s="71" t="s">
+      <c r="T86" s="65" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="87" spans="1:20" s="68" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A87" s="60" t="s">
+        <v>179</v>
+      </c>
+      <c r="B87" s="60"/>
+      <c r="C87" s="60" t="s">
+        <v>352</v>
+      </c>
+      <c r="D87" s="61" t="s">
+        <v>181</v>
+      </c>
+      <c r="E87" s="60" t="s">
+        <v>180</v>
+      </c>
+      <c r="F87" s="60" t="s">
+        <v>19</v>
+      </c>
+      <c r="G87" s="60" t="s">
+        <v>368</v>
+      </c>
+      <c r="H87" s="65">
+        <v>-82.425917999999996</v>
+      </c>
+      <c r="I87" s="65">
+        <v>38.421745999999999</v>
+      </c>
+      <c r="J87" s="65" t="s">
+        <v>579</v>
+      </c>
+      <c r="K87" s="60" t="s">
+        <v>157</v>
+      </c>
+      <c r="L87" s="62"/>
+      <c r="M87" s="62" t="s">
+        <v>583</v>
+      </c>
+      <c r="N87" s="62">
+        <v>5</v>
+      </c>
+      <c r="O87" s="62">
+        <v>100</v>
+      </c>
+      <c r="P87" s="62">
+        <v>30</v>
+      </c>
+      <c r="Q87" s="60" t="s">
+        <v>347</v>
+      </c>
+      <c r="R87" s="60" t="s">
+        <v>20</v>
+      </c>
+      <c r="S87" s="61">
+        <v>25703</v>
+      </c>
+      <c r="T87" s="65" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="88" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A88" s="60" t="s">
+        <v>175</v>
+      </c>
+      <c r="C88" s="60" t="s">
+        <v>352</v>
+      </c>
+      <c r="D88" s="61" t="s">
+        <v>181</v>
+      </c>
+      <c r="E88" s="60" t="s">
+        <v>176</v>
+      </c>
+      <c r="F88" s="60" t="s">
+        <v>19</v>
+      </c>
+      <c r="G88" s="60" t="s">
+        <v>368</v>
+      </c>
+      <c r="H88" s="65">
+        <v>-82.425557700629597</v>
+      </c>
+      <c r="I88" s="65">
+        <v>38.422913110104098</v>
+      </c>
+      <c r="J88" s="65" t="s">
+        <v>581</v>
+      </c>
+      <c r="K88" s="60" t="s">
+        <v>157</v>
+      </c>
+      <c r="L88" s="62"/>
+      <c r="M88" s="63" t="s">
+        <v>583</v>
+      </c>
+      <c r="N88" s="62">
+        <v>5</v>
+      </c>
+      <c r="O88" s="62">
+        <v>35</v>
+      </c>
+      <c r="P88" s="62">
+        <v>30</v>
+      </c>
+      <c r="Q88" s="60" t="s">
+        <v>347</v>
+      </c>
+      <c r="R88" s="60" t="s">
+        <v>20</v>
+      </c>
+      <c r="S88" s="61">
+        <v>25703</v>
+      </c>
+    </row>
+    <row r="89" spans="1:20" s="60" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A89" s="60" t="s">
+        <v>177</v>
+      </c>
+      <c r="C89" s="60" t="s">
+        <v>352</v>
+      </c>
+      <c r="D89" s="61" t="s">
+        <v>181</v>
+      </c>
+      <c r="E89" s="60" t="s">
+        <v>178</v>
+      </c>
+      <c r="F89" s="60" t="s">
+        <v>19</v>
+      </c>
+      <c r="G89" s="60" t="s">
+        <v>368</v>
+      </c>
+      <c r="H89" s="65">
+        <v>-82.424907815220195</v>
+      </c>
+      <c r="I89" s="65">
+        <v>38.423076174075902</v>
+      </c>
+      <c r="J89" s="65" t="s">
+        <v>582</v>
+      </c>
+      <c r="K89" s="60" t="s">
+        <v>157</v>
+      </c>
+      <c r="L89" s="62"/>
+      <c r="M89" s="63" t="s">
+        <v>583</v>
+      </c>
+      <c r="N89" s="62">
+        <v>24</v>
+      </c>
+      <c r="O89" s="62">
+        <v>100</v>
+      </c>
+      <c r="P89" s="62">
+        <v>30</v>
+      </c>
+      <c r="Q89" s="60" t="s">
+        <v>347</v>
+      </c>
+      <c r="R89" s="60" t="s">
+        <v>20</v>
+      </c>
+      <c r="S89" s="61">
+        <v>25703</v>
+      </c>
+    </row>
+    <row r="90" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A90" s="71" t="s">
         <v>653</v>
       </c>
-      <c r="B87" s="71"/>
-      <c r="C87" s="71" t="s">
+      <c r="B90" s="71"/>
+      <c r="C90" s="71" t="s">
         <v>352</v>
       </c>
-      <c r="D87" s="72" t="s">
+      <c r="D90" s="72" t="s">
         <v>103</v>
       </c>
-      <c r="E87" s="71" t="s">
+      <c r="E90" s="71" t="s">
         <v>654</v>
       </c>
-      <c r="F87" s="71" t="s">
+      <c r="F90" s="71" t="s">
         <v>340</v>
       </c>
-      <c r="G87" s="71" t="s">
+      <c r="G90" s="71" t="s">
         <v>368</v>
       </c>
-      <c r="H87" s="71">
+      <c r="H90" s="71">
         <v>-82.025433489999998</v>
       </c>
-      <c r="I87" s="71">
+      <c r="I90" s="71">
         <v>37.978467389999999</v>
       </c>
-      <c r="J87" s="71" t="s">
+      <c r="J90" s="71" t="s">
         <v>655</v>
       </c>
-      <c r="K87" s="71" t="s">
+      <c r="K90" s="71" t="s">
         <v>205</v>
       </c>
-      <c r="L87" s="73">
+      <c r="L90" s="73">
         <v>1200</v>
       </c>
-      <c r="M87" s="73" t="s">
+      <c r="M90" s="73" t="s">
         <v>338</v>
       </c>
-      <c r="N87" s="73">
+      <c r="N90" s="73">
         <v>8</v>
       </c>
-      <c r="O87" s="73">
+      <c r="O90" s="73">
         <v>200</v>
       </c>
-      <c r="P87" s="73">
+      <c r="P90" s="73">
         <v>60</v>
       </c>
-      <c r="Q87" s="71" t="s">
+      <c r="Q90" s="71" t="s">
         <v>347</v>
       </c>
-      <c r="R87" s="71" t="s">
-        <v>20</v>
-      </c>
-      <c r="S87" s="72">
+      <c r="R90" s="71" t="s">
+        <v>20</v>
+      </c>
+      <c r="S90" s="72">
         <v>25508</v>
       </c>
-      <c r="T87" s="71" t="s">
+      <c r="T90" s="71" t="s">
         <v>656</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T85" xr:uid="{D0856F7A-D0C0-3942-9027-9FB2F3C2C3E0}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:T86">
-    <sortCondition ref="D2:D86"/>
-    <sortCondition descending="1" ref="C2:C86"/>
-    <sortCondition descending="1" ref="F2:F86"/>
-    <sortCondition ref="A2:A86"/>
+  <autoFilter ref="A1:T88" xr:uid="{D0856F7A-D0C0-3942-9027-9FB2F3C2C3E0}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:T89">
+    <sortCondition ref="D2:D89"/>
+    <sortCondition descending="1" ref="C2:C89"/>
+    <sortCondition descending="1" ref="F2:F89"/>
+    <sortCondition ref="A2:A89"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>